<commit_message>
🤖 Progress: 2026-04-18 06:52 UTC
</commit_message>
<xml_diff>
--- a/rename_log.xlsx
+++ b/rename_log.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -474,6 +474,186 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>6362.psd</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0003.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>6361.psd</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>tamilpsd-0004.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>6360.psd</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0005.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>6359.psd</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>tamilpsd-0006.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>6358.psd</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0007.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>6357.psd</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>tamilpsd-0008.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>6356.psd</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0009.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>6355.psd</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>tamilpsd-0010.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>6354.psd</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0011.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>6353.psd</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>tamilpsd-0012.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>6352.psd</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0013.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>6351.psd</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>tamilpsd-0014.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>6350.psd</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0015.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>6349.psd</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>tamilpsd-0016.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>6348.psd</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0017.psd</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
🤖 Progress: 2026-04-18 07:20 UTC
</commit_message>
<xml_diff>
--- a/rename_log.xlsx
+++ b/rename_log.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B118"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -654,6 +654,1206 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>6347.psd</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>tamilpsd-0018.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>6346.psd</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0019.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>6345.psd</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>tamilpsd-0020.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>6342.psd</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0021.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>6341.psd</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>tamilpsd-0022.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>6340.psd</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0023.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>6339.psd</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>tamilpsd-0024.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>6338.psd</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0025.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>6337.psd</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>tamilpsd-0026.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>6336.psd</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0027.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>6335.psd</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>tamilpsd-0028.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>6334.psd</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0029.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>6333.psd</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>tamilpsd-0030.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>6332.psd</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0031.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>6331.psd</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>tamilpsd-0032.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>6330.psd</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0033.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>6329.psd</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>tamilpsd-0034.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>6328.psd</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0035.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>6327.psd</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>tamilpsd-0036.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>6326.psd</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0037.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>6325.psd</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>tamilpsd-0038.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>6324.psd</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0039.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>6323.psd</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>tamilpsd-0040.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>6322.psd</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0041.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>6321.psd</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>tamilpsd-0042.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>6320.psd</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0043.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>6319.psd</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>tamilpsd-0044.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>6318.psd</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0045.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>6317.psd</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>tamilpsd-0046.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>6316.psd</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0047.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>6315.psd</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>tamilpsd-0048.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>6314.psd</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0049.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>6313.psd</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>tamilpsd-0050.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>6312.psd</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0051.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>6311.psd</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>tamilpsd-0052.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>6310.psd</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0053.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>6309.psd</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>tamilpsd-0054.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>6307.psd</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0055.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>6306.psd</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>tamilpsd-0056.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>6305.psd</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0057.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>6304.psd</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>tamilpsd-0058.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>6303.psd</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0059.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>6302 - this file not suitable for photoshop 7.0 and cs3.psd</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>tamilpsd-0060.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>6301 - this file not suitable for photoshop 7.0 and cs3.psd</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0061.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>6300 - this file not suitable for photoshop 7.0 and cs3.psd</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>tamilpsd-0062.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>6299 - this file not suitable for photoshop 7.0 and cs3.psd</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0063.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>6298 - this file not suitable for photoshop 7.0 and cs3.psd</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>tamilpsd-0064.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>6297 - this file not suitable for photoshop 7.0 and cs3.psd</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0065.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>6296 - this file not suitable for photoshop 7.0 and cs3.psd</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>tamilpsd-0066.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>6295 - this file not suitable for photoshop 7.0 and cs3.psd</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0067.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>6294 - this file not suitable for photoshop 7.0 and cs3.psd</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>tamilpsd-0068.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>6293 - this file not suitable for photoshop 7.0 and cs3.psd</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0069.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>6292 - this file not suitable for photoshop 7.0 and cs3.psd</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>tamilpsd-0070.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>6291 - this file not suitable for photoshop 7.0 and cs3.psd</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0071.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>6290 - this file not suitable for photoshop 7.0 and cs3.psd</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>tamilpsd-0072.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>6289 - this file not suitable for photoshop 7.0 and cs3.psd</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0073.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>6288 - this file not suitable for photoshop 7.0 and cs3.psd</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>tamilpsd-0074.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>6287 - this file not suitable for photoshop 7.0 and cs3.psd</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0075.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>6286 - this file not suitable for photoshop 7.0 and cs3.psd</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>tamilpsd-0076.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>6285 - this file not suitable for photoshop 7.0 and cs3.psd</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0077.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>6284 - this file not suitable for photoshop 7.0 and cs3.psd</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>tamilpsd-0078.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>6283 - this file not suitable for photoshop 7.0 and cs3.psd</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0079.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>6282 - this file not suitable for photoshop 7.0 and cs3.psd</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>tamilpsd-0080.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>6281 - this file not suitable for photoshop 7.0 and cs3.psd</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0081.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>6280 - this file not suitable for photoshop 7.0 and cs3.psd</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>tamilpsd-0082.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>6279 - this file not suitable for photoshop 7.0 and cs3.psd</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0083.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>6278 - this file not suitable for photoshop 7.0 and cs3.psd</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>tamilpsd-0084.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>6277 - this file not suitable for photoshop 7.0 and cs3.psd</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0085.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>6276 - this file not suitable for photoshop 7.0 and cs3.psd</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>tamilpsd-0086.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>6275 - this file not suitable for photoshop 7.0 and cs3.psd</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0087.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>6274 - this file not suitable for photoshop 7.0 and cs3.psd</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>tamilpsd-0088.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>6273 - this file not suitable for photoshop 7.0 and cs3.psd</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0089.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>6272.psd</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>tamilpsd-0090.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>6271.psd</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0091.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>6270.psd</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>tamilpsd-0092.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>6269.psd</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0093.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>6268.psd</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>tamilpsd-0094.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>6267.psd</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0095.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>6266.psd</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>tamilpsd-0096.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>6265.psd</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0097.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>6264.psd</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>tamilpsd-0098.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>6263.psd</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0099.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>6262.psd</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>tamilpsd-0100.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>6261.psd</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0101.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>6260.psd</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>tamilpsd-0102.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>6259.psd</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0103.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>6258.psd</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>tamilpsd-0104.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>6257.psd</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0105.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>6256.psd</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>tamilpsd-0106.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>6255.psd</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0107.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>6254.psd</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>tamilpsd-0108.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>6253.psd</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0109.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>6252.psd</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>tamilpsd-0110.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>6251.psd</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0111.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>6250.psd</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>tamilpsd-0112.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>6249.psd</t>
+        </is>
+      </c>
+      <c r="B114" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0113.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>6248.psd</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>tamilpsd-0114.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>6247.psd</t>
+        </is>
+      </c>
+      <c r="B116" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0115.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>6246.psd</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>tamilpsd-0116.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>6245.psd</t>
+        </is>
+      </c>
+      <c r="B118" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0117.psd</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
🤖 Progress: 2026-04-18 07:34 UTC
</commit_message>
<xml_diff>
--- a/rename_log.xlsx
+++ b/rename_log.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B118"/>
+  <dimension ref="A1:B120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -1854,6 +1854,30 @@
         </is>
       </c>
     </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>6244.psd</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>tamilpsd-0118.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="inlineStr">
+        <is>
+          <t>6243.psd</t>
+        </is>
+      </c>
+      <c r="B120" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0119.psd</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
🤖 Progress: 2026-04-18 08:37 UTC
</commit_message>
<xml_diff>
--- a/rename_log.xlsx
+++ b/rename_log.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B120"/>
+  <dimension ref="A1:B251"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -1878,6 +1878,1578 @@
         </is>
       </c>
     </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>6242.psd</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>tamilpsd-0120.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
+          <t>6241.psd</t>
+        </is>
+      </c>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0121.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>6240.psd</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>tamilpsd-0122.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>6239.psd</t>
+        </is>
+      </c>
+      <c r="B124" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0123.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>6238.psd</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>tamilpsd-0124.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="inlineStr">
+        <is>
+          <t>6237.psd</t>
+        </is>
+      </c>
+      <c r="B126" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0125.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>6236.psd</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>tamilpsd-0126.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>6235.psd</t>
+        </is>
+      </c>
+      <c r="B128" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0127.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>6234.psd</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>tamilpsd-0128.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="inlineStr">
+        <is>
+          <t>6233.psd</t>
+        </is>
+      </c>
+      <c r="B130" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0129.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>6232.psd</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>tamilpsd-0130.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t>6231.psd</t>
+        </is>
+      </c>
+      <c r="B132" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0131.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>6230.psd</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>tamilpsd-0132.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="2" t="inlineStr">
+        <is>
+          <t>6229.psd</t>
+        </is>
+      </c>
+      <c r="B134" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0133.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>6228.psd</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>tamilpsd-0134.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="inlineStr">
+        <is>
+          <t>6227.psd</t>
+        </is>
+      </c>
+      <c r="B136" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0135.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>6226.psd</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>tamilpsd-0136.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="inlineStr">
+        <is>
+          <t>6225.psd</t>
+        </is>
+      </c>
+      <c r="B138" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0137.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>6224.psd</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>tamilpsd-0138.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>6223.psd</t>
+        </is>
+      </c>
+      <c r="B140" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0139.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>6222.psd</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>tamilpsd-0140.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t>6221.psd</t>
+        </is>
+      </c>
+      <c r="B142" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0141.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>6220.psd</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>tamilpsd-0142.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t>6219.psd</t>
+        </is>
+      </c>
+      <c r="B144" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0143.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>6218.psd</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>tamilpsd-0144.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="inlineStr">
+        <is>
+          <t>6217.psd</t>
+        </is>
+      </c>
+      <c r="B146" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0145.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>6216.psd</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>tamilpsd-0146.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="inlineStr">
+        <is>
+          <t>6215.psd</t>
+        </is>
+      </c>
+      <c r="B148" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0147.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>6214.psd</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>tamilpsd-0148.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="inlineStr">
+        <is>
+          <t>6213.psd</t>
+        </is>
+      </c>
+      <c r="B150" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0149.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>6212.psd</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>tamilpsd-0150.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="inlineStr">
+        <is>
+          <t>6211.psd</t>
+        </is>
+      </c>
+      <c r="B152" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0151.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>6210.psd</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>tamilpsd-0152.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="inlineStr">
+        <is>
+          <t>6209.psd</t>
+        </is>
+      </c>
+      <c r="B154" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0153.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>6208.psd</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>tamilpsd-0154.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="inlineStr">
+        <is>
+          <t>6207.psd</t>
+        </is>
+      </c>
+      <c r="B156" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0155.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>6206.psd</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>tamilpsd-0156.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="2" t="inlineStr">
+        <is>
+          <t>6205.psd</t>
+        </is>
+      </c>
+      <c r="B158" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0157.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>6203.psd</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>tamilpsd-0158.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="2" t="inlineStr">
+        <is>
+          <t>6202.psd</t>
+        </is>
+      </c>
+      <c r="B160" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0159.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>6201.psd</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>tamilpsd-0160.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="2" t="inlineStr">
+        <is>
+          <t>6200.psd</t>
+        </is>
+      </c>
+      <c r="B162" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0161.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>6199.psd</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>tamilpsd-0162.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="2" t="inlineStr">
+        <is>
+          <t>6198.psd</t>
+        </is>
+      </c>
+      <c r="B164" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0163.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>6197.psd</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>tamilpsd-0164.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="2" t="inlineStr">
+        <is>
+          <t>6196.psd</t>
+        </is>
+      </c>
+      <c r="B166" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0165.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>6195.psd</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>tamilpsd-0166.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="2" t="inlineStr">
+        <is>
+          <t>6194.psd</t>
+        </is>
+      </c>
+      <c r="B168" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0167.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>6193.psd</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>tamilpsd-0168.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="2" t="inlineStr">
+        <is>
+          <t>6192  This file is not suitable for photoshop 7.0 and cs3.psd</t>
+        </is>
+      </c>
+      <c r="B170" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0169.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>6188  This file is not suitable for photoshop 7.0 and cs3.psd</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>tamilpsd-0170.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="2" t="inlineStr">
+        <is>
+          <t>6187  This file is not suitable for photoshop 7.0 and cs3.psd</t>
+        </is>
+      </c>
+      <c r="B172" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0171.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>6185  This file is not suitable for photoshop 7.0 and cs3.psd</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>tamilpsd-0172.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="2" t="inlineStr">
+        <is>
+          <t>6184  This file is not suitable for photoshop 7.0 and cs3.psd</t>
+        </is>
+      </c>
+      <c r="B174" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0173.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>6183 This file is not suitable for photoshop 7.0 and cs3.psd</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>tamilpsd-0174.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="2" t="inlineStr">
+        <is>
+          <t>6240  This file is not suitable for photoshop 7.0 and cs3.psd</t>
+        </is>
+      </c>
+      <c r="B176" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0175.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>6344.psd</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>tamilpsd-0176.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="2" t="inlineStr">
+        <is>
+          <t>6343.psd</t>
+        </is>
+      </c>
+      <c r="B178" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0177.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>6308.psd</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>tamilpsd-0178.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="2" t="inlineStr">
+        <is>
+          <t>6302.psd</t>
+        </is>
+      </c>
+      <c r="B180" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0179.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>6301.psd</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>tamilpsd-0180.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="2" t="inlineStr">
+        <is>
+          <t>6299.psd</t>
+        </is>
+      </c>
+      <c r="B182" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0181.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>6298.psd</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>tamilpsd-0182.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="2" t="inlineStr">
+        <is>
+          <t>6297.psd</t>
+        </is>
+      </c>
+      <c r="B184" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0183.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>6296.psd</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>tamilpsd-0184.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="2" t="inlineStr">
+        <is>
+          <t>6295.psd</t>
+        </is>
+      </c>
+      <c r="B186" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0185.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>6294.psd</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>tamilpsd-0186.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="2" t="inlineStr">
+        <is>
+          <t>6293.psd</t>
+        </is>
+      </c>
+      <c r="B188" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0187.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>6292.psd</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>tamilpsd-0188.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="2" t="inlineStr">
+        <is>
+          <t>6291.psd</t>
+        </is>
+      </c>
+      <c r="B190" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0189.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>6290.psd</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>tamilpsd-0190.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="2" t="inlineStr">
+        <is>
+          <t>6289.psd</t>
+        </is>
+      </c>
+      <c r="B192" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0191.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>6288.psd</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>tamilpsd-0192.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="2" t="inlineStr">
+        <is>
+          <t>6287.psd</t>
+        </is>
+      </c>
+      <c r="B194" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0193.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>6286.psd</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>tamilpsd-0194.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="2" t="inlineStr">
+        <is>
+          <t>6285.psd</t>
+        </is>
+      </c>
+      <c r="B196" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0195.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>6284.psd</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>tamilpsd-0196.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="2" t="inlineStr">
+        <is>
+          <t>6283.psd</t>
+        </is>
+      </c>
+      <c r="B198" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0197.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>6282.psd</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>tamilpsd-0198.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="2" t="inlineStr">
+        <is>
+          <t>6281.psd</t>
+        </is>
+      </c>
+      <c r="B200" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0199.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>6280.psd</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>tamilpsd-0200.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="2" t="inlineStr">
+        <is>
+          <t>6279.psd</t>
+        </is>
+      </c>
+      <c r="B202" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0201.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>6278.psd</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>tamilpsd-0202.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="2" t="inlineStr">
+        <is>
+          <t>6277.psd</t>
+        </is>
+      </c>
+      <c r="B204" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0203.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>6205a.psd</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>tamilpsd-0204.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="2" t="inlineStr">
+        <is>
+          <t>6191.psd</t>
+        </is>
+      </c>
+      <c r="B206" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0205.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>6190.psd</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>tamilpsd-0206.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="2" t="inlineStr">
+        <is>
+          <t>6189.psd</t>
+        </is>
+      </c>
+      <c r="B208" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0207.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>6186.psd</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>tamilpsd-0208.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="2" t="inlineStr">
+        <is>
+          <t>6198 This file is not suitable for photoshop 7.0 and cs3.psd</t>
+        </is>
+      </c>
+      <c r="B210" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0209.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>6182.psd</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>tamilpsd-0210.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="2" t="inlineStr">
+        <is>
+          <t>6181.psd</t>
+        </is>
+      </c>
+      <c r="B212" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0211.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>6180.psd</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>tamilpsd-0212.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="2" t="inlineStr">
+        <is>
+          <t>6179.psd</t>
+        </is>
+      </c>
+      <c r="B214" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0213.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>6178.psd</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>tamilpsd-0214.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="2" t="inlineStr">
+        <is>
+          <t>6177.psd</t>
+        </is>
+      </c>
+      <c r="B216" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0215.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>6176.psd</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>tamilpsd-0216.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="2" t="inlineStr">
+        <is>
+          <t>6175.psd</t>
+        </is>
+      </c>
+      <c r="B218" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0217.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>6174.psd</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>tamilpsd-0218.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="2" t="inlineStr">
+        <is>
+          <t>6173.psd</t>
+        </is>
+      </c>
+      <c r="B220" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0219.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>6172.psd</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>tamilpsd-0220.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="2" t="inlineStr">
+        <is>
+          <t>6171.psd</t>
+        </is>
+      </c>
+      <c r="B222" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0221.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>6170.psd</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>tamilpsd-0222.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="2" t="inlineStr">
+        <is>
+          <t>6169.psd</t>
+        </is>
+      </c>
+      <c r="B224" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0223.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>6168.psd</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>tamilpsd-0224.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="2" t="inlineStr">
+        <is>
+          <t>6167.psd</t>
+        </is>
+      </c>
+      <c r="B226" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0225.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>6166.psd</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>tamilpsd-0226.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="2" t="inlineStr">
+        <is>
+          <t>6165.psd</t>
+        </is>
+      </c>
+      <c r="B228" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0227.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>6164.psd</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>tamilpsd-0228.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="2" t="inlineStr">
+        <is>
+          <t>6163.psd</t>
+        </is>
+      </c>
+      <c r="B230" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0229.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>6162.psd</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>tamilpsd-0230.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="2" t="inlineStr">
+        <is>
+          <t>6161.psd</t>
+        </is>
+      </c>
+      <c r="B232" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0231.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>6160.psd</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>tamilpsd-0232.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="2" t="inlineStr">
+        <is>
+          <t>6159.psd</t>
+        </is>
+      </c>
+      <c r="B234" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0233.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>6158.psd</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>tamilpsd-0234.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="2" t="inlineStr">
+        <is>
+          <t>6157.psd</t>
+        </is>
+      </c>
+      <c r="B236" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0235.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>6156.psd</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>tamilpsd-0236.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="2" t="inlineStr">
+        <is>
+          <t>6155.psd</t>
+        </is>
+      </c>
+      <c r="B238" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0237.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>6154.psd</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>tamilpsd-0238.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="2" t="inlineStr">
+        <is>
+          <t>6153.psd</t>
+        </is>
+      </c>
+      <c r="B240" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0239.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>6142.psd</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>tamilpsd-0240.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="2" t="inlineStr">
+        <is>
+          <t>6141.psd</t>
+        </is>
+      </c>
+      <c r="B242" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0241.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>6140.psd</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>tamilpsd-0242.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="2" t="inlineStr">
+        <is>
+          <t>6139.psd</t>
+        </is>
+      </c>
+      <c r="B244" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0243.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>6138.psd</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>tamilpsd-0244.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="2" t="inlineStr">
+        <is>
+          <t>6137.psd</t>
+        </is>
+      </c>
+      <c r="B246" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0245.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>6136.psd</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>tamilpsd-0246.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="2" t="inlineStr">
+        <is>
+          <t>6135.psd</t>
+        </is>
+      </c>
+      <c r="B248" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0247.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>6134.psd</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>tamilpsd-0248.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="2" t="inlineStr">
+        <is>
+          <t>6133.psd</t>
+        </is>
+      </c>
+      <c r="B250" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0249.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>6132.psd</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>tamilpsd-0250.psd</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
🤖 Progress: 2026-04-18 09:00 UTC
</commit_message>
<xml_diff>
--- a/rename_log.xlsx
+++ b/rename_log.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B251"/>
+  <dimension ref="A1:B351"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -3450,6 +3450,1206 @@
         </is>
       </c>
     </row>
+    <row r="252">
+      <c r="A252" s="2" t="inlineStr">
+        <is>
+          <t>6131.psd</t>
+        </is>
+      </c>
+      <c r="B252" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0252.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>6130.psd</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>tamilpsd-0253.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="2" t="inlineStr">
+        <is>
+          <t>6129.psd</t>
+        </is>
+      </c>
+      <c r="B254" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0254.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>6128.psd</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>tamilpsd-0255.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="2" t="inlineStr">
+        <is>
+          <t>6127.psd</t>
+        </is>
+      </c>
+      <c r="B256" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0256.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>6126.psd</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>tamilpsd-0257.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="2" t="inlineStr">
+        <is>
+          <t>6125.psd</t>
+        </is>
+      </c>
+      <c r="B258" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0258.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>6124.psd</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>tamilpsd-0259.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="2" t="inlineStr">
+        <is>
+          <t>6123.psd</t>
+        </is>
+      </c>
+      <c r="B260" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0260.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>6122.psd</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>tamilpsd-0261.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="2" t="inlineStr">
+        <is>
+          <t>6121.psd</t>
+        </is>
+      </c>
+      <c r="B262" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0262.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>6120.psd</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>tamilpsd-0263.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="2" t="inlineStr">
+        <is>
+          <t>6119.psd</t>
+        </is>
+      </c>
+      <c r="B264" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0264.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>6118.psd</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>tamilpsd-0265.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="2" t="inlineStr">
+        <is>
+          <t>6117.psd</t>
+        </is>
+      </c>
+      <c r="B266" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0266.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>6107.psd</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>tamilpsd-0267.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="2" t="inlineStr">
+        <is>
+          <t>6106.psd</t>
+        </is>
+      </c>
+      <c r="B268" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0268.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>6105.psd</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>tamilpsd-0269.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="2" t="inlineStr">
+        <is>
+          <t>6104.psd</t>
+        </is>
+      </c>
+      <c r="B270" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0270.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>6103.psd</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>tamilpsd-0271.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="2" t="inlineStr">
+        <is>
+          <t>6102.psd</t>
+        </is>
+      </c>
+      <c r="B272" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0272.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>6101.psd</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>tamilpsd-0273.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="2" t="inlineStr">
+        <is>
+          <t>6100.psd</t>
+        </is>
+      </c>
+      <c r="B274" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0274.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>6099.psd</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>tamilpsd-0275.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="2" t="inlineStr">
+        <is>
+          <t>6098.psd</t>
+        </is>
+      </c>
+      <c r="B276" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0276.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>6097.psd</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>tamilpsd-0277.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="2" t="inlineStr">
+        <is>
+          <t>6096.psd</t>
+        </is>
+      </c>
+      <c r="B278" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0278.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>6095.psd</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>tamilpsd-0279.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="2" t="inlineStr">
+        <is>
+          <t>6094.psd</t>
+        </is>
+      </c>
+      <c r="B280" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0280.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>6093.psd</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>tamilpsd-0281.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="2" t="inlineStr">
+        <is>
+          <t>6092.psd</t>
+        </is>
+      </c>
+      <c r="B282" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0282.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>6091.psd</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>tamilpsd-0283.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" s="2" t="inlineStr">
+        <is>
+          <t>6090.psd</t>
+        </is>
+      </c>
+      <c r="B284" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0284.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>6089.psd</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>tamilpsd-0285.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" s="2" t="inlineStr">
+        <is>
+          <t>6088.psd</t>
+        </is>
+      </c>
+      <c r="B286" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0286.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>6087.psd</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>tamilpsd-0287.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" s="2" t="inlineStr">
+        <is>
+          <t>6086.psd</t>
+        </is>
+      </c>
+      <c r="B288" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0288.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>6085.psd</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>tamilpsd-0289.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" s="2" t="inlineStr">
+        <is>
+          <t>6084.psd</t>
+        </is>
+      </c>
+      <c r="B290" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0290.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>6083.psd</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>tamilpsd-0291.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" s="2" t="inlineStr">
+        <is>
+          <t>6082.psd</t>
+        </is>
+      </c>
+      <c r="B292" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0292.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>6081.psd</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>tamilpsd-0293.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" s="2" t="inlineStr">
+        <is>
+          <t>6080.psd</t>
+        </is>
+      </c>
+      <c r="B294" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0294.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>6079.psd</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>tamilpsd-0295.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" s="2" t="inlineStr">
+        <is>
+          <t>6078.psd</t>
+        </is>
+      </c>
+      <c r="B296" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0296.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>6077.psd</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>tamilpsd-0297.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" s="2" t="inlineStr">
+        <is>
+          <t>6076.psd</t>
+        </is>
+      </c>
+      <c r="B298" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0298.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>6075.psd</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>tamilpsd-0299.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" s="2" t="inlineStr">
+        <is>
+          <t>6074.psd</t>
+        </is>
+      </c>
+      <c r="B300" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0300.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>6073.psd</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>tamilpsd-0301.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" s="2" t="inlineStr">
+        <is>
+          <t>6072.psd</t>
+        </is>
+      </c>
+      <c r="B302" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0302.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>6071.psd</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>tamilpsd-0303.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" s="2" t="inlineStr">
+        <is>
+          <t>6070.psd</t>
+        </is>
+      </c>
+      <c r="B304" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0304.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>6069.psd</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>tamilpsd-0305.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" s="2" t="inlineStr">
+        <is>
+          <t>6068.psd</t>
+        </is>
+      </c>
+      <c r="B306" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0306.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>6067.psd</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>tamilpsd-0307.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" s="2" t="inlineStr">
+        <is>
+          <t>6066.psd</t>
+        </is>
+      </c>
+      <c r="B308" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0308.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>6065.psd</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>tamilpsd-0309.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" s="2" t="inlineStr">
+        <is>
+          <t>6064.psd</t>
+        </is>
+      </c>
+      <c r="B310" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0310.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>6063.psd</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>tamilpsd-0311.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" s="2" t="inlineStr">
+        <is>
+          <t>6062.psd</t>
+        </is>
+      </c>
+      <c r="B312" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0312.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>6060.psd</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>tamilpsd-0313.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" s="2" t="inlineStr">
+        <is>
+          <t>6061.psd</t>
+        </is>
+      </c>
+      <c r="B314" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0314.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>6059.psd</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>tamilpsd-0315.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" s="2" t="inlineStr">
+        <is>
+          <t>6058.psd</t>
+        </is>
+      </c>
+      <c r="B316" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0316.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>6057.psd</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>tamilpsd-0317.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" s="2" t="inlineStr">
+        <is>
+          <t>6056.psd</t>
+        </is>
+      </c>
+      <c r="B318" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0318.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>6055.psd</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>tamilpsd-0319.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" s="2" t="inlineStr">
+        <is>
+          <t>6054.psd</t>
+        </is>
+      </c>
+      <c r="B320" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0320.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>6053.psd</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>tamilpsd-0321.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" s="2" t="inlineStr">
+        <is>
+          <t>6052.psd</t>
+        </is>
+      </c>
+      <c r="B322" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0322.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>6051.psd</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>tamilpsd-0323.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" s="2" t="inlineStr">
+        <is>
+          <t>6050.psd</t>
+        </is>
+      </c>
+      <c r="B324" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0324.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>6049.psd</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>tamilpsd-0325.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" s="2" t="inlineStr">
+        <is>
+          <t>6048.psd</t>
+        </is>
+      </c>
+      <c r="B326" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0326.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>6047.psd</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>tamilpsd-0327.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" s="2" t="inlineStr">
+        <is>
+          <t>6046.psd</t>
+        </is>
+      </c>
+      <c r="B328" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0328.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>6045.psd</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>tamilpsd-0329.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" s="2" t="inlineStr">
+        <is>
+          <t>6044.psd</t>
+        </is>
+      </c>
+      <c r="B330" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0330.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>6043.psd</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>tamilpsd-0331.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" s="2" t="inlineStr">
+        <is>
+          <t>6042.psd</t>
+        </is>
+      </c>
+      <c r="B332" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0332.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>6041.psd</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>tamilpsd-0333.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" s="2" t="inlineStr">
+        <is>
+          <t>6040.psd</t>
+        </is>
+      </c>
+      <c r="B334" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0334.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>6039.psd</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>tamilpsd-0335.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" s="2" t="inlineStr">
+        <is>
+          <t>6038.psd</t>
+        </is>
+      </c>
+      <c r="B336" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0336.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>6037.psd</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>tamilpsd-0337.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" s="2" t="inlineStr">
+        <is>
+          <t>6036.psd</t>
+        </is>
+      </c>
+      <c r="B338" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0338.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>6035.psd</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>tamilpsd-0339.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" s="2" t="inlineStr">
+        <is>
+          <t>6034.psd</t>
+        </is>
+      </c>
+      <c r="B340" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0340.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>6033.psd</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>tamilpsd-0341.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" s="2" t="inlineStr">
+        <is>
+          <t>6032.psd</t>
+        </is>
+      </c>
+      <c r="B342" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0342.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>6031.psd</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>tamilpsd-0343.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" s="2" t="inlineStr">
+        <is>
+          <t>6030.psd</t>
+        </is>
+      </c>
+      <c r="B344" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0344.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>6029.psd</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>tamilpsd-0345.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" s="2" t="inlineStr">
+        <is>
+          <t>6028.psd</t>
+        </is>
+      </c>
+      <c r="B346" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0346.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>6027.psd</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>tamilpsd-0347.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" s="2" t="inlineStr">
+        <is>
+          <t>6026.psd</t>
+        </is>
+      </c>
+      <c r="B348" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0348.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>6025.psd</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>tamilpsd-0349.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" s="2" t="inlineStr">
+        <is>
+          <t>6024.psd</t>
+        </is>
+      </c>
+      <c r="B350" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0350.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>6023.psd</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>tamilpsd-0351.psd</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
🤖 Progress: 2026-04-18 18:09 UTC
</commit_message>
<xml_diff>
--- a/rename_log.xlsx
+++ b/rename_log.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -474,6 +474,30 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>6362.psd</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0402.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>6361.psd</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>tamilpsd-0403.psd</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
🤖 Progress: 2026-04-18 18:19 UTC
</commit_message>
<xml_diff>
--- a/rename_log.xlsx
+++ b/rename_log.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -498,6 +498,126 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>6360.psd</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0404.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>6359.psd</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>tamilpsd-0405.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>6358.psd</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0406.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>6357.psd</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>tamilpsd-0407.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>6356.psd</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0408.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>6355.psd</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>tamilpsd-0409.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>6354.psd</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0410.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>6353.psd</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>tamilpsd-0411.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>6352.psd</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0412.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>6351.psd</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>tamilpsd-0413.psd</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
🤖 Progress: 2026-04-18 18:23 UTC
</commit_message>
<xml_diff>
--- a/rename_log.xlsx
+++ b/rename_log.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -618,6 +618,30 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>6350.psd</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0414.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>6349.psd</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>tamilpsd-0415.psd</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
🤖 Progress: 2026-04-19 06:44 UTC
</commit_message>
<xml_diff>
--- a/rename_log.xlsx
+++ b/rename_log.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -642,6 +642,234 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>6348.psd</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0815.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>6347.psd</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>tamilpsd-0816.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>6346.psd</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0817.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>6345.psd</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>tamilpsd-0818.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>6342.psd</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0819.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>6341.psd</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>tamilpsd-0820.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>6340.psd</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0821.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>6339.psd</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>tamilpsd-0822.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>6338.psd</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0823.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>6337.psd</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>tamilpsd-0824.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>6336.psd</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0825.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>6335.psd</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>tamilpsd-0826.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>6334.psd</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0827.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>6333.psd</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>tamilpsd-0828.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>6332.psd</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0829.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>6331.psd</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>tamilpsd-0830.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>6330.psd</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0831.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>6329.psd</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>tamilpsd-0832.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>6328.psd</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>tamilpsd-0833.psd</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
🤖 Progress: 2026-04-19 11:07 UTC
</commit_message>
<xml_diff>
--- a/rename_log.xlsx
+++ b/rename_log.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B136"/>
+  <dimension ref="A1:B550"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -1729,6 +1729,4974 @@
         </is>
       </c>
     </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>6226.psd</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>tamilpsd-0101.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="3" t="inlineStr">
+        <is>
+          <t>6225.psd</t>
+        </is>
+      </c>
+      <c r="B138" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0102.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>6224.psd</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>tamilpsd-0103.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="3" t="inlineStr">
+        <is>
+          <t>6223.psd</t>
+        </is>
+      </c>
+      <c r="B140" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0104.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>6222.psd</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>tamilpsd-0105.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="3" t="inlineStr">
+        <is>
+          <t>6221.psd</t>
+        </is>
+      </c>
+      <c r="B142" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0106.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>6220.psd</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>tamilpsd-0107.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="3" t="inlineStr">
+        <is>
+          <t>6219.psd</t>
+        </is>
+      </c>
+      <c r="B144" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0108.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>6218.psd</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>tamilpsd-0109.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="3" t="inlineStr">
+        <is>
+          <t>6217.psd</t>
+        </is>
+      </c>
+      <c r="B146" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0110.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>6216.psd</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>tamilpsd-0111.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="3" t="inlineStr">
+        <is>
+          <t>6215.psd</t>
+        </is>
+      </c>
+      <c r="B148" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0112.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>6214.psd</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>tamilpsd-0113.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="3" t="inlineStr">
+        <is>
+          <t>6213.psd</t>
+        </is>
+      </c>
+      <c r="B150" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0114.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>6212.psd</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>tamilpsd-0115.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="3" t="inlineStr">
+        <is>
+          <t>6211.psd</t>
+        </is>
+      </c>
+      <c r="B152" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0116.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>6210.psd</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>tamilpsd-0117.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="3" t="inlineStr">
+        <is>
+          <t>6209.psd</t>
+        </is>
+      </c>
+      <c r="B154" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0118.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>6208.psd</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>tamilpsd-0119.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="3" t="inlineStr">
+        <is>
+          <t>6207.psd</t>
+        </is>
+      </c>
+      <c r="B156" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0120.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>6206.psd</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>tamilpsd-0121.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="3" t="inlineStr">
+        <is>
+          <t>6205.psd</t>
+        </is>
+      </c>
+      <c r="B158" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0122.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>6203.psd</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>tamilpsd-0123.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="3" t="inlineStr">
+        <is>
+          <t>6202.psd</t>
+        </is>
+      </c>
+      <c r="B160" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0124.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>6201.psd</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>tamilpsd-0125.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="3" t="inlineStr">
+        <is>
+          <t>6200.psd</t>
+        </is>
+      </c>
+      <c r="B162" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0126.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>6199.psd</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>tamilpsd-0127.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="3" t="inlineStr">
+        <is>
+          <t>6198.psd</t>
+        </is>
+      </c>
+      <c r="B164" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0128.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>6197.psd</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>tamilpsd-0129.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="3" t="inlineStr">
+        <is>
+          <t>6196.psd</t>
+        </is>
+      </c>
+      <c r="B166" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0130.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>6195.psd</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>tamilpsd-0131.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="3" t="inlineStr">
+        <is>
+          <t>6194.psd</t>
+        </is>
+      </c>
+      <c r="B168" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0132.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>6193.psd</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>tamilpsd-0133.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="3" t="inlineStr">
+        <is>
+          <t>6192  This file is not suitable for photoshop 7.0 and cs3.psd</t>
+        </is>
+      </c>
+      <c r="B170" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0134.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>6188  This file is not suitable for photoshop 7.0 and cs3.psd</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>tamilpsd-0135.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="3" t="inlineStr">
+        <is>
+          <t>6187  This file is not suitable for photoshop 7.0 and cs3.psd</t>
+        </is>
+      </c>
+      <c r="B172" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0136.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>6185  This file is not suitable for photoshop 7.0 and cs3.psd</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>tamilpsd-0137.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="3" t="inlineStr">
+        <is>
+          <t>6184  This file is not suitable for photoshop 7.0 and cs3.psd</t>
+        </is>
+      </c>
+      <c r="B174" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0138.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>6183 This file is not suitable for photoshop 7.0 and cs3.psd</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>tamilpsd-0139.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="3" t="inlineStr">
+        <is>
+          <t>6240  This file is not suitable for photoshop 7.0 and cs3.psd</t>
+        </is>
+      </c>
+      <c r="B176" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0140.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>6346.psd</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>tamilpsd-0141.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="3" t="inlineStr">
+        <is>
+          <t>6345.psd</t>
+        </is>
+      </c>
+      <c r="B178" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0142.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>6344.psd</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>tamilpsd-0143.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="3" t="inlineStr">
+        <is>
+          <t>6343.psd</t>
+        </is>
+      </c>
+      <c r="B180" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0144.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>6342.psd</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>tamilpsd-0145.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="3" t="inlineStr">
+        <is>
+          <t>6341.psd</t>
+        </is>
+      </c>
+      <c r="B182" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0146.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>6340.psd</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>tamilpsd-0147.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="3" t="inlineStr">
+        <is>
+          <t>6339.psd</t>
+        </is>
+      </c>
+      <c r="B184" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0148.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>6338.psd</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>tamilpsd-0149.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="3" t="inlineStr">
+        <is>
+          <t>6337.psd</t>
+        </is>
+      </c>
+      <c r="B186" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0150.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>6336.psd</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>tamilpsd-0151.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="3" t="inlineStr">
+        <is>
+          <t>6335.psd</t>
+        </is>
+      </c>
+      <c r="B188" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0152.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>6334.psd</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>tamilpsd-0153.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="3" t="inlineStr">
+        <is>
+          <t>6333.psd</t>
+        </is>
+      </c>
+      <c r="B190" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0154.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>6332.psd</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>tamilpsd-0155.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="3" t="inlineStr">
+        <is>
+          <t>6331.psd</t>
+        </is>
+      </c>
+      <c r="B192" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0156.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>6330.psd</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>tamilpsd-0157.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="3" t="inlineStr">
+        <is>
+          <t>6329.psd</t>
+        </is>
+      </c>
+      <c r="B194" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0158.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>6328.psd</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>tamilpsd-0159.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="3" t="inlineStr">
+        <is>
+          <t>6308.psd</t>
+        </is>
+      </c>
+      <c r="B196" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0160.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>6302.psd</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>tamilpsd-0161.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="3" t="inlineStr">
+        <is>
+          <t>6301.psd</t>
+        </is>
+      </c>
+      <c r="B198" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0162.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>6299.psd</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>tamilpsd-0163.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="3" t="inlineStr">
+        <is>
+          <t>6298.psd</t>
+        </is>
+      </c>
+      <c r="B200" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0164.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>6297.psd</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>tamilpsd-0165.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="3" t="inlineStr">
+        <is>
+          <t>6296.psd</t>
+        </is>
+      </c>
+      <c r="B202" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0166.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>6295.psd</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>tamilpsd-0167.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="3" t="inlineStr">
+        <is>
+          <t>6294.psd</t>
+        </is>
+      </c>
+      <c r="B204" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0168.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>6293.psd</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>tamilpsd-0169.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="3" t="inlineStr">
+        <is>
+          <t>6292.psd</t>
+        </is>
+      </c>
+      <c r="B206" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0170.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>6291.psd</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>tamilpsd-0171.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="3" t="inlineStr">
+        <is>
+          <t>6290.psd</t>
+        </is>
+      </c>
+      <c r="B208" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0172.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>6289.psd</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>tamilpsd-0173.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="3" t="inlineStr">
+        <is>
+          <t>6288.psd</t>
+        </is>
+      </c>
+      <c r="B210" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0174.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>6287.psd</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>tamilpsd-0175.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="3" t="inlineStr">
+        <is>
+          <t>6286.psd</t>
+        </is>
+      </c>
+      <c r="B212" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0176.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>6285.psd</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>tamilpsd-0177.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="3" t="inlineStr">
+        <is>
+          <t>6284.psd</t>
+        </is>
+      </c>
+      <c r="B214" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0178.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>6283.psd</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>tamilpsd-0179.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="3" t="inlineStr">
+        <is>
+          <t>6282.psd</t>
+        </is>
+      </c>
+      <c r="B216" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0180.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>6281.psd</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>tamilpsd-0181.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="3" t="inlineStr">
+        <is>
+          <t>6280.psd</t>
+        </is>
+      </c>
+      <c r="B218" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0182.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>6279.psd</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>tamilpsd-0183.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="3" t="inlineStr">
+        <is>
+          <t>6278.psd</t>
+        </is>
+      </c>
+      <c r="B220" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0184.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>6277.psd</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>tamilpsd-0185.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="3" t="inlineStr">
+        <is>
+          <t>6205a.psd</t>
+        </is>
+      </c>
+      <c r="B222" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0186.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>6191.psd</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>tamilpsd-0187.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="3" t="inlineStr">
+        <is>
+          <t>6190.psd</t>
+        </is>
+      </c>
+      <c r="B224" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0188.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>6189.psd</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>tamilpsd-0189.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="3" t="inlineStr">
+        <is>
+          <t>6186.psd</t>
+        </is>
+      </c>
+      <c r="B226" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0190.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>6198 This file is not suitable for photoshop 7.0 and cs3.psd</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>tamilpsd-0191.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="3" t="inlineStr">
+        <is>
+          <t>6182.psd</t>
+        </is>
+      </c>
+      <c r="B228" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0192.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>6181.psd</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>tamilpsd-0193.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="3" t="inlineStr">
+        <is>
+          <t>6180.psd</t>
+        </is>
+      </c>
+      <c r="B230" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0194.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>6179.psd</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>tamilpsd-0195.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="3" t="inlineStr">
+        <is>
+          <t>6178.psd</t>
+        </is>
+      </c>
+      <c r="B232" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0196.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>6177.psd</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>tamilpsd-0197.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="3" t="inlineStr">
+        <is>
+          <t>6176.psd</t>
+        </is>
+      </c>
+      <c r="B234" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0198.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>6175.psd</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>tamilpsd-0199.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="3" t="inlineStr">
+        <is>
+          <t>6174.psd</t>
+        </is>
+      </c>
+      <c r="B236" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0200.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>6173.psd</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>tamilpsd-0201.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="3" t="inlineStr">
+        <is>
+          <t>6172.psd</t>
+        </is>
+      </c>
+      <c r="B238" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0202.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>6171.psd</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>tamilpsd-0203.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="3" t="inlineStr">
+        <is>
+          <t>6170.psd</t>
+        </is>
+      </c>
+      <c r="B240" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0204.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>6169.psd</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>tamilpsd-0205.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="3" t="inlineStr">
+        <is>
+          <t>6168.psd</t>
+        </is>
+      </c>
+      <c r="B242" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0206.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>6167.psd</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>tamilpsd-0207.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="3" t="inlineStr">
+        <is>
+          <t>6166.psd</t>
+        </is>
+      </c>
+      <c r="B244" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0208.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>6165.psd</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>tamilpsd-0209.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="3" t="inlineStr">
+        <is>
+          <t>6164.psd</t>
+        </is>
+      </c>
+      <c r="B246" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0210.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>6163.psd</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>tamilpsd-0211.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="3" t="inlineStr">
+        <is>
+          <t>6162.psd</t>
+        </is>
+      </c>
+      <c r="B248" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0212.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>6161.psd</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>tamilpsd-0213.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="3" t="inlineStr">
+        <is>
+          <t>6160.psd</t>
+        </is>
+      </c>
+      <c r="B250" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0214.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>6159.psd</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>tamilpsd-0215.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="3" t="inlineStr">
+        <is>
+          <t>6158.psd</t>
+        </is>
+      </c>
+      <c r="B252" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0216.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>6157.psd</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>tamilpsd-0217.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="3" t="inlineStr">
+        <is>
+          <t>6156.psd</t>
+        </is>
+      </c>
+      <c r="B254" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0218.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>6155.psd</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>tamilpsd-0219.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="3" t="inlineStr">
+        <is>
+          <t>6154.psd</t>
+        </is>
+      </c>
+      <c r="B256" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0220.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>6153.psd</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>tamilpsd-0221.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="3" t="inlineStr">
+        <is>
+          <t>6142.psd</t>
+        </is>
+      </c>
+      <c r="B258" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0222.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>6141.psd</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>tamilpsd-0223.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="3" t="inlineStr">
+        <is>
+          <t>6140.psd</t>
+        </is>
+      </c>
+      <c r="B260" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0224.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>6139.psd</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>tamilpsd-0225.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="3" t="inlineStr">
+        <is>
+          <t>6138.psd</t>
+        </is>
+      </c>
+      <c r="B262" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0226.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>6137.psd</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>tamilpsd-0227.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="3" t="inlineStr">
+        <is>
+          <t>6136.psd</t>
+        </is>
+      </c>
+      <c r="B264" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0228.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>6135.psd</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>tamilpsd-0229.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="3" t="inlineStr">
+        <is>
+          <t>6134.psd</t>
+        </is>
+      </c>
+      <c r="B266" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0230.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>6133.psd</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>tamilpsd-0231.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="3" t="inlineStr">
+        <is>
+          <t>6132.psd</t>
+        </is>
+      </c>
+      <c r="B268" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0232.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>6131.psd</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>tamilpsd-0233.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="3" t="inlineStr">
+        <is>
+          <t>6130.psd</t>
+        </is>
+      </c>
+      <c r="B270" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0234.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>6129.psd</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>tamilpsd-0235.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="3" t="inlineStr">
+        <is>
+          <t>6128.psd</t>
+        </is>
+      </c>
+      <c r="B272" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0236.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>6127.psd</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>tamilpsd-0237.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="3" t="inlineStr">
+        <is>
+          <t>6126.psd</t>
+        </is>
+      </c>
+      <c r="B274" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0238.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>6125.psd</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>tamilpsd-0239.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="3" t="inlineStr">
+        <is>
+          <t>6124.psd</t>
+        </is>
+      </c>
+      <c r="B276" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0240.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>6123.psd</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>tamilpsd-0241.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="3" t="inlineStr">
+        <is>
+          <t>6122.psd</t>
+        </is>
+      </c>
+      <c r="B278" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0242.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>6121.psd</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>tamilpsd-0243.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="3" t="inlineStr">
+        <is>
+          <t>6120.psd</t>
+        </is>
+      </c>
+      <c r="B280" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0244.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>6119.psd</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>tamilpsd-0245.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="3" t="inlineStr">
+        <is>
+          <t>6118.psd</t>
+        </is>
+      </c>
+      <c r="B282" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0246.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>6117.psd</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>tamilpsd-0247.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" s="3" t="inlineStr">
+        <is>
+          <t>6107.psd</t>
+        </is>
+      </c>
+      <c r="B284" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0248.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>6106.psd</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>tamilpsd-0249.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" s="3" t="inlineStr">
+        <is>
+          <t>6105.psd</t>
+        </is>
+      </c>
+      <c r="B286" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0250.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>6104.psd</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>tamilpsd-0251.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" s="3" t="inlineStr">
+        <is>
+          <t>6103.psd</t>
+        </is>
+      </c>
+      <c r="B288" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0252.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>6102.psd</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>tamilpsd-0253.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" s="3" t="inlineStr">
+        <is>
+          <t>6101.psd</t>
+        </is>
+      </c>
+      <c r="B290" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0254.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>6100.psd</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>tamilpsd-0255.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" s="3" t="inlineStr">
+        <is>
+          <t>6099.psd</t>
+        </is>
+      </c>
+      <c r="B292" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0256.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>6098.psd</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>tamilpsd-0257.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" s="3" t="inlineStr">
+        <is>
+          <t>6097.psd</t>
+        </is>
+      </c>
+      <c r="B294" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0258.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>6096.psd</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>tamilpsd-0259.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" s="3" t="inlineStr">
+        <is>
+          <t>6095.psd</t>
+        </is>
+      </c>
+      <c r="B296" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0260.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>6094.psd</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>tamilpsd-0261.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" s="3" t="inlineStr">
+        <is>
+          <t>6093.psd</t>
+        </is>
+      </c>
+      <c r="B298" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0262.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>6092.psd</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>tamilpsd-0263.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" s="3" t="inlineStr">
+        <is>
+          <t>6091.psd</t>
+        </is>
+      </c>
+      <c r="B300" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0264.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>6090.psd</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>tamilpsd-0265.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" s="3" t="inlineStr">
+        <is>
+          <t>6089.psd</t>
+        </is>
+      </c>
+      <c r="B302" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0266.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>6088.psd</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>tamilpsd-0267.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" s="3" t="inlineStr">
+        <is>
+          <t>6087.psd</t>
+        </is>
+      </c>
+      <c r="B304" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0268.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>6086.psd</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>tamilpsd-0269.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" s="3" t="inlineStr">
+        <is>
+          <t>6085.psd</t>
+        </is>
+      </c>
+      <c r="B306" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0270.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>6084.psd</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>tamilpsd-0271.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" s="3" t="inlineStr">
+        <is>
+          <t>6083.psd</t>
+        </is>
+      </c>
+      <c r="B308" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0272.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>6082.psd</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>tamilpsd-0273.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" s="3" t="inlineStr">
+        <is>
+          <t>6081.psd</t>
+        </is>
+      </c>
+      <c r="B310" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0274.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>6080.psd</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>tamilpsd-0275.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" s="3" t="inlineStr">
+        <is>
+          <t>6079.psd</t>
+        </is>
+      </c>
+      <c r="B312" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0276.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>6078.psd</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>tamilpsd-0277.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" s="3" t="inlineStr">
+        <is>
+          <t>6077.psd</t>
+        </is>
+      </c>
+      <c r="B314" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0278.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>6076.psd</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>tamilpsd-0279.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" s="3" t="inlineStr">
+        <is>
+          <t>6075.psd</t>
+        </is>
+      </c>
+      <c r="B316" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0280.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>6074.psd</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>tamilpsd-0281.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" s="3" t="inlineStr">
+        <is>
+          <t>6073.psd</t>
+        </is>
+      </c>
+      <c r="B318" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0282.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>6072.psd</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>tamilpsd-0283.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" s="3" t="inlineStr">
+        <is>
+          <t>6071.psd</t>
+        </is>
+      </c>
+      <c r="B320" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0284.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>6070.psd</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>tamilpsd-0285.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" s="3" t="inlineStr">
+        <is>
+          <t>6069.psd</t>
+        </is>
+      </c>
+      <c r="B322" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0286.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>6068.psd</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>tamilpsd-0287.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" s="3" t="inlineStr">
+        <is>
+          <t>6067.psd</t>
+        </is>
+      </c>
+      <c r="B324" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0288.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>6066.psd</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>tamilpsd-0289.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" s="3" t="inlineStr">
+        <is>
+          <t>6065.psd</t>
+        </is>
+      </c>
+      <c r="B326" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0290.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>6064.psd</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>tamilpsd-0291.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" s="3" t="inlineStr">
+        <is>
+          <t>6063.psd</t>
+        </is>
+      </c>
+      <c r="B328" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0292.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>6062.psd</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>tamilpsd-0293.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" s="3" t="inlineStr">
+        <is>
+          <t>6060.psd</t>
+        </is>
+      </c>
+      <c r="B330" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0294.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>6061.psd</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>tamilpsd-0295.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" s="3" t="inlineStr">
+        <is>
+          <t>6059.psd</t>
+        </is>
+      </c>
+      <c r="B332" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0296.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>6058.psd</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>tamilpsd-0297.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" s="3" t="inlineStr">
+        <is>
+          <t>6057.psd</t>
+        </is>
+      </c>
+      <c r="B334" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0298.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>6056.psd</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>tamilpsd-0299.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" s="3" t="inlineStr">
+        <is>
+          <t>6055.psd</t>
+        </is>
+      </c>
+      <c r="B336" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0300.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>6054.psd</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>tamilpsd-0301.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" s="3" t="inlineStr">
+        <is>
+          <t>6053.psd</t>
+        </is>
+      </c>
+      <c r="B338" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0302.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>6052.psd</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>tamilpsd-0303.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" s="3" t="inlineStr">
+        <is>
+          <t>6051.psd</t>
+        </is>
+      </c>
+      <c r="B340" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0304.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>6050.psd</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>tamilpsd-0305.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" s="3" t="inlineStr">
+        <is>
+          <t>6049.psd</t>
+        </is>
+      </c>
+      <c r="B342" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0306.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>6048.psd</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>tamilpsd-0307.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" s="3" t="inlineStr">
+        <is>
+          <t>6047.psd</t>
+        </is>
+      </c>
+      <c r="B344" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0308.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>6046.psd</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>tamilpsd-0309.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" s="3" t="inlineStr">
+        <is>
+          <t>6045.psd</t>
+        </is>
+      </c>
+      <c r="B346" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0310.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>6044.psd</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>tamilpsd-0311.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" s="3" t="inlineStr">
+        <is>
+          <t>6043.psd</t>
+        </is>
+      </c>
+      <c r="B348" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0312.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>6042.psd</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>tamilpsd-0313.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" s="3" t="inlineStr">
+        <is>
+          <t>6041.psd</t>
+        </is>
+      </c>
+      <c r="B350" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0314.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>6040.psd</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>tamilpsd-0315.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" s="3" t="inlineStr">
+        <is>
+          <t>6039.psd</t>
+        </is>
+      </c>
+      <c r="B352" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0316.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>6038.psd</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>tamilpsd-0317.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" s="3" t="inlineStr">
+        <is>
+          <t>6037.psd</t>
+        </is>
+      </c>
+      <c r="B354" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0318.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>6036.psd</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>tamilpsd-0319.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" s="3" t="inlineStr">
+        <is>
+          <t>6035.psd</t>
+        </is>
+      </c>
+      <c r="B356" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0320.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>6034.psd</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>tamilpsd-0321.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" s="3" t="inlineStr">
+        <is>
+          <t>6033.psd</t>
+        </is>
+      </c>
+      <c r="B358" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0322.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>6032.psd</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>tamilpsd-0323.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" s="3" t="inlineStr">
+        <is>
+          <t>6031.psd</t>
+        </is>
+      </c>
+      <c r="B360" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0324.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>6030.psd</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>tamilpsd-0325.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" s="3" t="inlineStr">
+        <is>
+          <t>6029.psd</t>
+        </is>
+      </c>
+      <c r="B362" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0326.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>6028.psd</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>tamilpsd-0327.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" s="3" t="inlineStr">
+        <is>
+          <t>6027.psd</t>
+        </is>
+      </c>
+      <c r="B364" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0328.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>6026.psd</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>tamilpsd-0329.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" s="3" t="inlineStr">
+        <is>
+          <t>6025.psd</t>
+        </is>
+      </c>
+      <c r="B366" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0330.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>6024.psd</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>tamilpsd-0331.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" s="3" t="inlineStr">
+        <is>
+          <t>6023.psd</t>
+        </is>
+      </c>
+      <c r="B368" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0332.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>6022.psd</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>tamilpsd-0333.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" s="3" t="inlineStr">
+        <is>
+          <t>6021.psd</t>
+        </is>
+      </c>
+      <c r="B370" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0334.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>6020.psd</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>tamilpsd-0335.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" s="3" t="inlineStr">
+        <is>
+          <t>6019.psd</t>
+        </is>
+      </c>
+      <c r="B372" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0336.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>6018.psd</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>tamilpsd-0337.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" s="3" t="inlineStr">
+        <is>
+          <t>6017.psd</t>
+        </is>
+      </c>
+      <c r="B374" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0338.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>6016.psd</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>tamilpsd-0339.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" s="3" t="inlineStr">
+        <is>
+          <t>6015.psd</t>
+        </is>
+      </c>
+      <c r="B376" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0340.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>6014.psd</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>tamilpsd-0341.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" s="3" t="inlineStr">
+        <is>
+          <t>6013.psd</t>
+        </is>
+      </c>
+      <c r="B378" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0342.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>6012.psd</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>tamilpsd-0343.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" s="3" t="inlineStr">
+        <is>
+          <t>6011.psd</t>
+        </is>
+      </c>
+      <c r="B380" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0344.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>6010.psd</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>tamilpsd-0345.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" s="3" t="inlineStr">
+        <is>
+          <t>6009.psd</t>
+        </is>
+      </c>
+      <c r="B382" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0346.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>6008.psd</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>tamilpsd-0347.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" s="3" t="inlineStr">
+        <is>
+          <t>6007.psd</t>
+        </is>
+      </c>
+      <c r="B384" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0348.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>6006.psd</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>tamilpsd-0349.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" s="3" t="inlineStr">
+        <is>
+          <t>6005.psd</t>
+        </is>
+      </c>
+      <c r="B386" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0350.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>6004.psd</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>tamilpsd-0351.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" s="3" t="inlineStr">
+        <is>
+          <t>6003.psd</t>
+        </is>
+      </c>
+      <c r="B388" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0352.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>6002.psd</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>tamilpsd-0353.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" s="3" t="inlineStr">
+        <is>
+          <t>6001.psd</t>
+        </is>
+      </c>
+      <c r="B390" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0354.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>6000.psd</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>tamilpsd-0355.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" s="3" t="inlineStr">
+        <is>
+          <t>5999.psd</t>
+        </is>
+      </c>
+      <c r="B392" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0356.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>5997.psd</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>tamilpsd-0357.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" s="3" t="inlineStr">
+        <is>
+          <t>5996.psd</t>
+        </is>
+      </c>
+      <c r="B394" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0358.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>5995.psd</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>tamilpsd-0359.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" s="3" t="inlineStr">
+        <is>
+          <t>5994.psd</t>
+        </is>
+      </c>
+      <c r="B396" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0360.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>5993.psd</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>tamilpsd-0361.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" s="3" t="inlineStr">
+        <is>
+          <t>5992.psd</t>
+        </is>
+      </c>
+      <c r="B398" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0362.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>5991.psd</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>tamilpsd-0363.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" s="3" t="inlineStr">
+        <is>
+          <t>5990.psd</t>
+        </is>
+      </c>
+      <c r="B400" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0364.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>5989.psd</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>tamilpsd-0365.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" s="3" t="inlineStr">
+        <is>
+          <t>5988.psd</t>
+        </is>
+      </c>
+      <c r="B402" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0366.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>5987.psd</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>tamilpsd-0367.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" s="3" t="inlineStr">
+        <is>
+          <t>5986.psd</t>
+        </is>
+      </c>
+      <c r="B404" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0368.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>5985.psd</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>tamilpsd-0369.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" s="3" t="inlineStr">
+        <is>
+          <t>5983.psd</t>
+        </is>
+      </c>
+      <c r="B406" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0370.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>5982.psd</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>tamilpsd-0371.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" s="3" t="inlineStr">
+        <is>
+          <t>5981.psd</t>
+        </is>
+      </c>
+      <c r="B408" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0372.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>5980.psd</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>tamilpsd-0373.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" s="3" t="inlineStr">
+        <is>
+          <t>5979.psd</t>
+        </is>
+      </c>
+      <c r="B410" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0374.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>5978.psd</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>tamilpsd-0375.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" s="3" t="inlineStr">
+        <is>
+          <t>5977.psd</t>
+        </is>
+      </c>
+      <c r="B412" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0376.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>5976.psd</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>tamilpsd-0377.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" s="3" t="inlineStr">
+        <is>
+          <t>5975.psd</t>
+        </is>
+      </c>
+      <c r="B414" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0378.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>5974.psd</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>tamilpsd-0379.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" s="3" t="inlineStr">
+        <is>
+          <t>5973.psd</t>
+        </is>
+      </c>
+      <c r="B416" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0380.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>5972.psd</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>tamilpsd-0381.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" s="3" t="inlineStr">
+        <is>
+          <t>5971.psd</t>
+        </is>
+      </c>
+      <c r="B418" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0382.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>5970.psd</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>tamilpsd-0383.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" s="3" t="inlineStr">
+        <is>
+          <t>5969.psd</t>
+        </is>
+      </c>
+      <c r="B420" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0384.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>5968.psd</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>tamilpsd-0385.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" s="3" t="inlineStr">
+        <is>
+          <t>5967.psd</t>
+        </is>
+      </c>
+      <c r="B422" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0386.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>5966.psd</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>tamilpsd-0387.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" s="3" t="inlineStr">
+        <is>
+          <t>5965.psd</t>
+        </is>
+      </c>
+      <c r="B424" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0388.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>5964.psd</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>tamilpsd-0389.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" s="3" t="inlineStr">
+        <is>
+          <t>5963.psd</t>
+        </is>
+      </c>
+      <c r="B426" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0390.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>5962.psd</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>tamilpsd-0391.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" s="3" t="inlineStr">
+        <is>
+          <t>5961.psd</t>
+        </is>
+      </c>
+      <c r="B428" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0392.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>5960.psd</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>tamilpsd-0393.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" s="3" t="inlineStr">
+        <is>
+          <t>5959.psd</t>
+        </is>
+      </c>
+      <c r="B430" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0394.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>5958.psd</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>tamilpsd-0395.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" s="3" t="inlineStr">
+        <is>
+          <t>5957.psd</t>
+        </is>
+      </c>
+      <c r="B432" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0396.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>5956.psd</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>tamilpsd-0397.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" s="3" t="inlineStr">
+        <is>
+          <t>5955.psd</t>
+        </is>
+      </c>
+      <c r="B434" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0398.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>5954.psd</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>tamilpsd-0399.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" s="3" t="inlineStr">
+        <is>
+          <t>5953.psd</t>
+        </is>
+      </c>
+      <c r="B436" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0400.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>5952.psd</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>tamilpsd-0401.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" s="3" t="inlineStr">
+        <is>
+          <t>5951.psd</t>
+        </is>
+      </c>
+      <c r="B438" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0402.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>5950.psd</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>tamilpsd-0403.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" s="3" t="inlineStr">
+        <is>
+          <t>5949.psd</t>
+        </is>
+      </c>
+      <c r="B440" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0404.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>5948.psd</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>tamilpsd-0405.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" s="3" t="inlineStr">
+        <is>
+          <t>5947.psd</t>
+        </is>
+      </c>
+      <c r="B442" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0406.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>5945.psd</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>tamilpsd-0407.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" s="3" t="inlineStr">
+        <is>
+          <t>5944.psd</t>
+        </is>
+      </c>
+      <c r="B444" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0408.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>5943.psd</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>tamilpsd-0409.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" s="3" t="inlineStr">
+        <is>
+          <t>5942.psd</t>
+        </is>
+      </c>
+      <c r="B446" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0410.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>5941.psd</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>tamilpsd-0411.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" s="3" t="inlineStr">
+        <is>
+          <t>5940.psd</t>
+        </is>
+      </c>
+      <c r="B448" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0412.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>5939.psd</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>tamilpsd-0413.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" s="3" t="inlineStr">
+        <is>
+          <t>5938.psd</t>
+        </is>
+      </c>
+      <c r="B450" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0414.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>5937.psd</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>tamilpsd-0415.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" s="3" t="inlineStr">
+        <is>
+          <t>5936.psd</t>
+        </is>
+      </c>
+      <c r="B452" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0416.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>5935.psd</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>tamilpsd-0417.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" s="3" t="inlineStr">
+        <is>
+          <t>5934.psd</t>
+        </is>
+      </c>
+      <c r="B454" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0418.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>5933.psd</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>tamilpsd-0419.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" s="3" t="inlineStr">
+        <is>
+          <t>5932.psd</t>
+        </is>
+      </c>
+      <c r="B456" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0420.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>5930.psd</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>tamilpsd-0421.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" s="3" t="inlineStr">
+        <is>
+          <t>5931.psd</t>
+        </is>
+      </c>
+      <c r="B458" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0422.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>5929.psd</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>tamilpsd-0423.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" s="3" t="inlineStr">
+        <is>
+          <t>5927.psd</t>
+        </is>
+      </c>
+      <c r="B460" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0424.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>5928.psd</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>tamilpsd-0425.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" s="3" t="inlineStr">
+        <is>
+          <t>5924.psd</t>
+        </is>
+      </c>
+      <c r="B462" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0426.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>5925.psd</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>tamilpsd-0427.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" s="3" t="inlineStr">
+        <is>
+          <t>5926.psd</t>
+        </is>
+      </c>
+      <c r="B464" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0428.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>5922.psd</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>tamilpsd-0429.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" s="3" t="inlineStr">
+        <is>
+          <t>5923.psd</t>
+        </is>
+      </c>
+      <c r="B466" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0430.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>5921.psd</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>tamilpsd-0431.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" s="3" t="inlineStr">
+        <is>
+          <t>5920.psd</t>
+        </is>
+      </c>
+      <c r="B468" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0432.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>5919.psd</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>tamilpsd-0433.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" s="3" t="inlineStr">
+        <is>
+          <t>5918.psd</t>
+        </is>
+      </c>
+      <c r="B470" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0434.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>5917.psd</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>tamilpsd-0435.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" s="3" t="inlineStr">
+        <is>
+          <t>5916.psd</t>
+        </is>
+      </c>
+      <c r="B472" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0436.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>5915.psd</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>tamilpsd-0437.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" s="3" t="inlineStr">
+        <is>
+          <t>5914.psd</t>
+        </is>
+      </c>
+      <c r="B474" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0438.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>5912.psd</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>tamilpsd-0439.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" s="3" t="inlineStr">
+        <is>
+          <t>5911.psd</t>
+        </is>
+      </c>
+      <c r="B476" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0440.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>5910.psd</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>tamilpsd-0441.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" s="3" t="inlineStr">
+        <is>
+          <t>5913.psd</t>
+        </is>
+      </c>
+      <c r="B478" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0442.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>5907.psd</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>tamilpsd-0443.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" s="3" t="inlineStr">
+        <is>
+          <t>5908.psd</t>
+        </is>
+      </c>
+      <c r="B480" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0444.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>5909.psd</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>tamilpsd-0445.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" s="3" t="inlineStr">
+        <is>
+          <t>5904.psd</t>
+        </is>
+      </c>
+      <c r="B482" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0446.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>5906.psd</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>tamilpsd-0447.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" s="3" t="inlineStr">
+        <is>
+          <t>5905.psd</t>
+        </is>
+      </c>
+      <c r="B484" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0448.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>5903.psd</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>tamilpsd-0449.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" s="3" t="inlineStr">
+        <is>
+          <t>5902.psd</t>
+        </is>
+      </c>
+      <c r="B486" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0450.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>5901.psd</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>tamilpsd-0451.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" s="3" t="inlineStr">
+        <is>
+          <t>5900.psd</t>
+        </is>
+      </c>
+      <c r="B488" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0452.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>5899.psd</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>tamilpsd-0453.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" s="3" t="inlineStr">
+        <is>
+          <t>5897.psd</t>
+        </is>
+      </c>
+      <c r="B490" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0454.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>5898.psd</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>tamilpsd-0455.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" s="3" t="inlineStr">
+        <is>
+          <t>5896.psd</t>
+        </is>
+      </c>
+      <c r="B492" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0456.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>5894.psd</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>tamilpsd-0457.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" s="3" t="inlineStr">
+        <is>
+          <t>5895.psd</t>
+        </is>
+      </c>
+      <c r="B494" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0458.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>5893.psd</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>tamilpsd-0459.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" s="3" t="inlineStr">
+        <is>
+          <t>5891.psd</t>
+        </is>
+      </c>
+      <c r="B496" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0460.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>5892.psd</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>tamilpsd-0461.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" s="3" t="inlineStr">
+        <is>
+          <t>5890.psd</t>
+        </is>
+      </c>
+      <c r="B498" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0462.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>5888.psd</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>tamilpsd-0463.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" s="3" t="inlineStr">
+        <is>
+          <t>5889.psd</t>
+        </is>
+      </c>
+      <c r="B500" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0464.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>5886.psd</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>tamilpsd-0465.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" s="3" t="inlineStr">
+        <is>
+          <t>5887.psd</t>
+        </is>
+      </c>
+      <c r="B502" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0466.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>5882.psd</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>tamilpsd-0467.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" s="3" t="inlineStr">
+        <is>
+          <t>5885.psd</t>
+        </is>
+      </c>
+      <c r="B504" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0468.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>5883.psd</t>
+        </is>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>tamilpsd-0469.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" s="3" t="inlineStr">
+        <is>
+          <t>5884.psd</t>
+        </is>
+      </c>
+      <c r="B506" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0470.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>5876.psd</t>
+        </is>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>tamilpsd-0471.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" s="3" t="inlineStr">
+        <is>
+          <t>5881.psd</t>
+        </is>
+      </c>
+      <c r="B508" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0472.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="inlineStr">
+        <is>
+          <t>5880.psd</t>
+        </is>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>tamilpsd-0473.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" s="3" t="inlineStr">
+        <is>
+          <t>5879.psd</t>
+        </is>
+      </c>
+      <c r="B510" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0474.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>5878.psd</t>
+        </is>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>tamilpsd-0475.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" s="3" t="inlineStr">
+        <is>
+          <t>5877.psd</t>
+        </is>
+      </c>
+      <c r="B512" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0476.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>5874.psd</t>
+        </is>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>tamilpsd-0477.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" s="3" t="inlineStr">
+        <is>
+          <t>5873.psd</t>
+        </is>
+      </c>
+      <c r="B514" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0478.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>5875.psd</t>
+        </is>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>tamilpsd-0479.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" s="3" t="inlineStr">
+        <is>
+          <t>5872.psd</t>
+        </is>
+      </c>
+      <c r="B516" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0480.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>5863.psd</t>
+        </is>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>tamilpsd-0481.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" s="3" t="inlineStr">
+        <is>
+          <t>5866.psd</t>
+        </is>
+      </c>
+      <c r="B518" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0482.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>5864.psd</t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>tamilpsd-0483.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" s="3" t="inlineStr">
+        <is>
+          <t>5871.psd</t>
+        </is>
+      </c>
+      <c r="B520" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0484.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t>5870.psd</t>
+        </is>
+      </c>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>tamilpsd-0485.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" s="3" t="inlineStr">
+        <is>
+          <t>5868.psd</t>
+        </is>
+      </c>
+      <c r="B522" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0486.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>5867.psd</t>
+        </is>
+      </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>tamilpsd-0487.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" s="3" t="inlineStr">
+        <is>
+          <t>5865.psd</t>
+        </is>
+      </c>
+      <c r="B524" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0488.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="inlineStr">
+        <is>
+          <t>5869.psd</t>
+        </is>
+      </c>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>tamilpsd-0489.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" s="3" t="inlineStr">
+        <is>
+          <t>5857.psd</t>
+        </is>
+      </c>
+      <c r="B526" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0490.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="inlineStr">
+        <is>
+          <t>5859.psd</t>
+        </is>
+      </c>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>tamilpsd-0491.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" s="3" t="inlineStr">
+        <is>
+          <t>5862.psd</t>
+        </is>
+      </c>
+      <c r="B528" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0492.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="inlineStr">
+        <is>
+          <t>5861.psd</t>
+        </is>
+      </c>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>tamilpsd-0493.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" s="3" t="inlineStr">
+        <is>
+          <t>5860.psd</t>
+        </is>
+      </c>
+      <c r="B530" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0494.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="inlineStr">
+        <is>
+          <t>5858.psd</t>
+        </is>
+      </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>tamilpsd-0495.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" s="3" t="inlineStr">
+        <is>
+          <t>5851.psd</t>
+        </is>
+      </c>
+      <c r="B532" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0496.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="inlineStr">
+        <is>
+          <t>5852.psd</t>
+        </is>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>tamilpsd-0497.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" s="3" t="inlineStr">
+        <is>
+          <t>5853.psd</t>
+        </is>
+      </c>
+      <c r="B534" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0498.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" t="inlineStr">
+        <is>
+          <t>5850.psd</t>
+        </is>
+      </c>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>tamilpsd-0499.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" s="3" t="inlineStr">
+        <is>
+          <t>5854.psd</t>
+        </is>
+      </c>
+      <c r="B536" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0500.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="inlineStr">
+        <is>
+          <t>5855.psd</t>
+        </is>
+      </c>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>tamilpsd-0501.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" s="3" t="inlineStr">
+        <is>
+          <t>5856.psd</t>
+        </is>
+      </c>
+      <c r="B538" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0502.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" t="inlineStr">
+        <is>
+          <t>5848.psd</t>
+        </is>
+      </c>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>tamilpsd-0503.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" s="3" t="inlineStr">
+        <is>
+          <t>5849.psd</t>
+        </is>
+      </c>
+      <c r="B540" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0504.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" t="inlineStr">
+        <is>
+          <t>5846.psd</t>
+        </is>
+      </c>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>tamilpsd-0505.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" s="3" t="inlineStr">
+        <is>
+          <t>5847.psd</t>
+        </is>
+      </c>
+      <c r="B542" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0506.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" t="inlineStr">
+        <is>
+          <t>5845.psd</t>
+        </is>
+      </c>
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>tamilpsd-0507.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" s="3" t="inlineStr">
+        <is>
+          <t>5843.psd</t>
+        </is>
+      </c>
+      <c r="B544" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0508.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="inlineStr">
+        <is>
+          <t>5842.psd</t>
+        </is>
+      </c>
+      <c r="B545" t="inlineStr">
+        <is>
+          <t>tamilpsd-0509.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" s="3" t="inlineStr">
+        <is>
+          <t>5840.psd</t>
+        </is>
+      </c>
+      <c r="B546" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0510.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>5838.psd</t>
+        </is>
+      </c>
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>tamilpsd-0511.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" s="3" t="inlineStr">
+        <is>
+          <t>5839.psd</t>
+        </is>
+      </c>
+      <c r="B548" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0512.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="inlineStr">
+        <is>
+          <t>5837.psd</t>
+        </is>
+      </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>tamilpsd-0513.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" s="3" t="inlineStr">
+        <is>
+          <t>5841.psd</t>
+        </is>
+      </c>
+      <c r="B550" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-0514.psd</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
🤖 Progress: 2026-04-19 18:01 UTC
</commit_message>
<xml_diff>
--- a/rename_log.xlsx
+++ b/rename_log.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2049"/>
+  <dimension ref="A1:B2325"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -24685,6 +24685,3318 @@
         </is>
       </c>
     </row>
+    <row r="2050">
+      <c r="A2050" s="3" t="inlineStr">
+        <is>
+          <t>5406.psd</t>
+        </is>
+      </c>
+      <c r="B2050" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2017.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2051">
+      <c r="A2051" t="inlineStr">
+        <is>
+          <t>4950.psd</t>
+        </is>
+      </c>
+      <c r="B2051" t="inlineStr">
+        <is>
+          <t>tamilpsd-2018.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2052">
+      <c r="A2052" s="3" t="inlineStr">
+        <is>
+          <t>4803.psd</t>
+        </is>
+      </c>
+      <c r="B2052" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2019.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2053">
+      <c r="A2053" t="inlineStr">
+        <is>
+          <t>4802.psd</t>
+        </is>
+      </c>
+      <c r="B2053" t="inlineStr">
+        <is>
+          <t>tamilpsd-2020.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2054">
+      <c r="A2054" s="3" t="inlineStr">
+        <is>
+          <t>4801.PSD</t>
+        </is>
+      </c>
+      <c r="B2054" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2021.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2055">
+      <c r="A2055" t="inlineStr">
+        <is>
+          <t>4800.psd</t>
+        </is>
+      </c>
+      <c r="B2055" t="inlineStr">
+        <is>
+          <t>tamilpsd-2022.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2056">
+      <c r="A2056" s="3" t="inlineStr">
+        <is>
+          <t>4799.psd</t>
+        </is>
+      </c>
+      <c r="B2056" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2023.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2057">
+      <c r="A2057" t="inlineStr">
+        <is>
+          <t>4798.psd</t>
+        </is>
+      </c>
+      <c r="B2057" t="inlineStr">
+        <is>
+          <t>tamilpsd-2024.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2058">
+      <c r="A2058" s="3" t="inlineStr">
+        <is>
+          <t>4797.PSD</t>
+        </is>
+      </c>
+      <c r="B2058" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2025.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2059">
+      <c r="A2059" t="inlineStr">
+        <is>
+          <t>4796.psd</t>
+        </is>
+      </c>
+      <c r="B2059" t="inlineStr">
+        <is>
+          <t>tamilpsd-2026.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2060">
+      <c r="A2060" s="3" t="inlineStr">
+        <is>
+          <t>4795.psd</t>
+        </is>
+      </c>
+      <c r="B2060" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2027.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2061">
+      <c r="A2061" t="inlineStr">
+        <is>
+          <t>4794.psd</t>
+        </is>
+      </c>
+      <c r="B2061" t="inlineStr">
+        <is>
+          <t>tamilpsd-2028.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2062">
+      <c r="A2062" s="3" t="inlineStr">
+        <is>
+          <t>4793.psd</t>
+        </is>
+      </c>
+      <c r="B2062" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2029.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2063">
+      <c r="A2063" t="inlineStr">
+        <is>
+          <t>4792.psd</t>
+        </is>
+      </c>
+      <c r="B2063" t="inlineStr">
+        <is>
+          <t>tamilpsd-2030.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2064">
+      <c r="A2064" s="3" t="inlineStr">
+        <is>
+          <t>4791.psd</t>
+        </is>
+      </c>
+      <c r="B2064" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2031.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2065">
+      <c r="A2065" t="inlineStr">
+        <is>
+          <t>4790.psd</t>
+        </is>
+      </c>
+      <c r="B2065" t="inlineStr">
+        <is>
+          <t>tamilpsd-2032.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2066">
+      <c r="A2066" s="3" t="inlineStr">
+        <is>
+          <t>4789.psd</t>
+        </is>
+      </c>
+      <c r="B2066" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2033.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2067">
+      <c r="A2067" t="inlineStr">
+        <is>
+          <t>4788.PSD</t>
+        </is>
+      </c>
+      <c r="B2067" t="inlineStr">
+        <is>
+          <t>tamilpsd-2034.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2068">
+      <c r="A2068" s="3" t="inlineStr">
+        <is>
+          <t>4787.PSD</t>
+        </is>
+      </c>
+      <c r="B2068" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2035.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2069">
+      <c r="A2069" t="inlineStr">
+        <is>
+          <t>4786.psd</t>
+        </is>
+      </c>
+      <c r="B2069" t="inlineStr">
+        <is>
+          <t>tamilpsd-2036.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2070">
+      <c r="A2070" s="3" t="inlineStr">
+        <is>
+          <t>4785.psd</t>
+        </is>
+      </c>
+      <c r="B2070" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2037.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2071">
+      <c r="A2071" t="inlineStr">
+        <is>
+          <t>4784.psd</t>
+        </is>
+      </c>
+      <c r="B2071" t="inlineStr">
+        <is>
+          <t>tamilpsd-2038.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2072">
+      <c r="A2072" s="3" t="inlineStr">
+        <is>
+          <t>4783.psd</t>
+        </is>
+      </c>
+      <c r="B2072" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2039.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2073">
+      <c r="A2073" t="inlineStr">
+        <is>
+          <t>4782.psd</t>
+        </is>
+      </c>
+      <c r="B2073" t="inlineStr">
+        <is>
+          <t>tamilpsd-2040.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2074">
+      <c r="A2074" s="3" t="inlineStr">
+        <is>
+          <t>4763.psd</t>
+        </is>
+      </c>
+      <c r="B2074" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2041.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2075">
+      <c r="A2075" t="inlineStr">
+        <is>
+          <t>4762.psd</t>
+        </is>
+      </c>
+      <c r="B2075" t="inlineStr">
+        <is>
+          <t>tamilpsd-2042.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2076">
+      <c r="A2076" s="3" t="inlineStr">
+        <is>
+          <t>4761.psd</t>
+        </is>
+      </c>
+      <c r="B2076" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2043.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2077">
+      <c r="A2077" t="inlineStr">
+        <is>
+          <t>4760.psd</t>
+        </is>
+      </c>
+      <c r="B2077" t="inlineStr">
+        <is>
+          <t>tamilpsd-2044.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2078">
+      <c r="A2078" s="3" t="inlineStr">
+        <is>
+          <t>4759.psd</t>
+        </is>
+      </c>
+      <c r="B2078" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2045.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2079">
+      <c r="A2079" t="inlineStr">
+        <is>
+          <t>4758.psd</t>
+        </is>
+      </c>
+      <c r="B2079" t="inlineStr">
+        <is>
+          <t>tamilpsd-2046.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2080">
+      <c r="A2080" s="3" t="inlineStr">
+        <is>
+          <t>4757.psd</t>
+        </is>
+      </c>
+      <c r="B2080" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2047.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2081">
+      <c r="A2081" t="inlineStr">
+        <is>
+          <t>4756.psd</t>
+        </is>
+      </c>
+      <c r="B2081" t="inlineStr">
+        <is>
+          <t>tamilpsd-2048.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2082">
+      <c r="A2082" s="3" t="inlineStr">
+        <is>
+          <t>4755.psd</t>
+        </is>
+      </c>
+      <c r="B2082" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2049.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2083">
+      <c r="A2083" t="inlineStr">
+        <is>
+          <t>4754.psd</t>
+        </is>
+      </c>
+      <c r="B2083" t="inlineStr">
+        <is>
+          <t>tamilpsd-2050.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2084">
+      <c r="A2084" s="3" t="inlineStr">
+        <is>
+          <t>4753.psd</t>
+        </is>
+      </c>
+      <c r="B2084" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2051.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2085">
+      <c r="A2085" t="inlineStr">
+        <is>
+          <t>4752.psd</t>
+        </is>
+      </c>
+      <c r="B2085" t="inlineStr">
+        <is>
+          <t>tamilpsd-2052.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2086">
+      <c r="A2086" s="3" t="inlineStr">
+        <is>
+          <t>4751.psd</t>
+        </is>
+      </c>
+      <c r="B2086" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2053.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2087">
+      <c r="A2087" t="inlineStr">
+        <is>
+          <t>4750.psd</t>
+        </is>
+      </c>
+      <c r="B2087" t="inlineStr">
+        <is>
+          <t>tamilpsd-2054.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2088">
+      <c r="A2088" s="3" t="inlineStr">
+        <is>
+          <t>4749.psd</t>
+        </is>
+      </c>
+      <c r="B2088" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2055.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2089">
+      <c r="A2089" t="inlineStr">
+        <is>
+          <t>4748.psd</t>
+        </is>
+      </c>
+      <c r="B2089" t="inlineStr">
+        <is>
+          <t>tamilpsd-2056.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2090">
+      <c r="A2090" s="3" t="inlineStr">
+        <is>
+          <t>4747.psd</t>
+        </is>
+      </c>
+      <c r="B2090" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2057.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2091">
+      <c r="A2091" t="inlineStr">
+        <is>
+          <t>4746.psd</t>
+        </is>
+      </c>
+      <c r="B2091" t="inlineStr">
+        <is>
+          <t>tamilpsd-2058.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2092">
+      <c r="A2092" s="3" t="inlineStr">
+        <is>
+          <t>4745.psd</t>
+        </is>
+      </c>
+      <c r="B2092" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2059.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2093">
+      <c r="A2093" t="inlineStr">
+        <is>
+          <t>4744.psd</t>
+        </is>
+      </c>
+      <c r="B2093" t="inlineStr">
+        <is>
+          <t>tamilpsd-2060.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2094">
+      <c r="A2094" s="3" t="inlineStr">
+        <is>
+          <t>4743.psd</t>
+        </is>
+      </c>
+      <c r="B2094" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2061.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2095">
+      <c r="A2095" t="inlineStr">
+        <is>
+          <t>4742.psd</t>
+        </is>
+      </c>
+      <c r="B2095" t="inlineStr">
+        <is>
+          <t>tamilpsd-2062.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2096">
+      <c r="A2096" s="3" t="inlineStr">
+        <is>
+          <t>4741.psd</t>
+        </is>
+      </c>
+      <c r="B2096" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2063.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2097">
+      <c r="A2097" t="inlineStr">
+        <is>
+          <t>4740.psd</t>
+        </is>
+      </c>
+      <c r="B2097" t="inlineStr">
+        <is>
+          <t>tamilpsd-2064.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2098">
+      <c r="A2098" s="3" t="inlineStr">
+        <is>
+          <t>4739.psd</t>
+        </is>
+      </c>
+      <c r="B2098" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2065.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2099">
+      <c r="A2099" t="inlineStr">
+        <is>
+          <t>4738.psd</t>
+        </is>
+      </c>
+      <c r="B2099" t="inlineStr">
+        <is>
+          <t>tamilpsd-2066.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2100">
+      <c r="A2100" s="3" t="inlineStr">
+        <is>
+          <t>4737.psd</t>
+        </is>
+      </c>
+      <c r="B2100" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2067.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2101">
+      <c r="A2101" t="inlineStr">
+        <is>
+          <t>4736.psd</t>
+        </is>
+      </c>
+      <c r="B2101" t="inlineStr">
+        <is>
+          <t>tamilpsd-2068.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2102">
+      <c r="A2102" s="3" t="inlineStr">
+        <is>
+          <t>4735.psd</t>
+        </is>
+      </c>
+      <c r="B2102" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2069.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2103">
+      <c r="A2103" t="inlineStr">
+        <is>
+          <t>4734.psd</t>
+        </is>
+      </c>
+      <c r="B2103" t="inlineStr">
+        <is>
+          <t>tamilpsd-2070.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2104">
+      <c r="A2104" s="3" t="inlineStr">
+        <is>
+          <t>4733.psd</t>
+        </is>
+      </c>
+      <c r="B2104" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2071.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2105">
+      <c r="A2105" t="inlineStr">
+        <is>
+          <t>4732.psd</t>
+        </is>
+      </c>
+      <c r="B2105" t="inlineStr">
+        <is>
+          <t>tamilpsd-2072.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2106">
+      <c r="A2106" s="3" t="inlineStr">
+        <is>
+          <t>4731.psd</t>
+        </is>
+      </c>
+      <c r="B2106" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2073.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2107">
+      <c r="A2107" t="inlineStr">
+        <is>
+          <t>4730.psd</t>
+        </is>
+      </c>
+      <c r="B2107" t="inlineStr">
+        <is>
+          <t>tamilpsd-2074.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2108">
+      <c r="A2108" s="3" t="inlineStr">
+        <is>
+          <t>4729.psd</t>
+        </is>
+      </c>
+      <c r="B2108" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2075.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2109">
+      <c r="A2109" t="inlineStr">
+        <is>
+          <t>4728.psd</t>
+        </is>
+      </c>
+      <c r="B2109" t="inlineStr">
+        <is>
+          <t>tamilpsd-2076.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2110">
+      <c r="A2110" s="3" t="inlineStr">
+        <is>
+          <t>4727.psd</t>
+        </is>
+      </c>
+      <c r="B2110" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2077.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2111">
+      <c r="A2111" t="inlineStr">
+        <is>
+          <t>4726.psd</t>
+        </is>
+      </c>
+      <c r="B2111" t="inlineStr">
+        <is>
+          <t>tamilpsd-2078.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2112">
+      <c r="A2112" s="3" t="inlineStr">
+        <is>
+          <t>4725.psd</t>
+        </is>
+      </c>
+      <c r="B2112" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2079.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2113">
+      <c r="A2113" t="inlineStr">
+        <is>
+          <t>4724.psd</t>
+        </is>
+      </c>
+      <c r="B2113" t="inlineStr">
+        <is>
+          <t>tamilpsd-2080.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2114">
+      <c r="A2114" s="3" t="inlineStr">
+        <is>
+          <t>4723.psd</t>
+        </is>
+      </c>
+      <c r="B2114" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2081.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2115">
+      <c r="A2115" t="inlineStr">
+        <is>
+          <t>4722.psd</t>
+        </is>
+      </c>
+      <c r="B2115" t="inlineStr">
+        <is>
+          <t>tamilpsd-2082.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2116">
+      <c r="A2116" s="3" t="inlineStr">
+        <is>
+          <t>4721.psd</t>
+        </is>
+      </c>
+      <c r="B2116" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2083.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2117">
+      <c r="A2117" t="inlineStr">
+        <is>
+          <t>4720.psd</t>
+        </is>
+      </c>
+      <c r="B2117" t="inlineStr">
+        <is>
+          <t>tamilpsd-2084.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2118">
+      <c r="A2118" s="3" t="inlineStr">
+        <is>
+          <t>4719.psd</t>
+        </is>
+      </c>
+      <c r="B2118" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2085.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2119">
+      <c r="A2119" t="inlineStr">
+        <is>
+          <t>4718.psd</t>
+        </is>
+      </c>
+      <c r="B2119" t="inlineStr">
+        <is>
+          <t>tamilpsd-2086.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2120">
+      <c r="A2120" s="3" t="inlineStr">
+        <is>
+          <t>4717.psd</t>
+        </is>
+      </c>
+      <c r="B2120" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2087.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2121">
+      <c r="A2121" t="inlineStr">
+        <is>
+          <t>4716.psd</t>
+        </is>
+      </c>
+      <c r="B2121" t="inlineStr">
+        <is>
+          <t>tamilpsd-2088.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2122">
+      <c r="A2122" s="3" t="inlineStr">
+        <is>
+          <t>4715.psd</t>
+        </is>
+      </c>
+      <c r="B2122" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2089.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2123">
+      <c r="A2123" t="inlineStr">
+        <is>
+          <t>4714.psd</t>
+        </is>
+      </c>
+      <c r="B2123" t="inlineStr">
+        <is>
+          <t>tamilpsd-2090.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2124">
+      <c r="A2124" s="3" t="inlineStr">
+        <is>
+          <t>4713.psd</t>
+        </is>
+      </c>
+      <c r="B2124" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2091.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2125">
+      <c r="A2125" t="inlineStr">
+        <is>
+          <t>4712.psd</t>
+        </is>
+      </c>
+      <c r="B2125" t="inlineStr">
+        <is>
+          <t>tamilpsd-2092.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2126">
+      <c r="A2126" s="3" t="inlineStr">
+        <is>
+          <t>4711.psd</t>
+        </is>
+      </c>
+      <c r="B2126" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2093.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2127">
+      <c r="A2127" t="inlineStr">
+        <is>
+          <t>4710.psd</t>
+        </is>
+      </c>
+      <c r="B2127" t="inlineStr">
+        <is>
+          <t>tamilpsd-2094.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2128">
+      <c r="A2128" s="3" t="inlineStr">
+        <is>
+          <t>4709.psd</t>
+        </is>
+      </c>
+      <c r="B2128" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2095.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2129">
+      <c r="A2129" t="inlineStr">
+        <is>
+          <t>4708.psd</t>
+        </is>
+      </c>
+      <c r="B2129" t="inlineStr">
+        <is>
+          <t>tamilpsd-2096.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2130">
+      <c r="A2130" s="3" t="inlineStr">
+        <is>
+          <t>4707.psd</t>
+        </is>
+      </c>
+      <c r="B2130" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2097.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2131">
+      <c r="A2131" t="inlineStr">
+        <is>
+          <t>4706.psd</t>
+        </is>
+      </c>
+      <c r="B2131" t="inlineStr">
+        <is>
+          <t>tamilpsd-2098.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2132">
+      <c r="A2132" s="3" t="inlineStr">
+        <is>
+          <t>4705.psd</t>
+        </is>
+      </c>
+      <c r="B2132" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2099.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2133">
+      <c r="A2133" t="inlineStr">
+        <is>
+          <t>4704.psd</t>
+        </is>
+      </c>
+      <c r="B2133" t="inlineStr">
+        <is>
+          <t>tamilpsd-2100.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2134">
+      <c r="A2134" s="3" t="inlineStr">
+        <is>
+          <t>4703.psd</t>
+        </is>
+      </c>
+      <c r="B2134" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2101.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2135">
+      <c r="A2135" t="inlineStr">
+        <is>
+          <t>4702.psd</t>
+        </is>
+      </c>
+      <c r="B2135" t="inlineStr">
+        <is>
+          <t>tamilpsd-2102.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2136">
+      <c r="A2136" s="3" t="inlineStr">
+        <is>
+          <t>4701.psd</t>
+        </is>
+      </c>
+      <c r="B2136" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2103.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2137">
+      <c r="A2137" t="inlineStr">
+        <is>
+          <t>4700.psd</t>
+        </is>
+      </c>
+      <c r="B2137" t="inlineStr">
+        <is>
+          <t>tamilpsd-2104.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2138">
+      <c r="A2138" s="3" t="inlineStr">
+        <is>
+          <t>4699.psd</t>
+        </is>
+      </c>
+      <c r="B2138" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2105.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2139">
+      <c r="A2139" t="inlineStr">
+        <is>
+          <t>4698.psd</t>
+        </is>
+      </c>
+      <c r="B2139" t="inlineStr">
+        <is>
+          <t>tamilpsd-2106.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2140">
+      <c r="A2140" s="3" t="inlineStr">
+        <is>
+          <t>4697.psd</t>
+        </is>
+      </c>
+      <c r="B2140" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2107.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2141">
+      <c r="A2141" t="inlineStr">
+        <is>
+          <t>4696.psd</t>
+        </is>
+      </c>
+      <c r="B2141" t="inlineStr">
+        <is>
+          <t>tamilpsd-2108.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2142">
+      <c r="A2142" s="3" t="inlineStr">
+        <is>
+          <t>4695.psd</t>
+        </is>
+      </c>
+      <c r="B2142" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2109.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2143">
+      <c r="A2143" t="inlineStr">
+        <is>
+          <t>4694.psd</t>
+        </is>
+      </c>
+      <c r="B2143" t="inlineStr">
+        <is>
+          <t>tamilpsd-2110.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2144">
+      <c r="A2144" s="3" t="inlineStr">
+        <is>
+          <t>4693.psd</t>
+        </is>
+      </c>
+      <c r="B2144" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2111.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2145">
+      <c r="A2145" t="inlineStr">
+        <is>
+          <t>4692.psd</t>
+        </is>
+      </c>
+      <c r="B2145" t="inlineStr">
+        <is>
+          <t>tamilpsd-2112.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2146">
+      <c r="A2146" s="3" t="inlineStr">
+        <is>
+          <t>4691.psd</t>
+        </is>
+      </c>
+      <c r="B2146" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2113.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2147">
+      <c r="A2147" t="inlineStr">
+        <is>
+          <t>4690.psd</t>
+        </is>
+      </c>
+      <c r="B2147" t="inlineStr">
+        <is>
+          <t>tamilpsd-2114.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2148">
+      <c r="A2148" s="3" t="inlineStr">
+        <is>
+          <t>4689.psd</t>
+        </is>
+      </c>
+      <c r="B2148" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2115.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2149">
+      <c r="A2149" t="inlineStr">
+        <is>
+          <t>4688.psd</t>
+        </is>
+      </c>
+      <c r="B2149" t="inlineStr">
+        <is>
+          <t>tamilpsd-2116.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2150">
+      <c r="A2150" s="3" t="inlineStr">
+        <is>
+          <t>4687.psd</t>
+        </is>
+      </c>
+      <c r="B2150" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2117.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2151">
+      <c r="A2151" t="inlineStr">
+        <is>
+          <t>4686.psd</t>
+        </is>
+      </c>
+      <c r="B2151" t="inlineStr">
+        <is>
+          <t>tamilpsd-2118.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2152">
+      <c r="A2152" s="3" t="inlineStr">
+        <is>
+          <t>4685.psd</t>
+        </is>
+      </c>
+      <c r="B2152" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2119.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2153">
+      <c r="A2153" t="inlineStr">
+        <is>
+          <t>4684.psd</t>
+        </is>
+      </c>
+      <c r="B2153" t="inlineStr">
+        <is>
+          <t>tamilpsd-2120.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2154">
+      <c r="A2154" s="3" t="inlineStr">
+        <is>
+          <t>4683.psd</t>
+        </is>
+      </c>
+      <c r="B2154" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2121.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2155">
+      <c r="A2155" t="inlineStr">
+        <is>
+          <t>4682.psd</t>
+        </is>
+      </c>
+      <c r="B2155" t="inlineStr">
+        <is>
+          <t>tamilpsd-2122.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2156">
+      <c r="A2156" s="3" t="inlineStr">
+        <is>
+          <t>4681.psd</t>
+        </is>
+      </c>
+      <c r="B2156" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2123.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2157">
+      <c r="A2157" t="inlineStr">
+        <is>
+          <t>4680.psd</t>
+        </is>
+      </c>
+      <c r="B2157" t="inlineStr">
+        <is>
+          <t>tamilpsd-2124.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2158">
+      <c r="A2158" s="3" t="inlineStr">
+        <is>
+          <t>4679.psd</t>
+        </is>
+      </c>
+      <c r="B2158" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2125.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2159">
+      <c r="A2159" t="inlineStr">
+        <is>
+          <t>4678.psd</t>
+        </is>
+      </c>
+      <c r="B2159" t="inlineStr">
+        <is>
+          <t>tamilpsd-2126.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2160">
+      <c r="A2160" s="3" t="inlineStr">
+        <is>
+          <t>4677.psd</t>
+        </is>
+      </c>
+      <c r="B2160" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2127.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2161">
+      <c r="A2161" t="inlineStr">
+        <is>
+          <t>4676.psd</t>
+        </is>
+      </c>
+      <c r="B2161" t="inlineStr">
+        <is>
+          <t>tamilpsd-2128.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2162">
+      <c r="A2162" s="3" t="inlineStr">
+        <is>
+          <t>4675.psd</t>
+        </is>
+      </c>
+      <c r="B2162" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2129.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2163">
+      <c r="A2163" t="inlineStr">
+        <is>
+          <t>4674.psd</t>
+        </is>
+      </c>
+      <c r="B2163" t="inlineStr">
+        <is>
+          <t>tamilpsd-2130.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2164">
+      <c r="A2164" s="3" t="inlineStr">
+        <is>
+          <t>4673.psd</t>
+        </is>
+      </c>
+      <c r="B2164" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2131.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2165">
+      <c r="A2165" t="inlineStr">
+        <is>
+          <t>4672.psd</t>
+        </is>
+      </c>
+      <c r="B2165" t="inlineStr">
+        <is>
+          <t>tamilpsd-2132.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2166">
+      <c r="A2166" s="3" t="inlineStr">
+        <is>
+          <t>4671.psd</t>
+        </is>
+      </c>
+      <c r="B2166" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2133.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2167">
+      <c r="A2167" t="inlineStr">
+        <is>
+          <t>4670.psd</t>
+        </is>
+      </c>
+      <c r="B2167" t="inlineStr">
+        <is>
+          <t>tamilpsd-2134.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2168">
+      <c r="A2168" s="3" t="inlineStr">
+        <is>
+          <t>4780.psd</t>
+        </is>
+      </c>
+      <c r="B2168" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2135.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2169">
+      <c r="A2169" t="inlineStr">
+        <is>
+          <t>4778.psd</t>
+        </is>
+      </c>
+      <c r="B2169" t="inlineStr">
+        <is>
+          <t>tamilpsd-2136.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2170">
+      <c r="A2170" s="3" t="inlineStr">
+        <is>
+          <t>4779.psd</t>
+        </is>
+      </c>
+      <c r="B2170" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2137.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2171">
+      <c r="A2171" t="inlineStr">
+        <is>
+          <t>4777.psd</t>
+        </is>
+      </c>
+      <c r="B2171" t="inlineStr">
+        <is>
+          <t>tamilpsd-2138.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2172">
+      <c r="A2172" s="3" t="inlineStr">
+        <is>
+          <t>4776.psd</t>
+        </is>
+      </c>
+      <c r="B2172" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2139.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2173">
+      <c r="A2173" t="inlineStr">
+        <is>
+          <t>4775.psd</t>
+        </is>
+      </c>
+      <c r="B2173" t="inlineStr">
+        <is>
+          <t>tamilpsd-2140.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2174">
+      <c r="A2174" s="3" t="inlineStr">
+        <is>
+          <t>4774.psd</t>
+        </is>
+      </c>
+      <c r="B2174" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2141.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2175">
+      <c r="A2175" t="inlineStr">
+        <is>
+          <t>4773.psd</t>
+        </is>
+      </c>
+      <c r="B2175" t="inlineStr">
+        <is>
+          <t>tamilpsd-2142.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2176">
+      <c r="A2176" s="3" t="inlineStr">
+        <is>
+          <t>4772.psd</t>
+        </is>
+      </c>
+      <c r="B2176" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2143.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2177">
+      <c r="A2177" t="inlineStr">
+        <is>
+          <t>4771.psd</t>
+        </is>
+      </c>
+      <c r="B2177" t="inlineStr">
+        <is>
+          <t>tamilpsd-2144.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2178">
+      <c r="A2178" s="3" t="inlineStr">
+        <is>
+          <t>4770.psd</t>
+        </is>
+      </c>
+      <c r="B2178" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2145.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2179">
+      <c r="A2179" t="inlineStr">
+        <is>
+          <t>4769.psd</t>
+        </is>
+      </c>
+      <c r="B2179" t="inlineStr">
+        <is>
+          <t>tamilpsd-2146.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2180">
+      <c r="A2180" s="3" t="inlineStr">
+        <is>
+          <t>4768.psd</t>
+        </is>
+      </c>
+      <c r="B2180" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2147.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2181">
+      <c r="A2181" t="inlineStr">
+        <is>
+          <t>4767.psd</t>
+        </is>
+      </c>
+      <c r="B2181" t="inlineStr">
+        <is>
+          <t>tamilpsd-2148.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2182">
+      <c r="A2182" s="3" t="inlineStr">
+        <is>
+          <t>4766.psd</t>
+        </is>
+      </c>
+      <c r="B2182" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2149.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2183">
+      <c r="A2183" t="inlineStr">
+        <is>
+          <t>4765.psd</t>
+        </is>
+      </c>
+      <c r="B2183" t="inlineStr">
+        <is>
+          <t>tamilpsd-2150.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2184">
+      <c r="A2184" s="3" t="inlineStr">
+        <is>
+          <t>4764.psd</t>
+        </is>
+      </c>
+      <c r="B2184" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2151.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2185">
+      <c r="A2185" t="inlineStr">
+        <is>
+          <t>4461.psd</t>
+        </is>
+      </c>
+      <c r="B2185" t="inlineStr">
+        <is>
+          <t>tamilpsd-2152.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2186">
+      <c r="A2186" s="3" t="inlineStr">
+        <is>
+          <t>017.psd</t>
+        </is>
+      </c>
+      <c r="B2186" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2153.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2187">
+      <c r="A2187" t="inlineStr">
+        <is>
+          <t>018.psd</t>
+        </is>
+      </c>
+      <c r="B2187" t="inlineStr">
+        <is>
+          <t>tamilpsd-2154.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2188">
+      <c r="A2188" s="3" t="inlineStr">
+        <is>
+          <t>019.psd</t>
+        </is>
+      </c>
+      <c r="B2188" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2155.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2189">
+      <c r="A2189" t="inlineStr">
+        <is>
+          <t>020.psd</t>
+        </is>
+      </c>
+      <c r="B2189" t="inlineStr">
+        <is>
+          <t>tamilpsd-2156.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2190">
+      <c r="A2190" s="3" t="inlineStr">
+        <is>
+          <t>021.psd</t>
+        </is>
+      </c>
+      <c r="B2190" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2157.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2191">
+      <c r="A2191" t="inlineStr">
+        <is>
+          <t>022.psd</t>
+        </is>
+      </c>
+      <c r="B2191" t="inlineStr">
+        <is>
+          <t>tamilpsd-2158.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2192">
+      <c r="A2192" s="3" t="inlineStr">
+        <is>
+          <t>023.psd</t>
+        </is>
+      </c>
+      <c r="B2192" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2159.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2193">
+      <c r="A2193" t="inlineStr">
+        <is>
+          <t>024.psd</t>
+        </is>
+      </c>
+      <c r="B2193" t="inlineStr">
+        <is>
+          <t>tamilpsd-2160.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2194">
+      <c r="A2194" s="3" t="inlineStr">
+        <is>
+          <t>025.psd</t>
+        </is>
+      </c>
+      <c r="B2194" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2161.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2195">
+      <c r="A2195" t="inlineStr">
+        <is>
+          <t>009.psd</t>
+        </is>
+      </c>
+      <c r="B2195" t="inlineStr">
+        <is>
+          <t>tamilpsd-2162.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2196">
+      <c r="A2196" s="3" t="inlineStr">
+        <is>
+          <t>010.psd</t>
+        </is>
+      </c>
+      <c r="B2196" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2163.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2197">
+      <c r="A2197" t="inlineStr">
+        <is>
+          <t>011.psd</t>
+        </is>
+      </c>
+      <c r="B2197" t="inlineStr">
+        <is>
+          <t>tamilpsd-2164.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2198">
+      <c r="A2198" s="3" t="inlineStr">
+        <is>
+          <t>012.psd</t>
+        </is>
+      </c>
+      <c r="B2198" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2165.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2199">
+      <c r="A2199" t="inlineStr">
+        <is>
+          <t>013.psd</t>
+        </is>
+      </c>
+      <c r="B2199" t="inlineStr">
+        <is>
+          <t>tamilpsd-2166.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2200">
+      <c r="A2200" s="3" t="inlineStr">
+        <is>
+          <t>014.psd</t>
+        </is>
+      </c>
+      <c r="B2200" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2167.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2201">
+      <c r="A2201" t="inlineStr">
+        <is>
+          <t>015.psd</t>
+        </is>
+      </c>
+      <c r="B2201" t="inlineStr">
+        <is>
+          <t>tamilpsd-2168.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2202">
+      <c r="A2202" s="3" t="inlineStr">
+        <is>
+          <t>016.psd</t>
+        </is>
+      </c>
+      <c r="B2202" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2169.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2203">
+      <c r="A2203" t="inlineStr">
+        <is>
+          <t>RC Design 12x36 (31).psd</t>
+        </is>
+      </c>
+      <c r="B2203" t="inlineStr">
+        <is>
+          <t>tamilpsd-2170.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2204">
+      <c r="A2204" s="3" t="inlineStr">
+        <is>
+          <t>RC Design 12x36 (32).psd</t>
+        </is>
+      </c>
+      <c r="B2204" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2171.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2205">
+      <c r="A2205" t="inlineStr">
+        <is>
+          <t>RC Design 12x36 (33).psd</t>
+        </is>
+      </c>
+      <c r="B2205" t="inlineStr">
+        <is>
+          <t>tamilpsd-2172.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2206">
+      <c r="A2206" s="3" t="inlineStr">
+        <is>
+          <t>RC Design 12x36 (34).psd</t>
+        </is>
+      </c>
+      <c r="B2206" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2173.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2207">
+      <c r="A2207" t="inlineStr">
+        <is>
+          <t>RC Design 12x36 (35).psd</t>
+        </is>
+      </c>
+      <c r="B2207" t="inlineStr">
+        <is>
+          <t>tamilpsd-2174.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2208">
+      <c r="A2208" s="3" t="inlineStr">
+        <is>
+          <t>RC Design 12x36 (36).psd</t>
+        </is>
+      </c>
+      <c r="B2208" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2175.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2209">
+      <c r="A2209" t="inlineStr">
+        <is>
+          <t>RC Design 12x36 (37).psd</t>
+        </is>
+      </c>
+      <c r="B2209" t="inlineStr">
+        <is>
+          <t>tamilpsd-2176.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2210">
+      <c r="A2210" s="3" t="inlineStr">
+        <is>
+          <t>RC Design 12x36 (38).psd</t>
+        </is>
+      </c>
+      <c r="B2210" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2177.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2211">
+      <c r="A2211" t="inlineStr">
+        <is>
+          <t>RC Design 12x36 (39).psd</t>
+        </is>
+      </c>
+      <c r="B2211" t="inlineStr">
+        <is>
+          <t>tamilpsd-2178.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2212">
+      <c r="A2212" s="3" t="inlineStr">
+        <is>
+          <t>RC Design 12x36 (40).psd</t>
+        </is>
+      </c>
+      <c r="B2212" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2179.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2213">
+      <c r="A2213" t="inlineStr">
+        <is>
+          <t>RC Design 12x36 (26).psd</t>
+        </is>
+      </c>
+      <c r="B2213" t="inlineStr">
+        <is>
+          <t>tamilpsd-2185.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2214">
+      <c r="A2214" s="3" t="inlineStr">
+        <is>
+          <t>RC Design 12x36 (27).psd</t>
+        </is>
+      </c>
+      <c r="B2214" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2186.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2215">
+      <c r="A2215" t="inlineStr">
+        <is>
+          <t>RC Design 12x36 (28).psd</t>
+        </is>
+      </c>
+      <c r="B2215" t="inlineStr">
+        <is>
+          <t>tamilpsd-2187.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2216">
+      <c r="A2216" s="3" t="inlineStr">
+        <is>
+          <t>RC Design 12x36 (29).psd</t>
+        </is>
+      </c>
+      <c r="B2216" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2188.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2217">
+      <c r="A2217" t="inlineStr">
+        <is>
+          <t>RC Design 12x36 (30).psd</t>
+        </is>
+      </c>
+      <c r="B2217" t="inlineStr">
+        <is>
+          <t>tamilpsd-2189.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2218">
+      <c r="A2218" s="3" t="inlineStr">
+        <is>
+          <t>RC Design 12 x 36 (1).psd</t>
+        </is>
+      </c>
+      <c r="B2218" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2190.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2219">
+      <c r="A2219" t="inlineStr">
+        <is>
+          <t>RC Design 12 x 36 (2).psd</t>
+        </is>
+      </c>
+      <c r="B2219" t="inlineStr">
+        <is>
+          <t>tamilpsd-2191.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2220">
+      <c r="A2220" s="3" t="inlineStr">
+        <is>
+          <t>RC Design 12 x 36 (3).psd</t>
+        </is>
+      </c>
+      <c r="B2220" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2192.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2221">
+      <c r="A2221" t="inlineStr">
+        <is>
+          <t>RC Design 12 x 36 (4).psd</t>
+        </is>
+      </c>
+      <c r="B2221" t="inlineStr">
+        <is>
+          <t>tamilpsd-2193.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2222">
+      <c r="A2222" s="3" t="inlineStr">
+        <is>
+          <t>RC Design 12 x 36 (5).psd</t>
+        </is>
+      </c>
+      <c r="B2222" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2194.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2223">
+      <c r="A2223" t="inlineStr">
+        <is>
+          <t>RC Design 12 x 36 (6).psd</t>
+        </is>
+      </c>
+      <c r="B2223" t="inlineStr">
+        <is>
+          <t>tamilpsd-2195.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2224">
+      <c r="A2224" s="3" t="inlineStr">
+        <is>
+          <t>RC Desing 12x36 (1).psd</t>
+        </is>
+      </c>
+      <c r="B2224" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2196.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2225">
+      <c r="A2225" t="inlineStr">
+        <is>
+          <t>RC Desing 12x36 (2).psd</t>
+        </is>
+      </c>
+      <c r="B2225" t="inlineStr">
+        <is>
+          <t>tamilpsd-2197.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2226">
+      <c r="A2226" s="3" t="inlineStr">
+        <is>
+          <t>RC Desing 12x36 (3).psd</t>
+        </is>
+      </c>
+      <c r="B2226" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2198.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2227">
+      <c r="A2227" t="inlineStr">
+        <is>
+          <t>RC Desing 12x36 (4).psd</t>
+        </is>
+      </c>
+      <c r="B2227" t="inlineStr">
+        <is>
+          <t>tamilpsd-2199.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2228">
+      <c r="A2228" s="3" t="inlineStr">
+        <is>
+          <t>RC Desing 12x36 (5).psd</t>
+        </is>
+      </c>
+      <c r="B2228" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2200.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2229">
+      <c r="A2229" t="inlineStr">
+        <is>
+          <t>RC Desing 12x36 (6).psd</t>
+        </is>
+      </c>
+      <c r="B2229" t="inlineStr">
+        <is>
+          <t>tamilpsd-2201.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2230">
+      <c r="A2230" s="3" t="inlineStr">
+        <is>
+          <t>RC Desing 12x36 (7).psd</t>
+        </is>
+      </c>
+      <c r="B2230" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2202.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2231">
+      <c r="A2231" t="inlineStr">
+        <is>
+          <t>RC Desing 12x36 (10).psd</t>
+        </is>
+      </c>
+      <c r="B2231" t="inlineStr">
+        <is>
+          <t>tamilpsd-2203.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2232">
+      <c r="A2232" s="3" t="inlineStr">
+        <is>
+          <t>RC Desing 12x36 (11).psd</t>
+        </is>
+      </c>
+      <c r="B2232" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2204.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2233">
+      <c r="A2233" t="inlineStr">
+        <is>
+          <t>RC Desing 12x36 (12).psd</t>
+        </is>
+      </c>
+      <c r="B2233" t="inlineStr">
+        <is>
+          <t>tamilpsd-2205.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2234">
+      <c r="A2234" s="3" t="inlineStr">
+        <is>
+          <t>RC Desing 12x36 (13).psd</t>
+        </is>
+      </c>
+      <c r="B2234" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2206.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2235">
+      <c r="A2235" t="inlineStr">
+        <is>
+          <t>RC Desing 12x36 (14).psd</t>
+        </is>
+      </c>
+      <c r="B2235" t="inlineStr">
+        <is>
+          <t>tamilpsd-2207.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2236">
+      <c r="A2236" s="3" t="inlineStr">
+        <is>
+          <t>RC Desing 12x36 (8).psd</t>
+        </is>
+      </c>
+      <c r="B2236" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2208.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2237">
+      <c r="A2237" t="inlineStr">
+        <is>
+          <t>RC Desing 12x36 (9).psd</t>
+        </is>
+      </c>
+      <c r="B2237" t="inlineStr">
+        <is>
+          <t>tamilpsd-2209.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2238">
+      <c r="A2238" s="3" t="inlineStr">
+        <is>
+          <t>DMAX LIVE VOL 242 (1).psd</t>
+        </is>
+      </c>
+      <c r="B2238" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2210.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2239">
+      <c r="A2239" t="inlineStr">
+        <is>
+          <t>DMAX LIVE VOL 242 (2).psd</t>
+        </is>
+      </c>
+      <c r="B2239" t="inlineStr">
+        <is>
+          <t>tamilpsd-2211.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2240">
+      <c r="A2240" s="3" t="inlineStr">
+        <is>
+          <t>DMAX LIVE VOL 242 (3).psd</t>
+        </is>
+      </c>
+      <c r="B2240" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2212.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2241">
+      <c r="A2241" t="inlineStr">
+        <is>
+          <t>DMAX LIVE VOL 242 (4).psd</t>
+        </is>
+      </c>
+      <c r="B2241" t="inlineStr">
+        <is>
+          <t>tamilpsd-2213.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2242">
+      <c r="A2242" s="3" t="inlineStr">
+        <is>
+          <t>DMAX LIVE VOL 242 (5).psd</t>
+        </is>
+      </c>
+      <c r="B2242" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2214.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2243">
+      <c r="A2243" t="inlineStr">
+        <is>
+          <t>DMAX LIVE VOL 242 (6).psd</t>
+        </is>
+      </c>
+      <c r="B2243" t="inlineStr">
+        <is>
+          <t>tamilpsd-2215.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2244">
+      <c r="A2244" s="3" t="inlineStr">
+        <is>
+          <t>DMAX LIVE VOL 242 (7).psd</t>
+        </is>
+      </c>
+      <c r="B2244" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2216.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2245">
+      <c r="A2245" t="inlineStr">
+        <is>
+          <t>DMAX LIVE VOL 242 (10).psd</t>
+        </is>
+      </c>
+      <c r="B2245" t="inlineStr">
+        <is>
+          <t>tamilpsd-2217.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2246">
+      <c r="A2246" s="3" t="inlineStr">
+        <is>
+          <t>DMAX LIVE VOL 242 (11).psd</t>
+        </is>
+      </c>
+      <c r="B2246" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2218.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2247">
+      <c r="A2247" t="inlineStr">
+        <is>
+          <t>DMAX LIVE VOL 242 (12).psd</t>
+        </is>
+      </c>
+      <c r="B2247" t="inlineStr">
+        <is>
+          <t>tamilpsd-2219.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2248">
+      <c r="A2248" s="3" t="inlineStr">
+        <is>
+          <t>DMAX LIVE VOL 242 (13).psd</t>
+        </is>
+      </c>
+      <c r="B2248" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2220.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2249">
+      <c r="A2249" t="inlineStr">
+        <is>
+          <t>DMAX LIVE VOL 242 (14).psd</t>
+        </is>
+      </c>
+      <c r="B2249" t="inlineStr">
+        <is>
+          <t>tamilpsd-2221.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2250">
+      <c r="A2250" s="3" t="inlineStr">
+        <is>
+          <t>DMAX LIVE VOL 242 (8).psd</t>
+        </is>
+      </c>
+      <c r="B2250" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2222.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2251">
+      <c r="A2251" t="inlineStr">
+        <is>
+          <t>DMAX LIVE VOL 242 (9).psd</t>
+        </is>
+      </c>
+      <c r="B2251" t="inlineStr">
+        <is>
+          <t>tamilpsd-2223.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2252">
+      <c r="A2252" s="3" t="inlineStr">
+        <is>
+          <t>RC Design 12 X 36 (8).psd</t>
+        </is>
+      </c>
+      <c r="B2252" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2227.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2253">
+      <c r="A2253" t="inlineStr">
+        <is>
+          <t>RC Design 12 X 36 (9).psd</t>
+        </is>
+      </c>
+      <c r="B2253" t="inlineStr">
+        <is>
+          <t>tamilpsd-2228.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2254">
+      <c r="A2254" s="3" t="inlineStr">
+        <is>
+          <t>RC Design 12 X 36 (10).psd</t>
+        </is>
+      </c>
+      <c r="B2254" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2229.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2255">
+      <c r="A2255" t="inlineStr">
+        <is>
+          <t>RC Design 12 X 36 (7).psd</t>
+        </is>
+      </c>
+      <c r="B2255" t="inlineStr">
+        <is>
+          <t>tamilpsd-2233.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2256">
+      <c r="A2256" s="3" t="inlineStr">
+        <is>
+          <t>4551.psd</t>
+        </is>
+      </c>
+      <c r="B2256" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2234.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2257">
+      <c r="A2257" t="inlineStr">
+        <is>
+          <t>4550.psd</t>
+        </is>
+      </c>
+      <c r="B2257" t="inlineStr">
+        <is>
+          <t>tamilpsd-2235.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2258">
+      <c r="A2258" s="3" t="inlineStr">
+        <is>
+          <t>4552.psd</t>
+        </is>
+      </c>
+      <c r="B2258" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2236.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2259">
+      <c r="A2259" t="inlineStr">
+        <is>
+          <t>4548.psd</t>
+        </is>
+      </c>
+      <c r="B2259" t="inlineStr">
+        <is>
+          <t>tamilpsd-2237.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2260">
+      <c r="A2260" s="3" t="inlineStr">
+        <is>
+          <t>4546.psd</t>
+        </is>
+      </c>
+      <c r="B2260" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2238.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2261">
+      <c r="A2261" t="inlineStr">
+        <is>
+          <t>4534.psd</t>
+        </is>
+      </c>
+      <c r="B2261" t="inlineStr">
+        <is>
+          <t>tamilpsd-2239.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2262">
+      <c r="A2262" s="3" t="inlineStr">
+        <is>
+          <t>4359.psd</t>
+        </is>
+      </c>
+      <c r="B2262" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2240.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2263">
+      <c r="A2263" t="inlineStr">
+        <is>
+          <t>4358.psd</t>
+        </is>
+      </c>
+      <c r="B2263" t="inlineStr">
+        <is>
+          <t>tamilpsd-2241.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2264">
+      <c r="A2264" s="3" t="inlineStr">
+        <is>
+          <t>4357.psd</t>
+        </is>
+      </c>
+      <c r="B2264" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2242.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2265">
+      <c r="A2265" t="inlineStr">
+        <is>
+          <t>4356.psd</t>
+        </is>
+      </c>
+      <c r="B2265" t="inlineStr">
+        <is>
+          <t>tamilpsd-2243.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2266">
+      <c r="A2266" s="3" t="inlineStr">
+        <is>
+          <t>4355.psd</t>
+        </is>
+      </c>
+      <c r="B2266" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2244.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2267">
+      <c r="A2267" t="inlineStr">
+        <is>
+          <t>4354.psd</t>
+        </is>
+      </c>
+      <c r="B2267" t="inlineStr">
+        <is>
+          <t>tamilpsd-2245.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2268">
+      <c r="A2268" s="3" t="inlineStr">
+        <is>
+          <t>4353.psd</t>
+        </is>
+      </c>
+      <c r="B2268" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2246.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2269">
+      <c r="A2269" t="inlineStr">
+        <is>
+          <t>4352.psd</t>
+        </is>
+      </c>
+      <c r="B2269" t="inlineStr">
+        <is>
+          <t>tamilpsd-2247.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2270">
+      <c r="A2270" s="3" t="inlineStr">
+        <is>
+          <t>4350.psd</t>
+        </is>
+      </c>
+      <c r="B2270" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2248.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2271">
+      <c r="A2271" t="inlineStr">
+        <is>
+          <t>4351.psd</t>
+        </is>
+      </c>
+      <c r="B2271" t="inlineStr">
+        <is>
+          <t>tamilpsd-2249.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2272">
+      <c r="A2272" s="3" t="inlineStr">
+        <is>
+          <t>4349.psd</t>
+        </is>
+      </c>
+      <c r="B2272" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2250.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2273">
+      <c r="A2273" t="inlineStr">
+        <is>
+          <t>4348.psd</t>
+        </is>
+      </c>
+      <c r="B2273" t="inlineStr">
+        <is>
+          <t>tamilpsd-2251.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2274">
+      <c r="A2274" s="3" t="inlineStr">
+        <is>
+          <t>4345.psd</t>
+        </is>
+      </c>
+      <c r="B2274" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2252.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2275">
+      <c r="A2275" t="inlineStr">
+        <is>
+          <t>4347.psd</t>
+        </is>
+      </c>
+      <c r="B2275" t="inlineStr">
+        <is>
+          <t>tamilpsd-2253.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2276">
+      <c r="A2276" s="3" t="inlineStr">
+        <is>
+          <t>4344.psd</t>
+        </is>
+      </c>
+      <c r="B2276" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2254.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2277">
+      <c r="A2277" t="inlineStr">
+        <is>
+          <t>4342.psd</t>
+        </is>
+      </c>
+      <c r="B2277" t="inlineStr">
+        <is>
+          <t>tamilpsd-2255.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2278">
+      <c r="A2278" s="3" t="inlineStr">
+        <is>
+          <t>4343.psd</t>
+        </is>
+      </c>
+      <c r="B2278" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2256.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2279">
+      <c r="A2279" t="inlineStr">
+        <is>
+          <t>4341.psd</t>
+        </is>
+      </c>
+      <c r="B2279" t="inlineStr">
+        <is>
+          <t>tamilpsd-2257.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2280">
+      <c r="A2280" s="3" t="inlineStr">
+        <is>
+          <t>4340.psd</t>
+        </is>
+      </c>
+      <c r="B2280" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2258.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2281">
+      <c r="A2281" t="inlineStr">
+        <is>
+          <t>4338.psd</t>
+        </is>
+      </c>
+      <c r="B2281" t="inlineStr">
+        <is>
+          <t>tamilpsd-2259.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2282">
+      <c r="A2282" s="3" t="inlineStr">
+        <is>
+          <t>4339.psd</t>
+        </is>
+      </c>
+      <c r="B2282" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2260.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2283">
+      <c r="A2283" t="inlineStr">
+        <is>
+          <t>4337.psd</t>
+        </is>
+      </c>
+      <c r="B2283" t="inlineStr">
+        <is>
+          <t>tamilpsd-2261.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2284">
+      <c r="A2284" s="3" t="inlineStr">
+        <is>
+          <t>4336.PSD</t>
+        </is>
+      </c>
+      <c r="B2284" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2262.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2285">
+      <c r="A2285" t="inlineStr">
+        <is>
+          <t>4335.psd</t>
+        </is>
+      </c>
+      <c r="B2285" t="inlineStr">
+        <is>
+          <t>tamilpsd-2263.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2286">
+      <c r="A2286" s="3" t="inlineStr">
+        <is>
+          <t>4334.psd</t>
+        </is>
+      </c>
+      <c r="B2286" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2264.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2287">
+      <c r="A2287" t="inlineStr">
+        <is>
+          <t>4333.psd</t>
+        </is>
+      </c>
+      <c r="B2287" t="inlineStr">
+        <is>
+          <t>tamilpsd-2265.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2288">
+      <c r="A2288" s="3" t="inlineStr">
+        <is>
+          <t>4332.psd</t>
+        </is>
+      </c>
+      <c r="B2288" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2266.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2289">
+      <c r="A2289" t="inlineStr">
+        <is>
+          <t>4331.psd</t>
+        </is>
+      </c>
+      <c r="B2289" t="inlineStr">
+        <is>
+          <t>tamilpsd-2267.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2290">
+      <c r="A2290" s="3" t="inlineStr">
+        <is>
+          <t>4330.psd</t>
+        </is>
+      </c>
+      <c r="B2290" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2268.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2291">
+      <c r="A2291" t="inlineStr">
+        <is>
+          <t>4329.psd</t>
+        </is>
+      </c>
+      <c r="B2291" t="inlineStr">
+        <is>
+          <t>tamilpsd-2269.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2292">
+      <c r="A2292" s="3" t="inlineStr">
+        <is>
+          <t>4328.psd</t>
+        </is>
+      </c>
+      <c r="B2292" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2270.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2293">
+      <c r="A2293" t="inlineStr">
+        <is>
+          <t>4327.psd</t>
+        </is>
+      </c>
+      <c r="B2293" t="inlineStr">
+        <is>
+          <t>tamilpsd-2271.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2294">
+      <c r="A2294" s="3" t="inlineStr">
+        <is>
+          <t>4326.psd</t>
+        </is>
+      </c>
+      <c r="B2294" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2272.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2295">
+      <c r="A2295" t="inlineStr">
+        <is>
+          <t>4325.psd</t>
+        </is>
+      </c>
+      <c r="B2295" t="inlineStr">
+        <is>
+          <t>tamilpsd-2273.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2296">
+      <c r="A2296" s="3" t="inlineStr">
+        <is>
+          <t>4324.psd</t>
+        </is>
+      </c>
+      <c r="B2296" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2274.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2297">
+      <c r="A2297" t="inlineStr">
+        <is>
+          <t>4323.psd</t>
+        </is>
+      </c>
+      <c r="B2297" t="inlineStr">
+        <is>
+          <t>tamilpsd-2275.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2298">
+      <c r="A2298" s="3" t="inlineStr">
+        <is>
+          <t>4322.psd</t>
+        </is>
+      </c>
+      <c r="B2298" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2276.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2299">
+      <c r="A2299" t="inlineStr">
+        <is>
+          <t>4321.psd</t>
+        </is>
+      </c>
+      <c r="B2299" t="inlineStr">
+        <is>
+          <t>tamilpsd-2277.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2300">
+      <c r="A2300" s="3" t="inlineStr">
+        <is>
+          <t>Rc Design 12x30 (2)25.psd</t>
+        </is>
+      </c>
+      <c r="B2300" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2278.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2301">
+      <c r="A2301" t="inlineStr">
+        <is>
+          <t>RC Design 12x36 (4)12.psd</t>
+        </is>
+      </c>
+      <c r="B2301" t="inlineStr">
+        <is>
+          <t>tamilpsd-2279.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2302">
+      <c r="A2302" s="3" t="inlineStr">
+        <is>
+          <t>RC Design 12x36 (4)22.psd</t>
+        </is>
+      </c>
+      <c r="B2302" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2280.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2303">
+      <c r="A2303" t="inlineStr">
+        <is>
+          <t>RC Design 12x36 (5)13.psd</t>
+        </is>
+      </c>
+      <c r="B2303" t="inlineStr">
+        <is>
+          <t>tamilpsd-2281.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2304">
+      <c r="A2304" s="3" t="inlineStr">
+        <is>
+          <t>RC Design 12x36 (5)23.psd</t>
+        </is>
+      </c>
+      <c r="B2304" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2282.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2305">
+      <c r="A2305" t="inlineStr">
+        <is>
+          <t>Rc Design 12x36 (5)8.psd</t>
+        </is>
+      </c>
+      <c r="B2305" t="inlineStr">
+        <is>
+          <t>tamilpsd-2283.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2306">
+      <c r="A2306" s="3" t="inlineStr">
+        <is>
+          <t>RC Design 12x36 (2)10.psd</t>
+        </is>
+      </c>
+      <c r="B2306" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2284.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2307">
+      <c r="A2307" t="inlineStr">
+        <is>
+          <t>RC Design 12x36 (2)20.psd</t>
+        </is>
+      </c>
+      <c r="B2307" t="inlineStr">
+        <is>
+          <t>tamilpsd-2285.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2308">
+      <c r="A2308" s="3" t="inlineStr">
+        <is>
+          <t>RC Design 12x36 (3)11.psd</t>
+        </is>
+      </c>
+      <c r="B2308" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2286.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2309">
+      <c r="A2309" t="inlineStr">
+        <is>
+          <t>RC Design 12x36 (3)21.psd</t>
+        </is>
+      </c>
+      <c r="B2309" t="inlineStr">
+        <is>
+          <t>tamilpsd-2287.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2310">
+      <c r="A2310" s="3" t="inlineStr">
+        <is>
+          <t>RC Design 12x36 (3)3.psd</t>
+        </is>
+      </c>
+      <c r="B2310" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2288.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2311">
+      <c r="A2311" t="inlineStr">
+        <is>
+          <t>Rc Design 12x36 (3)6.psd</t>
+        </is>
+      </c>
+      <c r="B2311" t="inlineStr">
+        <is>
+          <t>tamilpsd-2289.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2312">
+      <c r="A2312" s="3" t="inlineStr">
+        <is>
+          <t>Rc Design 12x36 (4)7.psd</t>
+        </is>
+      </c>
+      <c r="B2312" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2290.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2313">
+      <c r="A2313" t="inlineStr">
+        <is>
+          <t>Rc Design 12x30 (3)26.psd</t>
+        </is>
+      </c>
+      <c r="B2313" t="inlineStr">
+        <is>
+          <t>tamilpsd-2291.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2314">
+      <c r="A2314" s="3" t="inlineStr">
+        <is>
+          <t>RC Design 12x36 (1)1.psd</t>
+        </is>
+      </c>
+      <c r="B2314" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2292.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2315">
+      <c r="A2315" t="inlineStr">
+        <is>
+          <t>RC Design 12x36 (1)19.psd</t>
+        </is>
+      </c>
+      <c r="B2315" t="inlineStr">
+        <is>
+          <t>tamilpsd-2293.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2316">
+      <c r="A2316" s="3" t="inlineStr">
+        <is>
+          <t>Rc Design 12x36 (1)4.psd</t>
+        </is>
+      </c>
+      <c r="B2316" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2294.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2317">
+      <c r="A2317" t="inlineStr">
+        <is>
+          <t>RC Design 12x36 (1)9.psd</t>
+        </is>
+      </c>
+      <c r="B2317" t="inlineStr">
+        <is>
+          <t>tamilpsd-2295.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2318">
+      <c r="A2318" s="3" t="inlineStr">
+        <is>
+          <t>RC Design 12x36 (2)2.psd</t>
+        </is>
+      </c>
+      <c r="B2318" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2296.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2319">
+      <c r="A2319" t="inlineStr">
+        <is>
+          <t>Rc Design 12x36 (2)5.psd</t>
+        </is>
+      </c>
+      <c r="B2319" t="inlineStr">
+        <is>
+          <t>tamilpsd-2297.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2320">
+      <c r="A2320" s="3" t="inlineStr">
+        <is>
+          <t>RC Desgin 12x36 (1)14.psd</t>
+        </is>
+      </c>
+      <c r="B2320" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2298.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2321">
+      <c r="A2321" t="inlineStr">
+        <is>
+          <t>RC Desgin 12x36 (2)15.psd</t>
+        </is>
+      </c>
+      <c r="B2321" t="inlineStr">
+        <is>
+          <t>tamilpsd-2299.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2322">
+      <c r="A2322" s="3" t="inlineStr">
+        <is>
+          <t>RC Desgin 12x36 (3)16.psd</t>
+        </is>
+      </c>
+      <c r="B2322" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2300.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2323">
+      <c r="A2323" t="inlineStr">
+        <is>
+          <t>RC Desgin 12x36 (4)17.psd</t>
+        </is>
+      </c>
+      <c r="B2323" t="inlineStr">
+        <is>
+          <t>tamilpsd-2301.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2324">
+      <c r="A2324" s="3" t="inlineStr">
+        <is>
+          <t>RC Desgin 12x36 (5)18.psd</t>
+        </is>
+      </c>
+      <c r="B2324" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2302.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2325">
+      <c r="A2325" t="inlineStr">
+        <is>
+          <t>Rc Design 12x30 (1)24.psd</t>
+        </is>
+      </c>
+      <c r="B2325" t="inlineStr">
+        <is>
+          <t>tamilpsd-2303.psd</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
🤖 Progress: 2026-04-19 23:17 UTC
</commit_message>
<xml_diff>
--- a/rename_log.xlsx
+++ b/rename_log.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2325"/>
+  <dimension ref="A1:B2634"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -27997,6 +27997,3714 @@
         </is>
       </c>
     </row>
+    <row r="2326">
+      <c r="A2326" s="3" t="inlineStr">
+        <is>
+          <t>RC Design 12x36 (41).psd</t>
+        </is>
+      </c>
+      <c r="B2326" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2830.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2327">
+      <c r="A2327" t="inlineStr">
+        <is>
+          <t>RC Design 12x36 (42).psd</t>
+        </is>
+      </c>
+      <c r="B2327" t="inlineStr">
+        <is>
+          <t>tamilpsd-2831.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2328">
+      <c r="A2328" s="3" t="inlineStr">
+        <is>
+          <t>RC Design 12x36 (43).psd</t>
+        </is>
+      </c>
+      <c r="B2328" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2832.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2329">
+      <c r="A2329" t="inlineStr">
+        <is>
+          <t>RC Design 12x36 (44).psd</t>
+        </is>
+      </c>
+      <c r="B2329" t="inlineStr">
+        <is>
+          <t>tamilpsd-2833.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2330">
+      <c r="A2330" s="3" t="inlineStr">
+        <is>
+          <t>RC Design 12x36 (45).psd</t>
+        </is>
+      </c>
+      <c r="B2330" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2834.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2331">
+      <c r="A2331" t="inlineStr">
+        <is>
+          <t>RC Design 12x36 (46).psd</t>
+        </is>
+      </c>
+      <c r="B2331" t="inlineStr">
+        <is>
+          <t>tamilpsd-2835.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2332">
+      <c r="A2332" s="3" t="inlineStr">
+        <is>
+          <t>RC Design 12x36 (47).psd</t>
+        </is>
+      </c>
+      <c r="B2332" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2836.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2333">
+      <c r="A2333" t="inlineStr">
+        <is>
+          <t>RC Design 12x36 (48).psd</t>
+        </is>
+      </c>
+      <c r="B2333" t="inlineStr">
+        <is>
+          <t>tamilpsd-2837.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2334">
+      <c r="A2334" s="3" t="inlineStr">
+        <is>
+          <t>RC Design 12x36 (49).psd</t>
+        </is>
+      </c>
+      <c r="B2334" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2838.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2335">
+      <c r="A2335" t="inlineStr">
+        <is>
+          <t>RC Design 12x36 (50).psd</t>
+        </is>
+      </c>
+      <c r="B2335" t="inlineStr">
+        <is>
+          <t>tamilpsd-2839.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2336">
+      <c r="A2336" s="3" t="inlineStr">
+        <is>
+          <t>RC Design 12x36 1.psd</t>
+        </is>
+      </c>
+      <c r="B2336" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2845.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2337">
+      <c r="A2337" t="inlineStr">
+        <is>
+          <t>RC Design 12x36 2.psd</t>
+        </is>
+      </c>
+      <c r="B2337" t="inlineStr">
+        <is>
+          <t>tamilpsd-2846.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2338">
+      <c r="A2338" s="3" t="inlineStr">
+        <is>
+          <t>RC Design 12x36 3.psd</t>
+        </is>
+      </c>
+      <c r="B2338" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2847.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2339">
+      <c r="A2339" t="inlineStr">
+        <is>
+          <t>RC Design 12x36 4.psd</t>
+        </is>
+      </c>
+      <c r="B2339" t="inlineStr">
+        <is>
+          <t>tamilpsd-2848.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2340">
+      <c r="A2340" s="3" t="inlineStr">
+        <is>
+          <t>DMAX LIVE VOL 242 (15).psd</t>
+        </is>
+      </c>
+      <c r="B2340" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2849.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2341">
+      <c r="A2341" t="inlineStr">
+        <is>
+          <t>DMAX LIVE VOL 242 (16).psd</t>
+        </is>
+      </c>
+      <c r="B2341" t="inlineStr">
+        <is>
+          <t>tamilpsd-2850.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2342">
+      <c r="A2342" s="3" t="inlineStr">
+        <is>
+          <t>DMAX LIVE VOL 242 (17).psd</t>
+        </is>
+      </c>
+      <c r="B2342" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2851.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2343">
+      <c r="A2343" t="inlineStr">
+        <is>
+          <t>DMAX LIVE VOL 242 (18).psd</t>
+        </is>
+      </c>
+      <c r="B2343" t="inlineStr">
+        <is>
+          <t>tamilpsd-2852.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2344">
+      <c r="A2344" s="3" t="inlineStr">
+        <is>
+          <t>DMAX LIVE VOL 242 (19).psd</t>
+        </is>
+      </c>
+      <c r="B2344" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2853.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2345">
+      <c r="A2345" t="inlineStr">
+        <is>
+          <t>DMAX LIVE VOL 242 (20).psd</t>
+        </is>
+      </c>
+      <c r="B2345" t="inlineStr">
+        <is>
+          <t>tamilpsd-2854.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2346">
+      <c r="A2346" s="3" t="inlineStr">
+        <is>
+          <t>DMAX LIVE VOL 242 (21).psd</t>
+        </is>
+      </c>
+      <c r="B2346" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2855.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2347">
+      <c r="A2347" t="inlineStr">
+        <is>
+          <t>DMAX LIVE VOL 242 (22).psd</t>
+        </is>
+      </c>
+      <c r="B2347" t="inlineStr">
+        <is>
+          <t>tamilpsd-2856.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2348">
+      <c r="A2348" s="3" t="inlineStr">
+        <is>
+          <t>DMAX LIVE VOl245 (10).psd</t>
+        </is>
+      </c>
+      <c r="B2348" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2857.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2349">
+      <c r="A2349" t="inlineStr">
+        <is>
+          <t>DMAX LIVEVOL-99 (10).psd</t>
+        </is>
+      </c>
+      <c r="B2349" t="inlineStr">
+        <is>
+          <t>tamilpsd-2858.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2350">
+      <c r="A2350" s="3" t="inlineStr">
+        <is>
+          <t>DMAX LIVEVOL-99 (12).psd</t>
+        </is>
+      </c>
+      <c r="B2350" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2859.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2351">
+      <c r="A2351" t="inlineStr">
+        <is>
+          <t>DMAX LIVEVOL-99 (18).psd</t>
+        </is>
+      </c>
+      <c r="B2351" t="inlineStr">
+        <is>
+          <t>tamilpsd-2860.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2352">
+      <c r="A2352" s="3" t="inlineStr">
+        <is>
+          <t>DMAX LIVEVOL-99 (19).psd</t>
+        </is>
+      </c>
+      <c r="B2352" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2861.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2353">
+      <c r="A2353" t="inlineStr">
+        <is>
+          <t>SOORIYA 001.psd</t>
+        </is>
+      </c>
+      <c r="B2353" t="inlineStr">
+        <is>
+          <t>tamilpsd-2862.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2354">
+      <c r="A2354" s="3" t="inlineStr">
+        <is>
+          <t>SOORIYA 002.psd</t>
+        </is>
+      </c>
+      <c r="B2354" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2863.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2355">
+      <c r="A2355" t="inlineStr">
+        <is>
+          <t>SOORIYA 003.psd</t>
+        </is>
+      </c>
+      <c r="B2355" t="inlineStr">
+        <is>
+          <t>tamilpsd-2864.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2356">
+      <c r="A2356" s="3" t="inlineStr">
+        <is>
+          <t>SOORIYA 004.psd</t>
+        </is>
+      </c>
+      <c r="B2356" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2865.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2357">
+      <c r="A2357" t="inlineStr">
+        <is>
+          <t>SOORIYA 005.psd</t>
+        </is>
+      </c>
+      <c r="B2357" t="inlineStr">
+        <is>
+          <t>tamilpsd-2866.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2358">
+      <c r="A2358" s="3" t="inlineStr">
+        <is>
+          <t>SOORIYA 006.psd</t>
+        </is>
+      </c>
+      <c r="B2358" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2867.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2359">
+      <c r="A2359" t="inlineStr">
+        <is>
+          <t>SOORIYA 007.psd</t>
+        </is>
+      </c>
+      <c r="B2359" t="inlineStr">
+        <is>
+          <t>tamilpsd-2868.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2360">
+      <c r="A2360" s="3" t="inlineStr">
+        <is>
+          <t>SOORIYA 008.psd</t>
+        </is>
+      </c>
+      <c r="B2360" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2869.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2361">
+      <c r="A2361" t="inlineStr">
+        <is>
+          <t>SOORIYA 009.psd</t>
+        </is>
+      </c>
+      <c r="B2361" t="inlineStr">
+        <is>
+          <t>tamilpsd-2870.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2362">
+      <c r="A2362" s="3" t="inlineStr">
+        <is>
+          <t>SOORIYA 010.psd</t>
+        </is>
+      </c>
+      <c r="B2362" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2871.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2363">
+      <c r="A2363" t="inlineStr">
+        <is>
+          <t>SOORIYA 018.psd</t>
+        </is>
+      </c>
+      <c r="B2363" t="inlineStr">
+        <is>
+          <t>tamilpsd-2872.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2364">
+      <c r="A2364" s="3" t="inlineStr">
+        <is>
+          <t>SOORIYA 025.psd</t>
+        </is>
+      </c>
+      <c r="B2364" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2873.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2365">
+      <c r="A2365" t="inlineStr">
+        <is>
+          <t>SOORIYA 027.psd</t>
+        </is>
+      </c>
+      <c r="B2365" t="inlineStr">
+        <is>
+          <t>tamilpsd-2874.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2366">
+      <c r="A2366" s="3" t="inlineStr">
+        <is>
+          <t>SOORIYA001.psd</t>
+        </is>
+      </c>
+      <c r="B2366" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2875.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2367">
+      <c r="A2367" t="inlineStr">
+        <is>
+          <t>SOORIYA002.psd</t>
+        </is>
+      </c>
+      <c r="B2367" t="inlineStr">
+        <is>
+          <t>tamilpsd-2876.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2368">
+      <c r="A2368" s="3" t="inlineStr">
+        <is>
+          <t>SOORIYA003.psd</t>
+        </is>
+      </c>
+      <c r="B2368" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2877.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2369">
+      <c r="A2369" t="inlineStr">
+        <is>
+          <t>SOORIYA004.psd</t>
+        </is>
+      </c>
+      <c r="B2369" t="inlineStr">
+        <is>
+          <t>tamilpsd-2878.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2370">
+      <c r="A2370" s="3" t="inlineStr">
+        <is>
+          <t>SOORIYA005.psd</t>
+        </is>
+      </c>
+      <c r="B2370" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2879.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2371">
+      <c r="A2371" t="inlineStr">
+        <is>
+          <t>SOORIYA006.psd</t>
+        </is>
+      </c>
+      <c r="B2371" t="inlineStr">
+        <is>
+          <t>tamilpsd-2880.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2372">
+      <c r="A2372" s="3" t="inlineStr">
+        <is>
+          <t>SOORIYA007.psd</t>
+        </is>
+      </c>
+      <c r="B2372" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2881.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2373">
+      <c r="A2373" t="inlineStr">
+        <is>
+          <t>SOORIYA008.psd</t>
+        </is>
+      </c>
+      <c r="B2373" t="inlineStr">
+        <is>
+          <t>tamilpsd-2882.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2374">
+      <c r="A2374" s="3" t="inlineStr">
+        <is>
+          <t>SOORIYA009.psd</t>
+        </is>
+      </c>
+      <c r="B2374" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2883.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2375">
+      <c r="A2375" t="inlineStr">
+        <is>
+          <t>SOORIYA010.psd</t>
+        </is>
+      </c>
+      <c r="B2375" t="inlineStr">
+        <is>
+          <t>tamilpsd-2884.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2376">
+      <c r="A2376" s="3" t="inlineStr">
+        <is>
+          <t>RC Desing 12x36 (15).psd</t>
+        </is>
+      </c>
+      <c r="B2376" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2885.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2377">
+      <c r="A2377" t="inlineStr">
+        <is>
+          <t>RC Desing 12x36 (16).psd</t>
+        </is>
+      </c>
+      <c r="B2377" t="inlineStr">
+        <is>
+          <t>tamilpsd-2886.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2378">
+      <c r="A2378" s="3" t="inlineStr">
+        <is>
+          <t>RC Desing 12x36 (17).psd</t>
+        </is>
+      </c>
+      <c r="B2378" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2887.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2379">
+      <c r="A2379" t="inlineStr">
+        <is>
+          <t>RC Desing 12x36 (18).psd</t>
+        </is>
+      </c>
+      <c r="B2379" t="inlineStr">
+        <is>
+          <t>tamilpsd-2888.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2380">
+      <c r="A2380" s="3" t="inlineStr">
+        <is>
+          <t>RC Desing 12x36 (19).psd</t>
+        </is>
+      </c>
+      <c r="B2380" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2889.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2381">
+      <c r="A2381" t="inlineStr">
+        <is>
+          <t>RC Desing 12x36 (20).psd</t>
+        </is>
+      </c>
+      <c r="B2381" t="inlineStr">
+        <is>
+          <t>tamilpsd-2890.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2382">
+      <c r="A2382" s="3" t="inlineStr">
+        <is>
+          <t>RC Desing 12x36 (21).psd</t>
+        </is>
+      </c>
+      <c r="B2382" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2891.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2383">
+      <c r="A2383" t="inlineStr">
+        <is>
+          <t>RC Desing 12x36 (22).psd</t>
+        </is>
+      </c>
+      <c r="B2383" t="inlineStr">
+        <is>
+          <t>tamilpsd-2892.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2384">
+      <c r="A2384" s="3" t="inlineStr">
+        <is>
+          <t>RC Desing 12x36 (23).psd</t>
+        </is>
+      </c>
+      <c r="B2384" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2893.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2385">
+      <c r="A2385" t="inlineStr">
+        <is>
+          <t>RC Desing 12x36 (24).psd</t>
+        </is>
+      </c>
+      <c r="B2385" t="inlineStr">
+        <is>
+          <t>tamilpsd-2894.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2386">
+      <c r="A2386" s="3" t="inlineStr">
+        <is>
+          <t>RC Desing 12x36 (25).psd</t>
+        </is>
+      </c>
+      <c r="B2386" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2895.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2387">
+      <c r="A2387" t="inlineStr">
+        <is>
+          <t>RC Design 12x36 5.psd</t>
+        </is>
+      </c>
+      <c r="B2387" t="inlineStr">
+        <is>
+          <t>tamilpsd-2896.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2388">
+      <c r="A2388" s="3" t="inlineStr">
+        <is>
+          <t>RC Design 12x36 a.psd</t>
+        </is>
+      </c>
+      <c r="B2388" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2897.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2389">
+      <c r="A2389" t="inlineStr">
+        <is>
+          <t>RC Design 12x36 b.psd</t>
+        </is>
+      </c>
+      <c r="B2389" t="inlineStr">
+        <is>
+          <t>tamilpsd-2898.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2390">
+      <c r="A2390" s="3" t="inlineStr">
+        <is>
+          <t>RC Design 12x36 c.psd</t>
+        </is>
+      </c>
+      <c r="B2390" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2899.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2391">
+      <c r="A2391" t="inlineStr">
+        <is>
+          <t>RC Design 12x36 d.psd</t>
+        </is>
+      </c>
+      <c r="B2391" t="inlineStr">
+        <is>
+          <t>tamilpsd-2900.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2392">
+      <c r="A2392" s="3" t="inlineStr">
+        <is>
+          <t>RC Design 12x36 e.psd</t>
+        </is>
+      </c>
+      <c r="B2392" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2901.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2393">
+      <c r="A2393" t="inlineStr">
+        <is>
+          <t>4267.psd</t>
+        </is>
+      </c>
+      <c r="B2393" t="inlineStr">
+        <is>
+          <t>tamilpsd-2902.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2394">
+      <c r="A2394" s="3" t="inlineStr">
+        <is>
+          <t>4266.psd</t>
+        </is>
+      </c>
+      <c r="B2394" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2903.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2395">
+      <c r="A2395" t="inlineStr">
+        <is>
+          <t>4265.psd</t>
+        </is>
+      </c>
+      <c r="B2395" t="inlineStr">
+        <is>
+          <t>tamilpsd-2904.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2396">
+      <c r="A2396" s="3" t="inlineStr">
+        <is>
+          <t>4264.psd</t>
+        </is>
+      </c>
+      <c r="B2396" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2905.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2397">
+      <c r="A2397" t="inlineStr">
+        <is>
+          <t>4262.psd</t>
+        </is>
+      </c>
+      <c r="B2397" t="inlineStr">
+        <is>
+          <t>tamilpsd-2906.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2398">
+      <c r="A2398" s="3" t="inlineStr">
+        <is>
+          <t>4261.psd</t>
+        </is>
+      </c>
+      <c r="B2398" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2907.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2399">
+      <c r="A2399" t="inlineStr">
+        <is>
+          <t>4260.psd</t>
+        </is>
+      </c>
+      <c r="B2399" t="inlineStr">
+        <is>
+          <t>tamilpsd-2908.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2400">
+      <c r="A2400" s="3" t="inlineStr">
+        <is>
+          <t>4259.psd</t>
+        </is>
+      </c>
+      <c r="B2400" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2909.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2401">
+      <c r="A2401" t="inlineStr">
+        <is>
+          <t>4258.psd</t>
+        </is>
+      </c>
+      <c r="B2401" t="inlineStr">
+        <is>
+          <t>tamilpsd-2910.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2402">
+      <c r="A2402" s="3" t="inlineStr">
+        <is>
+          <t>4257.psd</t>
+        </is>
+      </c>
+      <c r="B2402" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2911.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2403">
+      <c r="A2403" t="inlineStr">
+        <is>
+          <t>4256.psd</t>
+        </is>
+      </c>
+      <c r="B2403" t="inlineStr">
+        <is>
+          <t>tamilpsd-2912.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2404">
+      <c r="A2404" s="3" t="inlineStr">
+        <is>
+          <t>4255.psd</t>
+        </is>
+      </c>
+      <c r="B2404" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2913.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2405">
+      <c r="A2405" t="inlineStr">
+        <is>
+          <t>4254.psd</t>
+        </is>
+      </c>
+      <c r="B2405" t="inlineStr">
+        <is>
+          <t>tamilpsd-2914.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2406">
+      <c r="A2406" s="3" t="inlineStr">
+        <is>
+          <t>4253.psd</t>
+        </is>
+      </c>
+      <c r="B2406" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2915.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2407">
+      <c r="A2407" t="inlineStr">
+        <is>
+          <t>4252.psd</t>
+        </is>
+      </c>
+      <c r="B2407" t="inlineStr">
+        <is>
+          <t>tamilpsd-2916.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2408">
+      <c r="A2408" s="3" t="inlineStr">
+        <is>
+          <t>4251.psd</t>
+        </is>
+      </c>
+      <c r="B2408" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2917.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2409">
+      <c r="A2409" t="inlineStr">
+        <is>
+          <t>4250.psd</t>
+        </is>
+      </c>
+      <c r="B2409" t="inlineStr">
+        <is>
+          <t>tamilpsd-2918.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2410">
+      <c r="A2410" s="3" t="inlineStr">
+        <is>
+          <t>4249.psd</t>
+        </is>
+      </c>
+      <c r="B2410" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2919.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2411">
+      <c r="A2411" t="inlineStr">
+        <is>
+          <t>4248.psd</t>
+        </is>
+      </c>
+      <c r="B2411" t="inlineStr">
+        <is>
+          <t>tamilpsd-2920.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2412">
+      <c r="A2412" s="3" t="inlineStr">
+        <is>
+          <t>4247.psd</t>
+        </is>
+      </c>
+      <c r="B2412" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2921.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2413">
+      <c r="A2413" t="inlineStr">
+        <is>
+          <t>4246.psd</t>
+        </is>
+      </c>
+      <c r="B2413" t="inlineStr">
+        <is>
+          <t>tamilpsd-2922.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2414">
+      <c r="A2414" s="3" t="inlineStr">
+        <is>
+          <t>4245.psd</t>
+        </is>
+      </c>
+      <c r="B2414" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2923.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2415">
+      <c r="A2415" t="inlineStr">
+        <is>
+          <t>4244.psd</t>
+        </is>
+      </c>
+      <c r="B2415" t="inlineStr">
+        <is>
+          <t>tamilpsd-2924.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2416">
+      <c r="A2416" s="3" t="inlineStr">
+        <is>
+          <t>4268.psd</t>
+        </is>
+      </c>
+      <c r="B2416" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2925.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2417">
+      <c r="A2417" t="inlineStr">
+        <is>
+          <t>4242.psd</t>
+        </is>
+      </c>
+      <c r="B2417" t="inlineStr">
+        <is>
+          <t>tamilpsd-2926.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2418">
+      <c r="A2418" s="3" t="inlineStr">
+        <is>
+          <t>4241.psd</t>
+        </is>
+      </c>
+      <c r="B2418" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2927.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2419">
+      <c r="A2419" t="inlineStr">
+        <is>
+          <t>4240.psd</t>
+        </is>
+      </c>
+      <c r="B2419" t="inlineStr">
+        <is>
+          <t>tamilpsd-2928.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2420">
+      <c r="A2420" s="3" t="inlineStr">
+        <is>
+          <t>4238.psd</t>
+        </is>
+      </c>
+      <c r="B2420" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2929.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2421">
+      <c r="A2421" t="inlineStr">
+        <is>
+          <t>4239.psd</t>
+        </is>
+      </c>
+      <c r="B2421" t="inlineStr">
+        <is>
+          <t>tamilpsd-2930.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2422">
+      <c r="A2422" s="3" t="inlineStr">
+        <is>
+          <t>4237.psd</t>
+        </is>
+      </c>
+      <c r="B2422" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2931.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2423">
+      <c r="A2423" t="inlineStr">
+        <is>
+          <t>4236.psd</t>
+        </is>
+      </c>
+      <c r="B2423" t="inlineStr">
+        <is>
+          <t>tamilpsd-2932.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2424">
+      <c r="A2424" s="3" t="inlineStr">
+        <is>
+          <t>4235.psd</t>
+        </is>
+      </c>
+      <c r="B2424" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2933.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2425">
+      <c r="A2425" t="inlineStr">
+        <is>
+          <t>4234.psd</t>
+        </is>
+      </c>
+      <c r="B2425" t="inlineStr">
+        <is>
+          <t>tamilpsd-2934.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2426">
+      <c r="A2426" s="3" t="inlineStr">
+        <is>
+          <t>4233.psd</t>
+        </is>
+      </c>
+      <c r="B2426" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2935.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2427">
+      <c r="A2427" t="inlineStr">
+        <is>
+          <t>4232.psd</t>
+        </is>
+      </c>
+      <c r="B2427" t="inlineStr">
+        <is>
+          <t>tamilpsd-2936.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2428">
+      <c r="A2428" s="3" t="inlineStr">
+        <is>
+          <t>4231.psd</t>
+        </is>
+      </c>
+      <c r="B2428" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2937.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2429">
+      <c r="A2429" t="inlineStr">
+        <is>
+          <t>4230.psd</t>
+        </is>
+      </c>
+      <c r="B2429" t="inlineStr">
+        <is>
+          <t>tamilpsd-2938.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2430">
+      <c r="A2430" s="3" t="inlineStr">
+        <is>
+          <t>4229.psd</t>
+        </is>
+      </c>
+      <c r="B2430" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2939.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2431">
+      <c r="A2431" t="inlineStr">
+        <is>
+          <t>4228.psd</t>
+        </is>
+      </c>
+      <c r="B2431" t="inlineStr">
+        <is>
+          <t>tamilpsd-2940.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2432">
+      <c r="A2432" s="3" t="inlineStr">
+        <is>
+          <t>4227.psd</t>
+        </is>
+      </c>
+      <c r="B2432" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2941.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2433">
+      <c r="A2433" t="inlineStr">
+        <is>
+          <t>4226.psd</t>
+        </is>
+      </c>
+      <c r="B2433" t="inlineStr">
+        <is>
+          <t>tamilpsd-2942.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2434">
+      <c r="A2434" s="3" t="inlineStr">
+        <is>
+          <t>4225.psd</t>
+        </is>
+      </c>
+      <c r="B2434" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2943.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2435">
+      <c r="A2435" t="inlineStr">
+        <is>
+          <t>4224.psd</t>
+        </is>
+      </c>
+      <c r="B2435" t="inlineStr">
+        <is>
+          <t>tamilpsd-2944.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2436">
+      <c r="A2436" s="3" t="inlineStr">
+        <is>
+          <t>4223.psd</t>
+        </is>
+      </c>
+      <c r="B2436" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2945.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2437">
+      <c r="A2437" t="inlineStr">
+        <is>
+          <t>4222.psd</t>
+        </is>
+      </c>
+      <c r="B2437" t="inlineStr">
+        <is>
+          <t>tamilpsd-2946.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2438">
+      <c r="A2438" s="3" t="inlineStr">
+        <is>
+          <t>4221.psd</t>
+        </is>
+      </c>
+      <c r="B2438" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2947.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2439">
+      <c r="A2439" t="inlineStr">
+        <is>
+          <t>4220.psd</t>
+        </is>
+      </c>
+      <c r="B2439" t="inlineStr">
+        <is>
+          <t>tamilpsd-2948.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2440">
+      <c r="A2440" s="3" t="inlineStr">
+        <is>
+          <t>4219.psd</t>
+        </is>
+      </c>
+      <c r="B2440" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2949.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2441">
+      <c r="A2441" t="inlineStr">
+        <is>
+          <t>4218.psd</t>
+        </is>
+      </c>
+      <c r="B2441" t="inlineStr">
+        <is>
+          <t>tamilpsd-2950.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2442">
+      <c r="A2442" s="3" t="inlineStr">
+        <is>
+          <t>4217.psd</t>
+        </is>
+      </c>
+      <c r="B2442" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2951.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2443">
+      <c r="A2443" t="inlineStr">
+        <is>
+          <t>4216.psd</t>
+        </is>
+      </c>
+      <c r="B2443" t="inlineStr">
+        <is>
+          <t>tamilpsd-2952.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2444">
+      <c r="A2444" s="3" t="inlineStr">
+        <is>
+          <t>4215.psd</t>
+        </is>
+      </c>
+      <c r="B2444" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2953.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2445">
+      <c r="A2445" t="inlineStr">
+        <is>
+          <t>4214.psd</t>
+        </is>
+      </c>
+      <c r="B2445" t="inlineStr">
+        <is>
+          <t>tamilpsd-2954.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2446">
+      <c r="A2446" s="3" t="inlineStr">
+        <is>
+          <t>4213.psd</t>
+        </is>
+      </c>
+      <c r="B2446" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2955.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2447">
+      <c r="A2447" t="inlineStr">
+        <is>
+          <t>4212.psd</t>
+        </is>
+      </c>
+      <c r="B2447" t="inlineStr">
+        <is>
+          <t>tamilpsd-2956.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2448">
+      <c r="A2448" s="3" t="inlineStr">
+        <is>
+          <t>4211.psd</t>
+        </is>
+      </c>
+      <c r="B2448" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2957.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2449">
+      <c r="A2449" t="inlineStr">
+        <is>
+          <t>4210.psd</t>
+        </is>
+      </c>
+      <c r="B2449" t="inlineStr">
+        <is>
+          <t>tamilpsd-2958.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2450">
+      <c r="A2450" s="3" t="inlineStr">
+        <is>
+          <t>4209.psd</t>
+        </is>
+      </c>
+      <c r="B2450" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2959.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2451">
+      <c r="A2451" t="inlineStr">
+        <is>
+          <t>4208.psd</t>
+        </is>
+      </c>
+      <c r="B2451" t="inlineStr">
+        <is>
+          <t>tamilpsd-2960.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2452">
+      <c r="A2452" s="3" t="inlineStr">
+        <is>
+          <t>4207.psd</t>
+        </is>
+      </c>
+      <c r="B2452" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2961.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2453">
+      <c r="A2453" t="inlineStr">
+        <is>
+          <t>4206.psd</t>
+        </is>
+      </c>
+      <c r="B2453" t="inlineStr">
+        <is>
+          <t>tamilpsd-2962.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2454">
+      <c r="A2454" s="3" t="inlineStr">
+        <is>
+          <t>4205.psd</t>
+        </is>
+      </c>
+      <c r="B2454" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2963.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2455">
+      <c r="A2455" t="inlineStr">
+        <is>
+          <t>4204.psd</t>
+        </is>
+      </c>
+      <c r="B2455" t="inlineStr">
+        <is>
+          <t>tamilpsd-2964.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2456">
+      <c r="A2456" s="3" t="inlineStr">
+        <is>
+          <t>4203.psd</t>
+        </is>
+      </c>
+      <c r="B2456" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2965.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2457">
+      <c r="A2457" t="inlineStr">
+        <is>
+          <t>4202.psd</t>
+        </is>
+      </c>
+      <c r="B2457" t="inlineStr">
+        <is>
+          <t>tamilpsd-2966.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2458">
+      <c r="A2458" s="3" t="inlineStr">
+        <is>
+          <t>4201.psd</t>
+        </is>
+      </c>
+      <c r="B2458" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2967.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2459">
+      <c r="A2459" t="inlineStr">
+        <is>
+          <t>4200.psd</t>
+        </is>
+      </c>
+      <c r="B2459" t="inlineStr">
+        <is>
+          <t>tamilpsd-2968.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2460">
+      <c r="A2460" s="3" t="inlineStr">
+        <is>
+          <t>4199.psd</t>
+        </is>
+      </c>
+      <c r="B2460" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2969.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2461">
+      <c r="A2461" t="inlineStr">
+        <is>
+          <t>4198.psd</t>
+        </is>
+      </c>
+      <c r="B2461" t="inlineStr">
+        <is>
+          <t>tamilpsd-2970.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2462">
+      <c r="A2462" s="3" t="inlineStr">
+        <is>
+          <t>4197.psd</t>
+        </is>
+      </c>
+      <c r="B2462" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2971.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2463">
+      <c r="A2463" t="inlineStr">
+        <is>
+          <t>4196.psd</t>
+        </is>
+      </c>
+      <c r="B2463" t="inlineStr">
+        <is>
+          <t>tamilpsd-2972.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2464">
+      <c r="A2464" s="3" t="inlineStr">
+        <is>
+          <t>4195.psd</t>
+        </is>
+      </c>
+      <c r="B2464" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2973.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2465">
+      <c r="A2465" t="inlineStr">
+        <is>
+          <t>4194.psd</t>
+        </is>
+      </c>
+      <c r="B2465" t="inlineStr">
+        <is>
+          <t>tamilpsd-2974.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2466">
+      <c r="A2466" s="3" t="inlineStr">
+        <is>
+          <t>4193.psd</t>
+        </is>
+      </c>
+      <c r="B2466" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2975.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2467">
+      <c r="A2467" t="inlineStr">
+        <is>
+          <t>4192.psd</t>
+        </is>
+      </c>
+      <c r="B2467" t="inlineStr">
+        <is>
+          <t>tamilpsd-2976.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2468">
+      <c r="A2468" s="3" t="inlineStr">
+        <is>
+          <t>4191.psd</t>
+        </is>
+      </c>
+      <c r="B2468" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2977.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2469">
+      <c r="A2469" t="inlineStr">
+        <is>
+          <t>4190.psd</t>
+        </is>
+      </c>
+      <c r="B2469" t="inlineStr">
+        <is>
+          <t>tamilpsd-2978.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2470">
+      <c r="A2470" s="3" t="inlineStr">
+        <is>
+          <t>4189.psd</t>
+        </is>
+      </c>
+      <c r="B2470" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2979.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2471">
+      <c r="A2471" t="inlineStr">
+        <is>
+          <t>4243.psd</t>
+        </is>
+      </c>
+      <c r="B2471" t="inlineStr">
+        <is>
+          <t>tamilpsd-2980.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2472">
+      <c r="A2472" s="3" t="inlineStr">
+        <is>
+          <t>4167.psd</t>
+        </is>
+      </c>
+      <c r="B2472" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2981.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2473">
+      <c r="A2473" t="inlineStr">
+        <is>
+          <t>4166.psd</t>
+        </is>
+      </c>
+      <c r="B2473" t="inlineStr">
+        <is>
+          <t>tamilpsd-2982.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2474">
+      <c r="A2474" s="3" t="inlineStr">
+        <is>
+          <t>4165.psd</t>
+        </is>
+      </c>
+      <c r="B2474" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2983.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2475">
+      <c r="A2475" t="inlineStr">
+        <is>
+          <t>4164.psd</t>
+        </is>
+      </c>
+      <c r="B2475" t="inlineStr">
+        <is>
+          <t>tamilpsd-2984.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2476">
+      <c r="A2476" s="3" t="inlineStr">
+        <is>
+          <t>4163.psd</t>
+        </is>
+      </c>
+      <c r="B2476" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2985.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2477">
+      <c r="A2477" t="inlineStr">
+        <is>
+          <t>4162.psd</t>
+        </is>
+      </c>
+      <c r="B2477" t="inlineStr">
+        <is>
+          <t>tamilpsd-2986.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2478">
+      <c r="A2478" s="3" t="inlineStr">
+        <is>
+          <t>4161.psd</t>
+        </is>
+      </c>
+      <c r="B2478" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2987.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2479">
+      <c r="A2479" t="inlineStr">
+        <is>
+          <t>4160.psd</t>
+        </is>
+      </c>
+      <c r="B2479" t="inlineStr">
+        <is>
+          <t>tamilpsd-2988.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2480">
+      <c r="A2480" s="3" t="inlineStr">
+        <is>
+          <t>4159.psd</t>
+        </is>
+      </c>
+      <c r="B2480" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2989.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2481">
+      <c r="A2481" t="inlineStr">
+        <is>
+          <t>4158.psd</t>
+        </is>
+      </c>
+      <c r="B2481" t="inlineStr">
+        <is>
+          <t>tamilpsd-2990.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2482">
+      <c r="A2482" s="3" t="inlineStr">
+        <is>
+          <t>4157.psd</t>
+        </is>
+      </c>
+      <c r="B2482" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2991.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2483">
+      <c r="A2483" t="inlineStr">
+        <is>
+          <t>4156.psd</t>
+        </is>
+      </c>
+      <c r="B2483" t="inlineStr">
+        <is>
+          <t>tamilpsd-2992.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2484">
+      <c r="A2484" s="3" t="inlineStr">
+        <is>
+          <t>4175.psd</t>
+        </is>
+      </c>
+      <c r="B2484" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2993.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2485">
+      <c r="A2485" t="inlineStr">
+        <is>
+          <t>4174.psd</t>
+        </is>
+      </c>
+      <c r="B2485" t="inlineStr">
+        <is>
+          <t>tamilpsd-2994.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2486">
+      <c r="A2486" s="3" t="inlineStr">
+        <is>
+          <t>4173.psd</t>
+        </is>
+      </c>
+      <c r="B2486" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2995.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2487">
+      <c r="A2487" t="inlineStr">
+        <is>
+          <t>4172.psd</t>
+        </is>
+      </c>
+      <c r="B2487" t="inlineStr">
+        <is>
+          <t>tamilpsd-2996.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2488">
+      <c r="A2488" s="3" t="inlineStr">
+        <is>
+          <t>4171.psd</t>
+        </is>
+      </c>
+      <c r="B2488" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2997.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2489">
+      <c r="A2489" t="inlineStr">
+        <is>
+          <t>4170.psd</t>
+        </is>
+      </c>
+      <c r="B2489" t="inlineStr">
+        <is>
+          <t>tamilpsd-2998.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2490">
+      <c r="A2490" s="3" t="inlineStr">
+        <is>
+          <t>4169.psd</t>
+        </is>
+      </c>
+      <c r="B2490" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-2999.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2491">
+      <c r="A2491" t="inlineStr">
+        <is>
+          <t>4168.psd</t>
+        </is>
+      </c>
+      <c r="B2491" t="inlineStr">
+        <is>
+          <t>tamilpsd-3000.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2492">
+      <c r="A2492" s="3" t="inlineStr">
+        <is>
+          <t>4154.psd</t>
+        </is>
+      </c>
+      <c r="B2492" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3001.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2493">
+      <c r="A2493" t="inlineStr">
+        <is>
+          <t>4153.psd</t>
+        </is>
+      </c>
+      <c r="B2493" t="inlineStr">
+        <is>
+          <t>tamilpsd-3002.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2494">
+      <c r="A2494" s="3" t="inlineStr">
+        <is>
+          <t>4152.psd</t>
+        </is>
+      </c>
+      <c r="B2494" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3003.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2495">
+      <c r="A2495" t="inlineStr">
+        <is>
+          <t>4151.psd</t>
+        </is>
+      </c>
+      <c r="B2495" t="inlineStr">
+        <is>
+          <t>tamilpsd-3004.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2496">
+      <c r="A2496" s="3" t="inlineStr">
+        <is>
+          <t>4150.psd</t>
+        </is>
+      </c>
+      <c r="B2496" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3005.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2497">
+      <c r="A2497" t="inlineStr">
+        <is>
+          <t>4149.psd</t>
+        </is>
+      </c>
+      <c r="B2497" t="inlineStr">
+        <is>
+          <t>tamilpsd-3006.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2498">
+      <c r="A2498" s="3" t="inlineStr">
+        <is>
+          <t>4148.psd</t>
+        </is>
+      </c>
+      <c r="B2498" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3007.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2499">
+      <c r="A2499" t="inlineStr">
+        <is>
+          <t>4147.psd</t>
+        </is>
+      </c>
+      <c r="B2499" t="inlineStr">
+        <is>
+          <t>tamilpsd-3008.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2500">
+      <c r="A2500" s="3" t="inlineStr">
+        <is>
+          <t>4146.psd</t>
+        </is>
+      </c>
+      <c r="B2500" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3009.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2501">
+      <c r="A2501" t="inlineStr">
+        <is>
+          <t>4145.psd</t>
+        </is>
+      </c>
+      <c r="B2501" t="inlineStr">
+        <is>
+          <t>tamilpsd-3010.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2502">
+      <c r="A2502" s="3" t="inlineStr">
+        <is>
+          <t>4144.psd</t>
+        </is>
+      </c>
+      <c r="B2502" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3011.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2503">
+      <c r="A2503" t="inlineStr">
+        <is>
+          <t>4143.psd</t>
+        </is>
+      </c>
+      <c r="B2503" t="inlineStr">
+        <is>
+          <t>tamilpsd-3012.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2504">
+      <c r="A2504" s="3" t="inlineStr">
+        <is>
+          <t>4142.psd</t>
+        </is>
+      </c>
+      <c r="B2504" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3013.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2505">
+      <c r="A2505" t="inlineStr">
+        <is>
+          <t>4141.psd</t>
+        </is>
+      </c>
+      <c r="B2505" t="inlineStr">
+        <is>
+          <t>tamilpsd-3014.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2506">
+      <c r="A2506" s="3" t="inlineStr">
+        <is>
+          <t>4140.psd</t>
+        </is>
+      </c>
+      <c r="B2506" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3015.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2507">
+      <c r="A2507" t="inlineStr">
+        <is>
+          <t>4139.psd</t>
+        </is>
+      </c>
+      <c r="B2507" t="inlineStr">
+        <is>
+          <t>tamilpsd-3016.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2508">
+      <c r="A2508" s="3" t="inlineStr">
+        <is>
+          <t>4138.psd</t>
+        </is>
+      </c>
+      <c r="B2508" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3017.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2509">
+      <c r="A2509" t="inlineStr">
+        <is>
+          <t>4137.psd</t>
+        </is>
+      </c>
+      <c r="B2509" t="inlineStr">
+        <is>
+          <t>tamilpsd-3018.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2510">
+      <c r="A2510" s="3" t="inlineStr">
+        <is>
+          <t>4136.psd</t>
+        </is>
+      </c>
+      <c r="B2510" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3019.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2511">
+      <c r="A2511" t="inlineStr">
+        <is>
+          <t>4155.psd</t>
+        </is>
+      </c>
+      <c r="B2511" t="inlineStr">
+        <is>
+          <t>tamilpsd-3020.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2512">
+      <c r="A2512" s="3" t="inlineStr">
+        <is>
+          <t>4134.psd</t>
+        </is>
+      </c>
+      <c r="B2512" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3021.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2513">
+      <c r="A2513" t="inlineStr">
+        <is>
+          <t>4133.psd</t>
+        </is>
+      </c>
+      <c r="B2513" t="inlineStr">
+        <is>
+          <t>tamilpsd-3022.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2514">
+      <c r="A2514" s="3" t="inlineStr">
+        <is>
+          <t>4132.psd</t>
+        </is>
+      </c>
+      <c r="B2514" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3023.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2515">
+      <c r="A2515" t="inlineStr">
+        <is>
+          <t>4131.psd</t>
+        </is>
+      </c>
+      <c r="B2515" t="inlineStr">
+        <is>
+          <t>tamilpsd-3024.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2516">
+      <c r="A2516" s="3" t="inlineStr">
+        <is>
+          <t>4130.psd</t>
+        </is>
+      </c>
+      <c r="B2516" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3025.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2517">
+      <c r="A2517" t="inlineStr">
+        <is>
+          <t>4129.psd</t>
+        </is>
+      </c>
+      <c r="B2517" t="inlineStr">
+        <is>
+          <t>tamilpsd-3026.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2518">
+      <c r="A2518" s="3" t="inlineStr">
+        <is>
+          <t>4128.psd</t>
+        </is>
+      </c>
+      <c r="B2518" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3027.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2519">
+      <c r="A2519" t="inlineStr">
+        <is>
+          <t>4127.PSD</t>
+        </is>
+      </c>
+      <c r="B2519" t="inlineStr">
+        <is>
+          <t>tamilpsd-3028.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2520">
+      <c r="A2520" s="3" t="inlineStr">
+        <is>
+          <t>4126.psd</t>
+        </is>
+      </c>
+      <c r="B2520" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3029.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2521">
+      <c r="A2521" t="inlineStr">
+        <is>
+          <t>4125.psd</t>
+        </is>
+      </c>
+      <c r="B2521" t="inlineStr">
+        <is>
+          <t>tamilpsd-3030.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2522">
+      <c r="A2522" s="3" t="inlineStr">
+        <is>
+          <t>4124.psd</t>
+        </is>
+      </c>
+      <c r="B2522" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3031.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2523">
+      <c r="A2523" t="inlineStr">
+        <is>
+          <t>4123.psd</t>
+        </is>
+      </c>
+      <c r="B2523" t="inlineStr">
+        <is>
+          <t>tamilpsd-3032.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2524">
+      <c r="A2524" s="3" t="inlineStr">
+        <is>
+          <t>4122.psd</t>
+        </is>
+      </c>
+      <c r="B2524" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3033.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2525">
+      <c r="A2525" t="inlineStr">
+        <is>
+          <t>4121.psd</t>
+        </is>
+      </c>
+      <c r="B2525" t="inlineStr">
+        <is>
+          <t>tamilpsd-3034.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2526">
+      <c r="A2526" s="3" t="inlineStr">
+        <is>
+          <t>4120.psd</t>
+        </is>
+      </c>
+      <c r="B2526" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3035.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2527">
+      <c r="A2527" t="inlineStr">
+        <is>
+          <t>4119.psd</t>
+        </is>
+      </c>
+      <c r="B2527" t="inlineStr">
+        <is>
+          <t>tamilpsd-3036.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2528">
+      <c r="A2528" s="3" t="inlineStr">
+        <is>
+          <t>4118.psd</t>
+        </is>
+      </c>
+      <c r="B2528" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3037.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2529">
+      <c r="A2529" t="inlineStr">
+        <is>
+          <t>4117.psd</t>
+        </is>
+      </c>
+      <c r="B2529" t="inlineStr">
+        <is>
+          <t>tamilpsd-3038.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2530">
+      <c r="A2530" s="3" t="inlineStr">
+        <is>
+          <t>4116.psd</t>
+        </is>
+      </c>
+      <c r="B2530" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3039.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2531">
+      <c r="A2531" t="inlineStr">
+        <is>
+          <t>4115.psd</t>
+        </is>
+      </c>
+      <c r="B2531" t="inlineStr">
+        <is>
+          <t>tamilpsd-3040.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2532">
+      <c r="A2532" s="3" t="inlineStr">
+        <is>
+          <t>4114.psd</t>
+        </is>
+      </c>
+      <c r="B2532" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3041.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2533">
+      <c r="A2533" t="inlineStr">
+        <is>
+          <t>4113.psd</t>
+        </is>
+      </c>
+      <c r="B2533" t="inlineStr">
+        <is>
+          <t>tamilpsd-3042.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2534">
+      <c r="A2534" s="3" t="inlineStr">
+        <is>
+          <t>4112.psd</t>
+        </is>
+      </c>
+      <c r="B2534" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3043.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2535">
+      <c r="A2535" t="inlineStr">
+        <is>
+          <t>4111.psd</t>
+        </is>
+      </c>
+      <c r="B2535" t="inlineStr">
+        <is>
+          <t>tamilpsd-3044.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2536">
+      <c r="A2536" s="3" t="inlineStr">
+        <is>
+          <t>4110.psd</t>
+        </is>
+      </c>
+      <c r="B2536" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3045.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2537">
+      <c r="A2537" t="inlineStr">
+        <is>
+          <t>4109.psd</t>
+        </is>
+      </c>
+      <c r="B2537" t="inlineStr">
+        <is>
+          <t>tamilpsd-3046.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2538">
+      <c r="A2538" s="3" t="inlineStr">
+        <is>
+          <t>4108.psd</t>
+        </is>
+      </c>
+      <c r="B2538" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3047.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2539">
+      <c r="A2539" t="inlineStr">
+        <is>
+          <t>4107.psd</t>
+        </is>
+      </c>
+      <c r="B2539" t="inlineStr">
+        <is>
+          <t>tamilpsd-3048.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2540">
+      <c r="A2540" s="3" t="inlineStr">
+        <is>
+          <t>4106.psd</t>
+        </is>
+      </c>
+      <c r="B2540" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3049.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2541">
+      <c r="A2541" t="inlineStr">
+        <is>
+          <t>4105.psd</t>
+        </is>
+      </c>
+      <c r="B2541" t="inlineStr">
+        <is>
+          <t>tamilpsd-3050.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2542">
+      <c r="A2542" s="3" t="inlineStr">
+        <is>
+          <t>4104.psd</t>
+        </is>
+      </c>
+      <c r="B2542" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3051.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2543">
+      <c r="A2543" t="inlineStr">
+        <is>
+          <t>4103.psd</t>
+        </is>
+      </c>
+      <c r="B2543" t="inlineStr">
+        <is>
+          <t>tamilpsd-3052.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2544">
+      <c r="A2544" s="3" t="inlineStr">
+        <is>
+          <t>4102.psd</t>
+        </is>
+      </c>
+      <c r="B2544" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3053.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2545">
+      <c r="A2545" t="inlineStr">
+        <is>
+          <t>4101.psd</t>
+        </is>
+      </c>
+      <c r="B2545" t="inlineStr">
+        <is>
+          <t>tamilpsd-3054.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2546">
+      <c r="A2546" s="3" t="inlineStr">
+        <is>
+          <t>4100.psd</t>
+        </is>
+      </c>
+      <c r="B2546" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3055.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2547">
+      <c r="A2547" t="inlineStr">
+        <is>
+          <t>4099.psd</t>
+        </is>
+      </c>
+      <c r="B2547" t="inlineStr">
+        <is>
+          <t>tamilpsd-3056.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2548">
+      <c r="A2548" s="3" t="inlineStr">
+        <is>
+          <t>4098.psd</t>
+        </is>
+      </c>
+      <c r="B2548" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3057.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2549">
+      <c r="A2549" t="inlineStr">
+        <is>
+          <t>4097.psd</t>
+        </is>
+      </c>
+      <c r="B2549" t="inlineStr">
+        <is>
+          <t>tamilpsd-3058.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2550">
+      <c r="A2550" s="3" t="inlineStr">
+        <is>
+          <t>4096.psd</t>
+        </is>
+      </c>
+      <c r="B2550" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3059.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2551">
+      <c r="A2551" t="inlineStr">
+        <is>
+          <t>4095.psd</t>
+        </is>
+      </c>
+      <c r="B2551" t="inlineStr">
+        <is>
+          <t>tamilpsd-3060.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2552">
+      <c r="A2552" s="3" t="inlineStr">
+        <is>
+          <t>4094.psd</t>
+        </is>
+      </c>
+      <c r="B2552" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3061.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2553">
+      <c r="A2553" t="inlineStr">
+        <is>
+          <t>4093.psd</t>
+        </is>
+      </c>
+      <c r="B2553" t="inlineStr">
+        <is>
+          <t>tamilpsd-3062.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2554">
+      <c r="A2554" s="3" t="inlineStr">
+        <is>
+          <t>4092.psd</t>
+        </is>
+      </c>
+      <c r="B2554" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3063.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2555">
+      <c r="A2555" t="inlineStr">
+        <is>
+          <t>4091.psd</t>
+        </is>
+      </c>
+      <c r="B2555" t="inlineStr">
+        <is>
+          <t>tamilpsd-3064.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2556">
+      <c r="A2556" s="3" t="inlineStr">
+        <is>
+          <t>4090.psd</t>
+        </is>
+      </c>
+      <c r="B2556" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3065.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2557">
+      <c r="A2557" t="inlineStr">
+        <is>
+          <t>4089.psd</t>
+        </is>
+      </c>
+      <c r="B2557" t="inlineStr">
+        <is>
+          <t>tamilpsd-3066.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2558">
+      <c r="A2558" s="3" t="inlineStr">
+        <is>
+          <t>4088.psd</t>
+        </is>
+      </c>
+      <c r="B2558" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3067.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2559">
+      <c r="A2559" t="inlineStr">
+        <is>
+          <t>4087.psd</t>
+        </is>
+      </c>
+      <c r="B2559" t="inlineStr">
+        <is>
+          <t>tamilpsd-3068.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2560">
+      <c r="A2560" s="3" t="inlineStr">
+        <is>
+          <t>4086.psd</t>
+        </is>
+      </c>
+      <c r="B2560" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3069.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2561">
+      <c r="A2561" t="inlineStr">
+        <is>
+          <t>4085.psd</t>
+        </is>
+      </c>
+      <c r="B2561" t="inlineStr">
+        <is>
+          <t>tamilpsd-3070.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2562">
+      <c r="A2562" s="3" t="inlineStr">
+        <is>
+          <t>4083.psd</t>
+        </is>
+      </c>
+      <c r="B2562" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3071.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2563">
+      <c r="A2563" t="inlineStr">
+        <is>
+          <t>4084.psd</t>
+        </is>
+      </c>
+      <c r="B2563" t="inlineStr">
+        <is>
+          <t>tamilpsd-3072.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2564">
+      <c r="A2564" s="3" t="inlineStr">
+        <is>
+          <t>4082.psd</t>
+        </is>
+      </c>
+      <c r="B2564" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3073.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2565">
+      <c r="A2565" t="inlineStr">
+        <is>
+          <t>4081.psd</t>
+        </is>
+      </c>
+      <c r="B2565" t="inlineStr">
+        <is>
+          <t>tamilpsd-3074.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2566">
+      <c r="A2566" s="3" t="inlineStr">
+        <is>
+          <t>4080.psd</t>
+        </is>
+      </c>
+      <c r="B2566" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3075.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2567">
+      <c r="A2567" t="inlineStr">
+        <is>
+          <t>4079.psd</t>
+        </is>
+      </c>
+      <c r="B2567" t="inlineStr">
+        <is>
+          <t>tamilpsd-3076.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2568">
+      <c r="A2568" s="3" t="inlineStr">
+        <is>
+          <t>4078.psd</t>
+        </is>
+      </c>
+      <c r="B2568" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3077.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2569">
+      <c r="A2569" t="inlineStr">
+        <is>
+          <t>4077.psd</t>
+        </is>
+      </c>
+      <c r="B2569" t="inlineStr">
+        <is>
+          <t>tamilpsd-3078.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2570">
+      <c r="A2570" s="3" t="inlineStr">
+        <is>
+          <t>4076.psd</t>
+        </is>
+      </c>
+      <c r="B2570" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3079.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2571">
+      <c r="A2571" t="inlineStr">
+        <is>
+          <t>4075.psd</t>
+        </is>
+      </c>
+      <c r="B2571" t="inlineStr">
+        <is>
+          <t>tamilpsd-3080.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2572">
+      <c r="A2572" s="3" t="inlineStr">
+        <is>
+          <t>4074.psd</t>
+        </is>
+      </c>
+      <c r="B2572" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3081.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2573">
+      <c r="A2573" t="inlineStr">
+        <is>
+          <t>4073.psd</t>
+        </is>
+      </c>
+      <c r="B2573" t="inlineStr">
+        <is>
+          <t>tamilpsd-3082.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2574">
+      <c r="A2574" s="3" t="inlineStr">
+        <is>
+          <t>4072.psd</t>
+        </is>
+      </c>
+      <c r="B2574" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3083.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2575">
+      <c r="A2575" t="inlineStr">
+        <is>
+          <t>4135.psd</t>
+        </is>
+      </c>
+      <c r="B2575" t="inlineStr">
+        <is>
+          <t>tamilpsd-3084.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2576">
+      <c r="A2576" s="3" t="inlineStr">
+        <is>
+          <t>4070.psd</t>
+        </is>
+      </c>
+      <c r="B2576" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3085.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2577">
+      <c r="A2577" t="inlineStr">
+        <is>
+          <t>4069.psd</t>
+        </is>
+      </c>
+      <c r="B2577" t="inlineStr">
+        <is>
+          <t>tamilpsd-3086.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2578">
+      <c r="A2578" s="3" t="inlineStr">
+        <is>
+          <t>4068.psd</t>
+        </is>
+      </c>
+      <c r="B2578" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3087.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2579">
+      <c r="A2579" t="inlineStr">
+        <is>
+          <t>4067.psd</t>
+        </is>
+      </c>
+      <c r="B2579" t="inlineStr">
+        <is>
+          <t>tamilpsd-3088.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2580">
+      <c r="A2580" s="3" t="inlineStr">
+        <is>
+          <t>4066.psd</t>
+        </is>
+      </c>
+      <c r="B2580" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3089.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2581">
+      <c r="A2581" t="inlineStr">
+        <is>
+          <t>4065.psd</t>
+        </is>
+      </c>
+      <c r="B2581" t="inlineStr">
+        <is>
+          <t>tamilpsd-3090.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2582">
+      <c r="A2582" s="3" t="inlineStr">
+        <is>
+          <t>4064.psd</t>
+        </is>
+      </c>
+      <c r="B2582" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3091.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2583">
+      <c r="A2583" t="inlineStr">
+        <is>
+          <t>4063.psd</t>
+        </is>
+      </c>
+      <c r="B2583" t="inlineStr">
+        <is>
+          <t>tamilpsd-3092.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2584">
+      <c r="A2584" s="3" t="inlineStr">
+        <is>
+          <t>4062.psd</t>
+        </is>
+      </c>
+      <c r="B2584" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3093.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2585">
+      <c r="A2585" t="inlineStr">
+        <is>
+          <t>4061.psd</t>
+        </is>
+      </c>
+      <c r="B2585" t="inlineStr">
+        <is>
+          <t>tamilpsd-3094.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2586">
+      <c r="A2586" s="3" t="inlineStr">
+        <is>
+          <t>4060.psd</t>
+        </is>
+      </c>
+      <c r="B2586" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3095.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2587">
+      <c r="A2587" t="inlineStr">
+        <is>
+          <t>4059.psd</t>
+        </is>
+      </c>
+      <c r="B2587" t="inlineStr">
+        <is>
+          <t>tamilpsd-3096.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2588">
+      <c r="A2588" s="3" t="inlineStr">
+        <is>
+          <t>4058.psd</t>
+        </is>
+      </c>
+      <c r="B2588" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3097.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2589">
+      <c r="A2589" t="inlineStr">
+        <is>
+          <t>4057.psd</t>
+        </is>
+      </c>
+      <c r="B2589" t="inlineStr">
+        <is>
+          <t>tamilpsd-3098.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2590">
+      <c r="A2590" s="3" t="inlineStr">
+        <is>
+          <t>4056.psd</t>
+        </is>
+      </c>
+      <c r="B2590" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3099.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2591">
+      <c r="A2591" t="inlineStr">
+        <is>
+          <t>4055.psd</t>
+        </is>
+      </c>
+      <c r="B2591" t="inlineStr">
+        <is>
+          <t>tamilpsd-3100.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2592">
+      <c r="A2592" s="3" t="inlineStr">
+        <is>
+          <t>4054.psd</t>
+        </is>
+      </c>
+      <c r="B2592" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3101.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2593">
+      <c r="A2593" t="inlineStr">
+        <is>
+          <t>4053.psd</t>
+        </is>
+      </c>
+      <c r="B2593" t="inlineStr">
+        <is>
+          <t>tamilpsd-3102.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2594">
+      <c r="A2594" s="3" t="inlineStr">
+        <is>
+          <t>4052.psd</t>
+        </is>
+      </c>
+      <c r="B2594" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3103.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2595">
+      <c r="A2595" t="inlineStr">
+        <is>
+          <t>4051.psd</t>
+        </is>
+      </c>
+      <c r="B2595" t="inlineStr">
+        <is>
+          <t>tamilpsd-3104.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2596">
+      <c r="A2596" s="3" t="inlineStr">
+        <is>
+          <t>4050.psd</t>
+        </is>
+      </c>
+      <c r="B2596" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3105.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2597">
+      <c r="A2597" t="inlineStr">
+        <is>
+          <t>4049.psd</t>
+        </is>
+      </c>
+      <c r="B2597" t="inlineStr">
+        <is>
+          <t>tamilpsd-3106.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2598">
+      <c r="A2598" s="3" t="inlineStr">
+        <is>
+          <t>4048.psd</t>
+        </is>
+      </c>
+      <c r="B2598" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3107.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2599">
+      <c r="A2599" t="inlineStr">
+        <is>
+          <t>4047.psd</t>
+        </is>
+      </c>
+      <c r="B2599" t="inlineStr">
+        <is>
+          <t>tamilpsd-3108.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2600">
+      <c r="A2600" s="3" t="inlineStr">
+        <is>
+          <t>4071.psd</t>
+        </is>
+      </c>
+      <c r="B2600" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3109.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2601">
+      <c r="A2601" t="inlineStr">
+        <is>
+          <t>4044.psd</t>
+        </is>
+      </c>
+      <c r="B2601" t="inlineStr">
+        <is>
+          <t>tamilpsd-3110.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2602">
+      <c r="A2602" s="3" t="inlineStr">
+        <is>
+          <t>4043.psd</t>
+        </is>
+      </c>
+      <c r="B2602" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3111.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2603">
+      <c r="A2603" t="inlineStr">
+        <is>
+          <t>4042.psd</t>
+        </is>
+      </c>
+      <c r="B2603" t="inlineStr">
+        <is>
+          <t>tamilpsd-3112.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2604">
+      <c r="A2604" s="3" t="inlineStr">
+        <is>
+          <t>4041.psd</t>
+        </is>
+      </c>
+      <c r="B2604" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3113.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2605">
+      <c r="A2605" t="inlineStr">
+        <is>
+          <t>4040.psd</t>
+        </is>
+      </c>
+      <c r="B2605" t="inlineStr">
+        <is>
+          <t>tamilpsd-3114.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2606">
+      <c r="A2606" s="3" t="inlineStr">
+        <is>
+          <t>4039.psd</t>
+        </is>
+      </c>
+      <c r="B2606" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3115.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2607">
+      <c r="A2607" t="inlineStr">
+        <is>
+          <t>4038.psd</t>
+        </is>
+      </c>
+      <c r="B2607" t="inlineStr">
+        <is>
+          <t>tamilpsd-3116.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2608">
+      <c r="A2608" s="3" t="inlineStr">
+        <is>
+          <t>4037.psd</t>
+        </is>
+      </c>
+      <c r="B2608" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3117.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2609">
+      <c r="A2609" t="inlineStr">
+        <is>
+          <t>4036.psd</t>
+        </is>
+      </c>
+      <c r="B2609" t="inlineStr">
+        <is>
+          <t>tamilpsd-3118.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2610">
+      <c r="A2610" s="3" t="inlineStr">
+        <is>
+          <t>4035.psd</t>
+        </is>
+      </c>
+      <c r="B2610" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3119.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2611">
+      <c r="A2611" t="inlineStr">
+        <is>
+          <t>4034.psd</t>
+        </is>
+      </c>
+      <c r="B2611" t="inlineStr">
+        <is>
+          <t>tamilpsd-3120.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2612">
+      <c r="A2612" s="3" t="inlineStr">
+        <is>
+          <t>4033.psd</t>
+        </is>
+      </c>
+      <c r="B2612" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3121.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2613">
+      <c r="A2613" t="inlineStr">
+        <is>
+          <t>4032.psd</t>
+        </is>
+      </c>
+      <c r="B2613" t="inlineStr">
+        <is>
+          <t>tamilpsd-3122.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2614">
+      <c r="A2614" s="3" t="inlineStr">
+        <is>
+          <t>4031.psd</t>
+        </is>
+      </c>
+      <c r="B2614" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3123.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2615">
+      <c r="A2615" t="inlineStr">
+        <is>
+          <t>4030.psd</t>
+        </is>
+      </c>
+      <c r="B2615" t="inlineStr">
+        <is>
+          <t>tamilpsd-3124.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2616">
+      <c r="A2616" s="3" t="inlineStr">
+        <is>
+          <t>4029.psd</t>
+        </is>
+      </c>
+      <c r="B2616" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3125.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2617">
+      <c r="A2617" t="inlineStr">
+        <is>
+          <t>4028.psd</t>
+        </is>
+      </c>
+      <c r="B2617" t="inlineStr">
+        <is>
+          <t>tamilpsd-3126.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2618">
+      <c r="A2618" s="3" t="inlineStr">
+        <is>
+          <t>4027.psd</t>
+        </is>
+      </c>
+      <c r="B2618" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3127.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2619">
+      <c r="A2619" t="inlineStr">
+        <is>
+          <t>4026.psd</t>
+        </is>
+      </c>
+      <c r="B2619" t="inlineStr">
+        <is>
+          <t>tamilpsd-3128.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2620">
+      <c r="A2620" s="3" t="inlineStr">
+        <is>
+          <t>4025.psd</t>
+        </is>
+      </c>
+      <c r="B2620" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3129.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2621">
+      <c r="A2621" t="inlineStr">
+        <is>
+          <t>4024.psd</t>
+        </is>
+      </c>
+      <c r="B2621" t="inlineStr">
+        <is>
+          <t>tamilpsd-3130.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2622">
+      <c r="A2622" s="3" t="inlineStr">
+        <is>
+          <t>4023.psd</t>
+        </is>
+      </c>
+      <c r="B2622" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3131.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2623">
+      <c r="A2623" t="inlineStr">
+        <is>
+          <t>4022.psd</t>
+        </is>
+      </c>
+      <c r="B2623" t="inlineStr">
+        <is>
+          <t>tamilpsd-3132.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2624">
+      <c r="A2624" s="3" t="inlineStr">
+        <is>
+          <t>4021.psd</t>
+        </is>
+      </c>
+      <c r="B2624" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3133.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2625">
+      <c r="A2625" t="inlineStr">
+        <is>
+          <t>4020.psd</t>
+        </is>
+      </c>
+      <c r="B2625" t="inlineStr">
+        <is>
+          <t>tamilpsd-3134.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2626">
+      <c r="A2626" s="3" t="inlineStr">
+        <is>
+          <t>4019.psd</t>
+        </is>
+      </c>
+      <c r="B2626" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3135.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2627">
+      <c r="A2627" t="inlineStr">
+        <is>
+          <t>4018.psd</t>
+        </is>
+      </c>
+      <c r="B2627" t="inlineStr">
+        <is>
+          <t>tamilpsd-3136.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2628">
+      <c r="A2628" s="3" t="inlineStr">
+        <is>
+          <t>4017.psd</t>
+        </is>
+      </c>
+      <c r="B2628" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3137.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2629">
+      <c r="A2629" t="inlineStr">
+        <is>
+          <t>4016.psd</t>
+        </is>
+      </c>
+      <c r="B2629" t="inlineStr">
+        <is>
+          <t>tamilpsd-3138.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2630">
+      <c r="A2630" s="3" t="inlineStr">
+        <is>
+          <t>4015.psd</t>
+        </is>
+      </c>
+      <c r="B2630" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3139.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2631">
+      <c r="A2631" t="inlineStr">
+        <is>
+          <t>4014.psd</t>
+        </is>
+      </c>
+      <c r="B2631" t="inlineStr">
+        <is>
+          <t>tamilpsd-3140.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2632">
+      <c r="A2632" s="3" t="inlineStr">
+        <is>
+          <t>4013.psd</t>
+        </is>
+      </c>
+      <c r="B2632" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3141.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2633">
+      <c r="A2633" t="inlineStr">
+        <is>
+          <t>4012.psd</t>
+        </is>
+      </c>
+      <c r="B2633" t="inlineStr">
+        <is>
+          <t>tamilpsd-3142.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2634">
+      <c r="A2634" s="3" t="inlineStr">
+        <is>
+          <t>4011.psd</t>
+        </is>
+      </c>
+      <c r="B2634" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-3143.psd</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
🤖 Progress: 2026-04-20 17:06 UTC
</commit_message>
<xml_diff>
--- a/rename_log.xlsx
+++ b/rename_log.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2634"/>
+  <dimension ref="A1:B2961"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -31705,6 +31705,3930 @@
         </is>
       </c>
     </row>
+    <row r="2635">
+      <c r="A2635" t="inlineStr">
+        <is>
+          <t>4554.psd</t>
+        </is>
+      </c>
+      <c r="B2635" t="inlineStr">
+        <is>
+          <t>tamilpsd-5452.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2636">
+      <c r="A2636" s="3" t="inlineStr">
+        <is>
+          <t>4010.psd</t>
+        </is>
+      </c>
+      <c r="B2636" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5453.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2637">
+      <c r="A2637" t="inlineStr">
+        <is>
+          <t>4009.psd</t>
+        </is>
+      </c>
+      <c r="B2637" t="inlineStr">
+        <is>
+          <t>tamilpsd-5454.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2638">
+      <c r="A2638" s="3" t="inlineStr">
+        <is>
+          <t>4008.psd</t>
+        </is>
+      </c>
+      <c r="B2638" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5455.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2639">
+      <c r="A2639" t="inlineStr">
+        <is>
+          <t>4007.psd</t>
+        </is>
+      </c>
+      <c r="B2639" t="inlineStr">
+        <is>
+          <t>tamilpsd-5456.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2640">
+      <c r="A2640" s="3" t="inlineStr">
+        <is>
+          <t>4006.psd</t>
+        </is>
+      </c>
+      <c r="B2640" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5457.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2641">
+      <c r="A2641" t="inlineStr">
+        <is>
+          <t>4005.psd</t>
+        </is>
+      </c>
+      <c r="B2641" t="inlineStr">
+        <is>
+          <t>tamilpsd-5458.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2642">
+      <c r="A2642" s="3" t="inlineStr">
+        <is>
+          <t>4004.psd</t>
+        </is>
+      </c>
+      <c r="B2642" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5459.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2643">
+      <c r="A2643" t="inlineStr">
+        <is>
+          <t>4003.psd</t>
+        </is>
+      </c>
+      <c r="B2643" t="inlineStr">
+        <is>
+          <t>tamilpsd-5460.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2644">
+      <c r="A2644" s="3" t="inlineStr">
+        <is>
+          <t>4002.psd</t>
+        </is>
+      </c>
+      <c r="B2644" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5461.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2645">
+      <c r="A2645" t="inlineStr">
+        <is>
+          <t>4001.psd</t>
+        </is>
+      </c>
+      <c r="B2645" t="inlineStr">
+        <is>
+          <t>tamilpsd-5462.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2646">
+      <c r="A2646" s="3" t="inlineStr">
+        <is>
+          <t>4000.psd</t>
+        </is>
+      </c>
+      <c r="B2646" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5463.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2647">
+      <c r="A2647" t="inlineStr">
+        <is>
+          <t>3999.psd</t>
+        </is>
+      </c>
+      <c r="B2647" t="inlineStr">
+        <is>
+          <t>tamilpsd-5464.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2648">
+      <c r="A2648" s="3" t="inlineStr">
+        <is>
+          <t>3998.psd</t>
+        </is>
+      </c>
+      <c r="B2648" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5465.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2649">
+      <c r="A2649" t="inlineStr">
+        <is>
+          <t>3997.psd</t>
+        </is>
+      </c>
+      <c r="B2649" t="inlineStr">
+        <is>
+          <t>tamilpsd-5466.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2650">
+      <c r="A2650" s="3" t="inlineStr">
+        <is>
+          <t>4046.psd</t>
+        </is>
+      </c>
+      <c r="B2650" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5467.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2651">
+      <c r="A2651" t="inlineStr">
+        <is>
+          <t>3996.psd</t>
+        </is>
+      </c>
+      <c r="B2651" t="inlineStr">
+        <is>
+          <t>tamilpsd-5468.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2652">
+      <c r="A2652" s="3" t="inlineStr">
+        <is>
+          <t>3995.psd</t>
+        </is>
+      </c>
+      <c r="B2652" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5469.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2653">
+      <c r="A2653" t="inlineStr">
+        <is>
+          <t>3994.psd</t>
+        </is>
+      </c>
+      <c r="B2653" t="inlineStr">
+        <is>
+          <t>tamilpsd-5470.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2654">
+      <c r="A2654" s="3" t="inlineStr">
+        <is>
+          <t>3993.psd</t>
+        </is>
+      </c>
+      <c r="B2654" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5471.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2655">
+      <c r="A2655" t="inlineStr">
+        <is>
+          <t>3992.psd</t>
+        </is>
+      </c>
+      <c r="B2655" t="inlineStr">
+        <is>
+          <t>tamilpsd-5472.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2656">
+      <c r="A2656" s="3" t="inlineStr">
+        <is>
+          <t>3991.psd</t>
+        </is>
+      </c>
+      <c r="B2656" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5473.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2657">
+      <c r="A2657" t="inlineStr">
+        <is>
+          <t>3990.psd</t>
+        </is>
+      </c>
+      <c r="B2657" t="inlineStr">
+        <is>
+          <t>tamilpsd-5474.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2658">
+      <c r="A2658" s="3" t="inlineStr">
+        <is>
+          <t>3989.psd</t>
+        </is>
+      </c>
+      <c r="B2658" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5475.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2659">
+      <c r="A2659" t="inlineStr">
+        <is>
+          <t>3988.psd</t>
+        </is>
+      </c>
+      <c r="B2659" t="inlineStr">
+        <is>
+          <t>tamilpsd-5476.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2660">
+      <c r="A2660" s="3" t="inlineStr">
+        <is>
+          <t>3987.psd</t>
+        </is>
+      </c>
+      <c r="B2660" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5477.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2661">
+      <c r="A2661" t="inlineStr">
+        <is>
+          <t>3986.psd</t>
+        </is>
+      </c>
+      <c r="B2661" t="inlineStr">
+        <is>
+          <t>tamilpsd-5478.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2662">
+      <c r="A2662" s="3" t="inlineStr">
+        <is>
+          <t>3985.psd</t>
+        </is>
+      </c>
+      <c r="B2662" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5479.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2663">
+      <c r="A2663" t="inlineStr">
+        <is>
+          <t>3984.psd</t>
+        </is>
+      </c>
+      <c r="B2663" t="inlineStr">
+        <is>
+          <t>tamilpsd-5480.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2664">
+      <c r="A2664" s="3" t="inlineStr">
+        <is>
+          <t>3983.psd</t>
+        </is>
+      </c>
+      <c r="B2664" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5481.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2665">
+      <c r="A2665" t="inlineStr">
+        <is>
+          <t>3982.PSD</t>
+        </is>
+      </c>
+      <c r="B2665" t="inlineStr">
+        <is>
+          <t>tamilpsd-5482.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2666">
+      <c r="A2666" s="3" t="inlineStr">
+        <is>
+          <t>3981.psd</t>
+        </is>
+      </c>
+      <c r="B2666" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5483.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2667">
+      <c r="A2667" t="inlineStr">
+        <is>
+          <t>3980.psd</t>
+        </is>
+      </c>
+      <c r="B2667" t="inlineStr">
+        <is>
+          <t>tamilpsd-5484.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2668">
+      <c r="A2668" s="3" t="inlineStr">
+        <is>
+          <t>3979.psd</t>
+        </is>
+      </c>
+      <c r="B2668" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5485.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2669">
+      <c r="A2669" t="inlineStr">
+        <is>
+          <t>3978.psd</t>
+        </is>
+      </c>
+      <c r="B2669" t="inlineStr">
+        <is>
+          <t>tamilpsd-5486.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2670">
+      <c r="A2670" s="3" t="inlineStr">
+        <is>
+          <t>3977.psd</t>
+        </is>
+      </c>
+      <c r="B2670" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5487.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2671">
+      <c r="A2671" t="inlineStr">
+        <is>
+          <t>3976.psd</t>
+        </is>
+      </c>
+      <c r="B2671" t="inlineStr">
+        <is>
+          <t>tamilpsd-5488.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2672">
+      <c r="A2672" s="3" t="inlineStr">
+        <is>
+          <t>3975.psd</t>
+        </is>
+      </c>
+      <c r="B2672" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5489.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2673">
+      <c r="A2673" t="inlineStr">
+        <is>
+          <t>3974.psd</t>
+        </is>
+      </c>
+      <c r="B2673" t="inlineStr">
+        <is>
+          <t>tamilpsd-5490.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2674">
+      <c r="A2674" s="3" t="inlineStr">
+        <is>
+          <t>3973.psd</t>
+        </is>
+      </c>
+      <c r="B2674" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5491.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2675">
+      <c r="A2675" t="inlineStr">
+        <is>
+          <t>3972.psd</t>
+        </is>
+      </c>
+      <c r="B2675" t="inlineStr">
+        <is>
+          <t>tamilpsd-5492.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2676">
+      <c r="A2676" s="3" t="inlineStr">
+        <is>
+          <t>3971.psd</t>
+        </is>
+      </c>
+      <c r="B2676" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5493.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2677">
+      <c r="A2677" t="inlineStr">
+        <is>
+          <t>3970.psd</t>
+        </is>
+      </c>
+      <c r="B2677" t="inlineStr">
+        <is>
+          <t>tamilpsd-5494.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2678">
+      <c r="A2678" s="3" t="inlineStr">
+        <is>
+          <t>3969.psd</t>
+        </is>
+      </c>
+      <c r="B2678" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5495.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2679">
+      <c r="A2679" t="inlineStr">
+        <is>
+          <t>3968.psd</t>
+        </is>
+      </c>
+      <c r="B2679" t="inlineStr">
+        <is>
+          <t>tamilpsd-5496.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2680">
+      <c r="A2680" s="3" t="inlineStr">
+        <is>
+          <t>3967.psd</t>
+        </is>
+      </c>
+      <c r="B2680" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5497.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2681">
+      <c r="A2681" t="inlineStr">
+        <is>
+          <t>3966.psd</t>
+        </is>
+      </c>
+      <c r="B2681" t="inlineStr">
+        <is>
+          <t>tamilpsd-5498.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2682">
+      <c r="A2682" s="3" t="inlineStr">
+        <is>
+          <t>3965.psd</t>
+        </is>
+      </c>
+      <c r="B2682" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5499.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2683">
+      <c r="A2683" t="inlineStr">
+        <is>
+          <t>3964.psd</t>
+        </is>
+      </c>
+      <c r="B2683" t="inlineStr">
+        <is>
+          <t>tamilpsd-5500.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2684">
+      <c r="A2684" s="3" t="inlineStr">
+        <is>
+          <t>3963.psd</t>
+        </is>
+      </c>
+      <c r="B2684" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5501.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2685">
+      <c r="A2685" t="inlineStr">
+        <is>
+          <t>3962.psd</t>
+        </is>
+      </c>
+      <c r="B2685" t="inlineStr">
+        <is>
+          <t>tamilpsd-5502.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2686">
+      <c r="A2686" s="3" t="inlineStr">
+        <is>
+          <t>3961.psd</t>
+        </is>
+      </c>
+      <c r="B2686" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5503.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2687">
+      <c r="A2687" t="inlineStr">
+        <is>
+          <t>3960.psd</t>
+        </is>
+      </c>
+      <c r="B2687" t="inlineStr">
+        <is>
+          <t>tamilpsd-5504.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2688">
+      <c r="A2688" s="3" t="inlineStr">
+        <is>
+          <t>3959.psd</t>
+        </is>
+      </c>
+      <c r="B2688" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5505.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2689">
+      <c r="A2689" t="inlineStr">
+        <is>
+          <t>3958.psd</t>
+        </is>
+      </c>
+      <c r="B2689" t="inlineStr">
+        <is>
+          <t>tamilpsd-5506.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2690">
+      <c r="A2690" s="3" t="inlineStr">
+        <is>
+          <t>3957.psd</t>
+        </is>
+      </c>
+      <c r="B2690" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5507.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2691">
+      <c r="A2691" t="inlineStr">
+        <is>
+          <t>3956.psd</t>
+        </is>
+      </c>
+      <c r="B2691" t="inlineStr">
+        <is>
+          <t>tamilpsd-5508.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2692">
+      <c r="A2692" s="3" t="inlineStr">
+        <is>
+          <t>3955.psd</t>
+        </is>
+      </c>
+      <c r="B2692" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5509.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2693">
+      <c r="A2693" t="inlineStr">
+        <is>
+          <t>3954.psd</t>
+        </is>
+      </c>
+      <c r="B2693" t="inlineStr">
+        <is>
+          <t>tamilpsd-5510.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2694">
+      <c r="A2694" s="3" t="inlineStr">
+        <is>
+          <t>3953.psd</t>
+        </is>
+      </c>
+      <c r="B2694" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5511.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2695">
+      <c r="A2695" t="inlineStr">
+        <is>
+          <t>3952.psd</t>
+        </is>
+      </c>
+      <c r="B2695" t="inlineStr">
+        <is>
+          <t>tamilpsd-5512.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2696">
+      <c r="A2696" s="3" t="inlineStr">
+        <is>
+          <t>3951.psd</t>
+        </is>
+      </c>
+      <c r="B2696" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5513.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2697">
+      <c r="A2697" t="inlineStr">
+        <is>
+          <t>3950.psd</t>
+        </is>
+      </c>
+      <c r="B2697" t="inlineStr">
+        <is>
+          <t>tamilpsd-5514.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2698">
+      <c r="A2698" s="3" t="inlineStr">
+        <is>
+          <t>3949.psd</t>
+        </is>
+      </c>
+      <c r="B2698" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5515.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2699">
+      <c r="A2699" t="inlineStr">
+        <is>
+          <t>3948.psd</t>
+        </is>
+      </c>
+      <c r="B2699" t="inlineStr">
+        <is>
+          <t>tamilpsd-5516.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2700">
+      <c r="A2700" s="3" t="inlineStr">
+        <is>
+          <t>3947.PSD</t>
+        </is>
+      </c>
+      <c r="B2700" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5517.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2701">
+      <c r="A2701" t="inlineStr">
+        <is>
+          <t>3465.psd</t>
+        </is>
+      </c>
+      <c r="B2701" t="inlineStr">
+        <is>
+          <t>tamilpsd-5518.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2702">
+      <c r="A2702" s="3" t="inlineStr">
+        <is>
+          <t>3463.psd</t>
+        </is>
+      </c>
+      <c r="B2702" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5519.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2703">
+      <c r="A2703" t="inlineStr">
+        <is>
+          <t>3462.psd</t>
+        </is>
+      </c>
+      <c r="B2703" t="inlineStr">
+        <is>
+          <t>tamilpsd-5520.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2704">
+      <c r="A2704" s="3" t="inlineStr">
+        <is>
+          <t>3461.psd</t>
+        </is>
+      </c>
+      <c r="B2704" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5521.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2705">
+      <c r="A2705" t="inlineStr">
+        <is>
+          <t>3460.psd</t>
+        </is>
+      </c>
+      <c r="B2705" t="inlineStr">
+        <is>
+          <t>tamilpsd-5522.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2706">
+      <c r="A2706" s="3" t="inlineStr">
+        <is>
+          <t>3459.psd</t>
+        </is>
+      </c>
+      <c r="B2706" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5523.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2707">
+      <c r="A2707" t="inlineStr">
+        <is>
+          <t>3458.psd</t>
+        </is>
+      </c>
+      <c r="B2707" t="inlineStr">
+        <is>
+          <t>tamilpsd-5524.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2708">
+      <c r="A2708" s="3" t="inlineStr">
+        <is>
+          <t>3456.psd</t>
+        </is>
+      </c>
+      <c r="B2708" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5525.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2709">
+      <c r="A2709" t="inlineStr">
+        <is>
+          <t>3454.psd</t>
+        </is>
+      </c>
+      <c r="B2709" t="inlineStr">
+        <is>
+          <t>tamilpsd-5526.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2710">
+      <c r="A2710" s="3" t="inlineStr">
+        <is>
+          <t>3453.psd</t>
+        </is>
+      </c>
+      <c r="B2710" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5527.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2711">
+      <c r="A2711" t="inlineStr">
+        <is>
+          <t>3452.psd</t>
+        </is>
+      </c>
+      <c r="B2711" t="inlineStr">
+        <is>
+          <t>tamilpsd-5528.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2712">
+      <c r="A2712" s="3" t="inlineStr">
+        <is>
+          <t>3451.psd</t>
+        </is>
+      </c>
+      <c r="B2712" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5529.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2713">
+      <c r="A2713" t="inlineStr">
+        <is>
+          <t>3450.psd</t>
+        </is>
+      </c>
+      <c r="B2713" t="inlineStr">
+        <is>
+          <t>tamilpsd-5530.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2714">
+      <c r="A2714" s="3" t="inlineStr">
+        <is>
+          <t>3449.psd</t>
+        </is>
+      </c>
+      <c r="B2714" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5531.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2715">
+      <c r="A2715" t="inlineStr">
+        <is>
+          <t>3447.psd</t>
+        </is>
+      </c>
+      <c r="B2715" t="inlineStr">
+        <is>
+          <t>tamilpsd-5532.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2716">
+      <c r="A2716" s="3" t="inlineStr">
+        <is>
+          <t>3446.psd</t>
+        </is>
+      </c>
+      <c r="B2716" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5533.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2717">
+      <c r="A2717" t="inlineStr">
+        <is>
+          <t>3445.psd</t>
+        </is>
+      </c>
+      <c r="B2717" t="inlineStr">
+        <is>
+          <t>tamilpsd-5534.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2718">
+      <c r="A2718" s="3" t="inlineStr">
+        <is>
+          <t>3443.psd</t>
+        </is>
+      </c>
+      <c r="B2718" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5535.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2719">
+      <c r="A2719" t="inlineStr">
+        <is>
+          <t>3442.psd</t>
+        </is>
+      </c>
+      <c r="B2719" t="inlineStr">
+        <is>
+          <t>tamilpsd-5536.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2720">
+      <c r="A2720" s="3" t="inlineStr">
+        <is>
+          <t>3441.psd</t>
+        </is>
+      </c>
+      <c r="B2720" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5537.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2721">
+      <c r="A2721" t="inlineStr">
+        <is>
+          <t>3440.psd</t>
+        </is>
+      </c>
+      <c r="B2721" t="inlineStr">
+        <is>
+          <t>tamilpsd-5538.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2722">
+      <c r="A2722" s="3" t="inlineStr">
+        <is>
+          <t>3439.psd</t>
+        </is>
+      </c>
+      <c r="B2722" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5539.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2723">
+      <c r="A2723" t="inlineStr">
+        <is>
+          <t>3438.psd</t>
+        </is>
+      </c>
+      <c r="B2723" t="inlineStr">
+        <is>
+          <t>tamilpsd-5540.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2724">
+      <c r="A2724" s="3" t="inlineStr">
+        <is>
+          <t>3437.psd</t>
+        </is>
+      </c>
+      <c r="B2724" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5541.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2725">
+      <c r="A2725" t="inlineStr">
+        <is>
+          <t>3436.psd</t>
+        </is>
+      </c>
+      <c r="B2725" t="inlineStr">
+        <is>
+          <t>tamilpsd-5542.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2726">
+      <c r="A2726" s="3" t="inlineStr">
+        <is>
+          <t>3435.psd</t>
+        </is>
+      </c>
+      <c r="B2726" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5543.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2727">
+      <c r="A2727" t="inlineStr">
+        <is>
+          <t>3434.psd</t>
+        </is>
+      </c>
+      <c r="B2727" t="inlineStr">
+        <is>
+          <t>tamilpsd-5544.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2728">
+      <c r="A2728" s="3" t="inlineStr">
+        <is>
+          <t>3433.psd</t>
+        </is>
+      </c>
+      <c r="B2728" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5545.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2729">
+      <c r="A2729" t="inlineStr">
+        <is>
+          <t>3432.psd</t>
+        </is>
+      </c>
+      <c r="B2729" t="inlineStr">
+        <is>
+          <t>tamilpsd-5546.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2730">
+      <c r="A2730" s="3" t="inlineStr">
+        <is>
+          <t>3431.psd</t>
+        </is>
+      </c>
+      <c r="B2730" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5547.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2731">
+      <c r="A2731" t="inlineStr">
+        <is>
+          <t>3430.psd</t>
+        </is>
+      </c>
+      <c r="B2731" t="inlineStr">
+        <is>
+          <t>tamilpsd-5548.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2732">
+      <c r="A2732" s="3" t="inlineStr">
+        <is>
+          <t>3429.psd</t>
+        </is>
+      </c>
+      <c r="B2732" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5549.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2733">
+      <c r="A2733" t="inlineStr">
+        <is>
+          <t>3428.psd</t>
+        </is>
+      </c>
+      <c r="B2733" t="inlineStr">
+        <is>
+          <t>tamilpsd-5550.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2734">
+      <c r="A2734" s="3" t="inlineStr">
+        <is>
+          <t>3427.psd</t>
+        </is>
+      </c>
+      <c r="B2734" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5551.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2735">
+      <c r="A2735" t="inlineStr">
+        <is>
+          <t>3426.psd</t>
+        </is>
+      </c>
+      <c r="B2735" t="inlineStr">
+        <is>
+          <t>tamilpsd-5552.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2736">
+      <c r="A2736" s="3" t="inlineStr">
+        <is>
+          <t>3425.psd</t>
+        </is>
+      </c>
+      <c r="B2736" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5553.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2737">
+      <c r="A2737" t="inlineStr">
+        <is>
+          <t>3423.psd</t>
+        </is>
+      </c>
+      <c r="B2737" t="inlineStr">
+        <is>
+          <t>tamilpsd-5554.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2738">
+      <c r="A2738" s="3" t="inlineStr">
+        <is>
+          <t>3422.psd</t>
+        </is>
+      </c>
+      <c r="B2738" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5555.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2739">
+      <c r="A2739" t="inlineStr">
+        <is>
+          <t>3421.psd</t>
+        </is>
+      </c>
+      <c r="B2739" t="inlineStr">
+        <is>
+          <t>tamilpsd-5556.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2740">
+      <c r="A2740" s="3" t="inlineStr">
+        <is>
+          <t>3420.psd</t>
+        </is>
+      </c>
+      <c r="B2740" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5557.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2741">
+      <c r="A2741" t="inlineStr">
+        <is>
+          <t>3419.psd</t>
+        </is>
+      </c>
+      <c r="B2741" t="inlineStr">
+        <is>
+          <t>tamilpsd-5558.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2742">
+      <c r="A2742" s="3" t="inlineStr">
+        <is>
+          <t>3418.psd</t>
+        </is>
+      </c>
+      <c r="B2742" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5559.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2743">
+      <c r="A2743" t="inlineStr">
+        <is>
+          <t>3417.psd</t>
+        </is>
+      </c>
+      <c r="B2743" t="inlineStr">
+        <is>
+          <t>tamilpsd-5560.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2744">
+      <c r="A2744" s="3" t="inlineStr">
+        <is>
+          <t>3416.psd</t>
+        </is>
+      </c>
+      <c r="B2744" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5561.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2745">
+      <c r="A2745" t="inlineStr">
+        <is>
+          <t>3415.psd</t>
+        </is>
+      </c>
+      <c r="B2745" t="inlineStr">
+        <is>
+          <t>tamilpsd-5562.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2746">
+      <c r="A2746" s="3" t="inlineStr">
+        <is>
+          <t>3414.psd</t>
+        </is>
+      </c>
+      <c r="B2746" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5563.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2747">
+      <c r="A2747" t="inlineStr">
+        <is>
+          <t>3413.psd</t>
+        </is>
+      </c>
+      <c r="B2747" t="inlineStr">
+        <is>
+          <t>tamilpsd-5564.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2748">
+      <c r="A2748" s="3" t="inlineStr">
+        <is>
+          <t>3412.psd</t>
+        </is>
+      </c>
+      <c r="B2748" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5565.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2749">
+      <c r="A2749" t="inlineStr">
+        <is>
+          <t>3411.psd</t>
+        </is>
+      </c>
+      <c r="B2749" t="inlineStr">
+        <is>
+          <t>tamilpsd-5566.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2750">
+      <c r="A2750" s="3" t="inlineStr">
+        <is>
+          <t>3410.psd</t>
+        </is>
+      </c>
+      <c r="B2750" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5567.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2751">
+      <c r="A2751" t="inlineStr">
+        <is>
+          <t>3409.psd</t>
+        </is>
+      </c>
+      <c r="B2751" t="inlineStr">
+        <is>
+          <t>tamilpsd-5568.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2752">
+      <c r="A2752" s="3" t="inlineStr">
+        <is>
+          <t>3408.psd</t>
+        </is>
+      </c>
+      <c r="B2752" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5569.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2753">
+      <c r="A2753" t="inlineStr">
+        <is>
+          <t>3407.psd</t>
+        </is>
+      </c>
+      <c r="B2753" t="inlineStr">
+        <is>
+          <t>tamilpsd-5570.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2754">
+      <c r="A2754" s="3" t="inlineStr">
+        <is>
+          <t>3405.psd</t>
+        </is>
+      </c>
+      <c r="B2754" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5571.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2755">
+      <c r="A2755" t="inlineStr">
+        <is>
+          <t>3404.psd</t>
+        </is>
+      </c>
+      <c r="B2755" t="inlineStr">
+        <is>
+          <t>tamilpsd-5572.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2756">
+      <c r="A2756" s="3" t="inlineStr">
+        <is>
+          <t>3403.psd</t>
+        </is>
+      </c>
+      <c r="B2756" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5573.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2757">
+      <c r="A2757" t="inlineStr">
+        <is>
+          <t>3402.psd</t>
+        </is>
+      </c>
+      <c r="B2757" t="inlineStr">
+        <is>
+          <t>tamilpsd-5574.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2758">
+      <c r="A2758" s="3" t="inlineStr">
+        <is>
+          <t>3401.psd</t>
+        </is>
+      </c>
+      <c r="B2758" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5575.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2759">
+      <c r="A2759" t="inlineStr">
+        <is>
+          <t>3400.psd</t>
+        </is>
+      </c>
+      <c r="B2759" t="inlineStr">
+        <is>
+          <t>tamilpsd-5576.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2760">
+      <c r="A2760" s="3" t="inlineStr">
+        <is>
+          <t>3399.psd</t>
+        </is>
+      </c>
+      <c r="B2760" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5577.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2761">
+      <c r="A2761" t="inlineStr">
+        <is>
+          <t>3398.psd</t>
+        </is>
+      </c>
+      <c r="B2761" t="inlineStr">
+        <is>
+          <t>tamilpsd-5578.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2762">
+      <c r="A2762" s="3" t="inlineStr">
+        <is>
+          <t>3397.psd</t>
+        </is>
+      </c>
+      <c r="B2762" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5579.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2763">
+      <c r="A2763" t="inlineStr">
+        <is>
+          <t>3945.PSD</t>
+        </is>
+      </c>
+      <c r="B2763" t="inlineStr">
+        <is>
+          <t>tamilpsd-5580.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2764">
+      <c r="A2764" s="3" t="inlineStr">
+        <is>
+          <t>3944.psd</t>
+        </is>
+      </c>
+      <c r="B2764" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5581.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2765">
+      <c r="A2765" t="inlineStr">
+        <is>
+          <t>3943.psd</t>
+        </is>
+      </c>
+      <c r="B2765" t="inlineStr">
+        <is>
+          <t>tamilpsd-5582.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2766">
+      <c r="A2766" s="3" t="inlineStr">
+        <is>
+          <t>3942.psd</t>
+        </is>
+      </c>
+      <c r="B2766" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5583.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2767">
+      <c r="A2767" t="inlineStr">
+        <is>
+          <t>3941.psd</t>
+        </is>
+      </c>
+      <c r="B2767" t="inlineStr">
+        <is>
+          <t>tamilpsd-5584.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2768">
+      <c r="A2768" s="3" t="inlineStr">
+        <is>
+          <t>3940.psd</t>
+        </is>
+      </c>
+      <c r="B2768" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5585.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2769">
+      <c r="A2769" t="inlineStr">
+        <is>
+          <t>3939.psd</t>
+        </is>
+      </c>
+      <c r="B2769" t="inlineStr">
+        <is>
+          <t>tamilpsd-5586.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2770">
+      <c r="A2770" s="3" t="inlineStr">
+        <is>
+          <t>3938.psd</t>
+        </is>
+      </c>
+      <c r="B2770" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5587.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2771">
+      <c r="A2771" t="inlineStr">
+        <is>
+          <t>3937.psd</t>
+        </is>
+      </c>
+      <c r="B2771" t="inlineStr">
+        <is>
+          <t>tamilpsd-5588.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2772">
+      <c r="A2772" s="3" t="inlineStr">
+        <is>
+          <t>3935.psd</t>
+        </is>
+      </c>
+      <c r="B2772" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5589.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2773">
+      <c r="A2773" t="inlineStr">
+        <is>
+          <t>3936.psd</t>
+        </is>
+      </c>
+      <c r="B2773" t="inlineStr">
+        <is>
+          <t>tamilpsd-5590.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2774">
+      <c r="A2774" s="3" t="inlineStr">
+        <is>
+          <t>3934.psd</t>
+        </is>
+      </c>
+      <c r="B2774" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5591.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2775">
+      <c r="A2775" t="inlineStr">
+        <is>
+          <t>3933.psd</t>
+        </is>
+      </c>
+      <c r="B2775" t="inlineStr">
+        <is>
+          <t>tamilpsd-5592.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2776">
+      <c r="A2776" s="3" t="inlineStr">
+        <is>
+          <t>3932.psd</t>
+        </is>
+      </c>
+      <c r="B2776" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5593.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2777">
+      <c r="A2777" t="inlineStr">
+        <is>
+          <t>3931.psd</t>
+        </is>
+      </c>
+      <c r="B2777" t="inlineStr">
+        <is>
+          <t>tamilpsd-5594.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2778">
+      <c r="A2778" s="3" t="inlineStr">
+        <is>
+          <t>3930.psd</t>
+        </is>
+      </c>
+      <c r="B2778" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5595.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2779">
+      <c r="A2779" t="inlineStr">
+        <is>
+          <t>3929.psd</t>
+        </is>
+      </c>
+      <c r="B2779" t="inlineStr">
+        <is>
+          <t>tamilpsd-5596.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2780">
+      <c r="A2780" s="3" t="inlineStr">
+        <is>
+          <t>3928.psd</t>
+        </is>
+      </c>
+      <c r="B2780" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5597.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2781">
+      <c r="A2781" t="inlineStr">
+        <is>
+          <t>3927.psd</t>
+        </is>
+      </c>
+      <c r="B2781" t="inlineStr">
+        <is>
+          <t>tamilpsd-5598.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2782">
+      <c r="A2782" s="3" t="inlineStr">
+        <is>
+          <t>3926.psd</t>
+        </is>
+      </c>
+      <c r="B2782" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5599.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2783">
+      <c r="A2783" t="inlineStr">
+        <is>
+          <t>3925.psd</t>
+        </is>
+      </c>
+      <c r="B2783" t="inlineStr">
+        <is>
+          <t>tamilpsd-5600.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2784">
+      <c r="A2784" s="3" t="inlineStr">
+        <is>
+          <t>3946.PSD</t>
+        </is>
+      </c>
+      <c r="B2784" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5601.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2785">
+      <c r="A2785" t="inlineStr">
+        <is>
+          <t>3923.psd</t>
+        </is>
+      </c>
+      <c r="B2785" t="inlineStr">
+        <is>
+          <t>tamilpsd-5602.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2786">
+      <c r="A2786" s="3" t="inlineStr">
+        <is>
+          <t>3922.psd</t>
+        </is>
+      </c>
+      <c r="B2786" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5603.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2787">
+      <c r="A2787" t="inlineStr">
+        <is>
+          <t>3921.psd</t>
+        </is>
+      </c>
+      <c r="B2787" t="inlineStr">
+        <is>
+          <t>tamilpsd-5604.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2788">
+      <c r="A2788" s="3" t="inlineStr">
+        <is>
+          <t>3920.psd</t>
+        </is>
+      </c>
+      <c r="B2788" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5605.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2789">
+      <c r="A2789" t="inlineStr">
+        <is>
+          <t>3919.psd</t>
+        </is>
+      </c>
+      <c r="B2789" t="inlineStr">
+        <is>
+          <t>tamilpsd-5606.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2790">
+      <c r="A2790" s="3" t="inlineStr">
+        <is>
+          <t>3918.psd</t>
+        </is>
+      </c>
+      <c r="B2790" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5607.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2791">
+      <c r="A2791" t="inlineStr">
+        <is>
+          <t>3917.psd</t>
+        </is>
+      </c>
+      <c r="B2791" t="inlineStr">
+        <is>
+          <t>tamilpsd-5608.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2792">
+      <c r="A2792" s="3" t="inlineStr">
+        <is>
+          <t>3916.psd</t>
+        </is>
+      </c>
+      <c r="B2792" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5609.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2793">
+      <c r="A2793" t="inlineStr">
+        <is>
+          <t>3915.psd</t>
+        </is>
+      </c>
+      <c r="B2793" t="inlineStr">
+        <is>
+          <t>tamilpsd-5610.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2794">
+      <c r="A2794" s="3" t="inlineStr">
+        <is>
+          <t>3914.psd</t>
+        </is>
+      </c>
+      <c r="B2794" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5611.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2795">
+      <c r="A2795" t="inlineStr">
+        <is>
+          <t>3913.psd</t>
+        </is>
+      </c>
+      <c r="B2795" t="inlineStr">
+        <is>
+          <t>tamilpsd-5612.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2796">
+      <c r="A2796" s="3" t="inlineStr">
+        <is>
+          <t>3912.psd</t>
+        </is>
+      </c>
+      <c r="B2796" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5613.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2797">
+      <c r="A2797" t="inlineStr">
+        <is>
+          <t>3911.psd</t>
+        </is>
+      </c>
+      <c r="B2797" t="inlineStr">
+        <is>
+          <t>tamilpsd-5614.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2798">
+      <c r="A2798" s="3" t="inlineStr">
+        <is>
+          <t>3910.psd</t>
+        </is>
+      </c>
+      <c r="B2798" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5615.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2799">
+      <c r="A2799" t="inlineStr">
+        <is>
+          <t>3908.psd</t>
+        </is>
+      </c>
+      <c r="B2799" t="inlineStr">
+        <is>
+          <t>tamilpsd-5616.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2800">
+      <c r="A2800" s="3" t="inlineStr">
+        <is>
+          <t>3907.psd</t>
+        </is>
+      </c>
+      <c r="B2800" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5617.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2801">
+      <c r="A2801" t="inlineStr">
+        <is>
+          <t>3906.psd</t>
+        </is>
+      </c>
+      <c r="B2801" t="inlineStr">
+        <is>
+          <t>tamilpsd-5618.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2802">
+      <c r="A2802" s="3" t="inlineStr">
+        <is>
+          <t>3905.psd</t>
+        </is>
+      </c>
+      <c r="B2802" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5619.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2803">
+      <c r="A2803" t="inlineStr">
+        <is>
+          <t>3924.psd</t>
+        </is>
+      </c>
+      <c r="B2803" t="inlineStr">
+        <is>
+          <t>tamilpsd-5620.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2804">
+      <c r="A2804" s="3" t="inlineStr">
+        <is>
+          <t>49.psd</t>
+        </is>
+      </c>
+      <c r="B2804" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5621.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2805">
+      <c r="A2805" t="inlineStr">
+        <is>
+          <t>50.psd</t>
+        </is>
+      </c>
+      <c r="B2805" t="inlineStr">
+        <is>
+          <t>tamilpsd-5622.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2806">
+      <c r="A2806" s="3" t="inlineStr">
+        <is>
+          <t>34.psd</t>
+        </is>
+      </c>
+      <c r="B2806" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5623.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2807">
+      <c r="A2807" t="inlineStr">
+        <is>
+          <t>44.psd</t>
+        </is>
+      </c>
+      <c r="B2807" t="inlineStr">
+        <is>
+          <t>tamilpsd-5624.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2808">
+      <c r="A2808" s="3" t="inlineStr">
+        <is>
+          <t>43.psd</t>
+        </is>
+      </c>
+      <c r="B2808" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5625.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2809">
+      <c r="A2809" t="inlineStr">
+        <is>
+          <t>57.psd</t>
+        </is>
+      </c>
+      <c r="B2809" t="inlineStr">
+        <is>
+          <t>tamilpsd-5626.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2810">
+      <c r="A2810" s="3" t="inlineStr">
+        <is>
+          <t>58.psd</t>
+        </is>
+      </c>
+      <c r="B2810" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5627.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2811">
+      <c r="A2811" t="inlineStr">
+        <is>
+          <t>62.psd</t>
+        </is>
+      </c>
+      <c r="B2811" t="inlineStr">
+        <is>
+          <t>tamilpsd-5628.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2812">
+      <c r="A2812" s="3" t="inlineStr">
+        <is>
+          <t>67.psd</t>
+        </is>
+      </c>
+      <c r="B2812" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5629.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2813">
+      <c r="A2813" t="inlineStr">
+        <is>
+          <t>64.psd</t>
+        </is>
+      </c>
+      <c r="B2813" t="inlineStr">
+        <is>
+          <t>tamilpsd-5630.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2814">
+      <c r="A2814" s="3" t="inlineStr">
+        <is>
+          <t>65.psd</t>
+        </is>
+      </c>
+      <c r="B2814" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5631.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2815">
+      <c r="A2815" t="inlineStr">
+        <is>
+          <t>66.psd</t>
+        </is>
+      </c>
+      <c r="B2815" t="inlineStr">
+        <is>
+          <t>tamilpsd-5632.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2816">
+      <c r="A2816" s="3" t="inlineStr">
+        <is>
+          <t>73.psd</t>
+        </is>
+      </c>
+      <c r="B2816" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5633.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2817">
+      <c r="A2817" t="inlineStr">
+        <is>
+          <t>72.psd</t>
+        </is>
+      </c>
+      <c r="B2817" t="inlineStr">
+        <is>
+          <t>tamilpsd-5634.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2818">
+      <c r="A2818" s="3" t="inlineStr">
+        <is>
+          <t>74.psd</t>
+        </is>
+      </c>
+      <c r="B2818" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5635.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2819">
+      <c r="A2819" t="inlineStr">
+        <is>
+          <t>80.psd</t>
+        </is>
+      </c>
+      <c r="B2819" t="inlineStr">
+        <is>
+          <t>tamilpsd-5636.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2820">
+      <c r="A2820" s="3" t="inlineStr">
+        <is>
+          <t>70.psd</t>
+        </is>
+      </c>
+      <c r="B2820" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5637.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2821">
+      <c r="A2821" t="inlineStr">
+        <is>
+          <t>71.psd</t>
+        </is>
+      </c>
+      <c r="B2821" t="inlineStr">
+        <is>
+          <t>tamilpsd-5638.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2822">
+      <c r="A2822" s="3" t="inlineStr">
+        <is>
+          <t>56.psd</t>
+        </is>
+      </c>
+      <c r="B2822" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5639.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2823">
+      <c r="A2823" t="inlineStr">
+        <is>
+          <t>31.psd</t>
+        </is>
+      </c>
+      <c r="B2823" t="inlineStr">
+        <is>
+          <t>tamilpsd-5640.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2824">
+      <c r="A2824" s="3" t="inlineStr">
+        <is>
+          <t>16.psd</t>
+        </is>
+      </c>
+      <c r="B2824" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5642.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2825">
+      <c r="A2825" t="inlineStr">
+        <is>
+          <t>19.psd</t>
+        </is>
+      </c>
+      <c r="B2825" t="inlineStr">
+        <is>
+          <t>tamilpsd-5643.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2826">
+      <c r="A2826" s="3" t="inlineStr">
+        <is>
+          <t>21.psd</t>
+        </is>
+      </c>
+      <c r="B2826" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5644.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2827">
+      <c r="A2827" t="inlineStr">
+        <is>
+          <t>15.psd</t>
+        </is>
+      </c>
+      <c r="B2827" t="inlineStr">
+        <is>
+          <t>tamilpsd-5646.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2828">
+      <c r="A2828" s="3" t="inlineStr">
+        <is>
+          <t>00.psd</t>
+        </is>
+      </c>
+      <c r="B2828" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5647.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2829">
+      <c r="A2829" t="inlineStr">
+        <is>
+          <t>00a.psd</t>
+        </is>
+      </c>
+      <c r="B2829" t="inlineStr">
+        <is>
+          <t>tamilpsd-5648.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2830">
+      <c r="A2830" s="3" t="inlineStr">
+        <is>
+          <t>3877.psd</t>
+        </is>
+      </c>
+      <c r="B2830" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5649.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2831">
+      <c r="A2831" t="inlineStr">
+        <is>
+          <t>3876.psd</t>
+        </is>
+      </c>
+      <c r="B2831" t="inlineStr">
+        <is>
+          <t>tamilpsd-5650.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2832">
+      <c r="A2832" s="3" t="inlineStr">
+        <is>
+          <t>3875.psd</t>
+        </is>
+      </c>
+      <c r="B2832" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5651.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2833">
+      <c r="A2833" t="inlineStr">
+        <is>
+          <t>3874.psd</t>
+        </is>
+      </c>
+      <c r="B2833" t="inlineStr">
+        <is>
+          <t>tamilpsd-5652.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2834">
+      <c r="A2834" s="3" t="inlineStr">
+        <is>
+          <t>3873.psd</t>
+        </is>
+      </c>
+      <c r="B2834" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5653.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2835">
+      <c r="A2835" t="inlineStr">
+        <is>
+          <t>3872.psd</t>
+        </is>
+      </c>
+      <c r="B2835" t="inlineStr">
+        <is>
+          <t>tamilpsd-5654.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2836">
+      <c r="A2836" s="3" t="inlineStr">
+        <is>
+          <t>3871.psd</t>
+        </is>
+      </c>
+      <c r="B2836" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5655.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2837">
+      <c r="A2837" t="inlineStr">
+        <is>
+          <t>3870.psd</t>
+        </is>
+      </c>
+      <c r="B2837" t="inlineStr">
+        <is>
+          <t>tamilpsd-5656.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2838">
+      <c r="A2838" s="3" t="inlineStr">
+        <is>
+          <t>3869.psd</t>
+        </is>
+      </c>
+      <c r="B2838" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5657.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2839">
+      <c r="A2839" t="inlineStr">
+        <is>
+          <t>3868.psd</t>
+        </is>
+      </c>
+      <c r="B2839" t="inlineStr">
+        <is>
+          <t>tamilpsd-5658.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2840">
+      <c r="A2840" s="3" t="inlineStr">
+        <is>
+          <t>3867.psd</t>
+        </is>
+      </c>
+      <c r="B2840" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5659.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2841">
+      <c r="A2841" t="inlineStr">
+        <is>
+          <t>3866.psd</t>
+        </is>
+      </c>
+      <c r="B2841" t="inlineStr">
+        <is>
+          <t>tamilpsd-5660.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2842">
+      <c r="A2842" s="3" t="inlineStr">
+        <is>
+          <t>3865.psd</t>
+        </is>
+      </c>
+      <c r="B2842" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5661.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2843">
+      <c r="A2843" t="inlineStr">
+        <is>
+          <t>3864.psd</t>
+        </is>
+      </c>
+      <c r="B2843" t="inlineStr">
+        <is>
+          <t>tamilpsd-5662.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2844">
+      <c r="A2844" s="3" t="inlineStr">
+        <is>
+          <t>3863.psd</t>
+        </is>
+      </c>
+      <c r="B2844" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5663.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2845">
+      <c r="A2845" t="inlineStr">
+        <is>
+          <t>3862.psd</t>
+        </is>
+      </c>
+      <c r="B2845" t="inlineStr">
+        <is>
+          <t>tamilpsd-5664.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2846">
+      <c r="A2846" s="3" t="inlineStr">
+        <is>
+          <t>3861.psd</t>
+        </is>
+      </c>
+      <c r="B2846" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5665.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2847">
+      <c r="A2847" t="inlineStr">
+        <is>
+          <t>3860.psd</t>
+        </is>
+      </c>
+      <c r="B2847" t="inlineStr">
+        <is>
+          <t>tamilpsd-5666.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2848">
+      <c r="A2848" s="3" t="inlineStr">
+        <is>
+          <t>3859.psd</t>
+        </is>
+      </c>
+      <c r="B2848" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5667.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2849">
+      <c r="A2849" t="inlineStr">
+        <is>
+          <t>3878.psd</t>
+        </is>
+      </c>
+      <c r="B2849" t="inlineStr">
+        <is>
+          <t>tamilpsd-5668.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2850">
+      <c r="A2850" s="3" t="inlineStr">
+        <is>
+          <t>3857.psd</t>
+        </is>
+      </c>
+      <c r="B2850" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5669.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2851">
+      <c r="A2851" t="inlineStr">
+        <is>
+          <t>3856.psd</t>
+        </is>
+      </c>
+      <c r="B2851" t="inlineStr">
+        <is>
+          <t>tamilpsd-5670.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2852">
+      <c r="A2852" s="3" t="inlineStr">
+        <is>
+          <t>3855.psd</t>
+        </is>
+      </c>
+      <c r="B2852" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5671.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2853">
+      <c r="A2853" t="inlineStr">
+        <is>
+          <t>3854.psd</t>
+        </is>
+      </c>
+      <c r="B2853" t="inlineStr">
+        <is>
+          <t>tamilpsd-5672.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2854">
+      <c r="A2854" s="3" t="inlineStr">
+        <is>
+          <t>3853.psd</t>
+        </is>
+      </c>
+      <c r="B2854" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5673.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2855">
+      <c r="A2855" t="inlineStr">
+        <is>
+          <t>3852.psd</t>
+        </is>
+      </c>
+      <c r="B2855" t="inlineStr">
+        <is>
+          <t>tamilpsd-5674.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2856">
+      <c r="A2856" s="3" t="inlineStr">
+        <is>
+          <t>3851.psd</t>
+        </is>
+      </c>
+      <c r="B2856" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5675.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2857">
+      <c r="A2857" t="inlineStr">
+        <is>
+          <t>3850.psd</t>
+        </is>
+      </c>
+      <c r="B2857" t="inlineStr">
+        <is>
+          <t>tamilpsd-5676.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2858">
+      <c r="A2858" s="3" t="inlineStr">
+        <is>
+          <t>3849.psd</t>
+        </is>
+      </c>
+      <c r="B2858" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5677.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2859">
+      <c r="A2859" t="inlineStr">
+        <is>
+          <t>3848.psd</t>
+        </is>
+      </c>
+      <c r="B2859" t="inlineStr">
+        <is>
+          <t>tamilpsd-5678.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2860">
+      <c r="A2860" s="3" t="inlineStr">
+        <is>
+          <t>3847.psd</t>
+        </is>
+      </c>
+      <c r="B2860" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5679.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2861">
+      <c r="A2861" t="inlineStr">
+        <is>
+          <t>3846.psd</t>
+        </is>
+      </c>
+      <c r="B2861" t="inlineStr">
+        <is>
+          <t>tamilpsd-5680.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2862">
+      <c r="A2862" s="3" t="inlineStr">
+        <is>
+          <t>3845.psd</t>
+        </is>
+      </c>
+      <c r="B2862" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5681.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2863">
+      <c r="A2863" t="inlineStr">
+        <is>
+          <t>3844.psd</t>
+        </is>
+      </c>
+      <c r="B2863" t="inlineStr">
+        <is>
+          <t>tamilpsd-5682.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2864">
+      <c r="A2864" s="3" t="inlineStr">
+        <is>
+          <t>3843.psd</t>
+        </is>
+      </c>
+      <c r="B2864" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5683.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2865">
+      <c r="A2865" t="inlineStr">
+        <is>
+          <t>3842.psd</t>
+        </is>
+      </c>
+      <c r="B2865" t="inlineStr">
+        <is>
+          <t>tamilpsd-5684.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2866">
+      <c r="A2866" s="3" t="inlineStr">
+        <is>
+          <t>3841.psd</t>
+        </is>
+      </c>
+      <c r="B2866" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5685.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2867">
+      <c r="A2867" t="inlineStr">
+        <is>
+          <t>3840.psd</t>
+        </is>
+      </c>
+      <c r="B2867" t="inlineStr">
+        <is>
+          <t>tamilpsd-5686.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2868">
+      <c r="A2868" s="3" t="inlineStr">
+        <is>
+          <t>3839.psd</t>
+        </is>
+      </c>
+      <c r="B2868" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5687.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2869">
+      <c r="A2869" t="inlineStr">
+        <is>
+          <t>3838.psd</t>
+        </is>
+      </c>
+      <c r="B2869" t="inlineStr">
+        <is>
+          <t>tamilpsd-5688.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2870">
+      <c r="A2870" s="3" t="inlineStr">
+        <is>
+          <t>3837.psd</t>
+        </is>
+      </c>
+      <c r="B2870" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5689.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2871">
+      <c r="A2871" t="inlineStr">
+        <is>
+          <t>3836.psd</t>
+        </is>
+      </c>
+      <c r="B2871" t="inlineStr">
+        <is>
+          <t>tamilpsd-5690.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2872">
+      <c r="A2872" s="3" t="inlineStr">
+        <is>
+          <t>3835.psd</t>
+        </is>
+      </c>
+      <c r="B2872" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5691.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2873">
+      <c r="A2873" t="inlineStr">
+        <is>
+          <t>3834.psd</t>
+        </is>
+      </c>
+      <c r="B2873" t="inlineStr">
+        <is>
+          <t>tamilpsd-5692.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2874">
+      <c r="A2874" s="3" t="inlineStr">
+        <is>
+          <t>3833.psd</t>
+        </is>
+      </c>
+      <c r="B2874" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5693.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2875">
+      <c r="A2875" t="inlineStr">
+        <is>
+          <t>3832.psd</t>
+        </is>
+      </c>
+      <c r="B2875" t="inlineStr">
+        <is>
+          <t>tamilpsd-5694.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2876">
+      <c r="A2876" s="3" t="inlineStr">
+        <is>
+          <t>3831.psd</t>
+        </is>
+      </c>
+      <c r="B2876" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5695.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2877">
+      <c r="A2877" t="inlineStr">
+        <is>
+          <t>3858.psd</t>
+        </is>
+      </c>
+      <c r="B2877" t="inlineStr">
+        <is>
+          <t>tamilpsd-5696.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2878">
+      <c r="A2878" s="3" t="inlineStr">
+        <is>
+          <t>28.psd</t>
+        </is>
+      </c>
+      <c r="B2878" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5697.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2879">
+      <c r="A2879" t="inlineStr">
+        <is>
+          <t>29.psd</t>
+        </is>
+      </c>
+      <c r="B2879" t="inlineStr">
+        <is>
+          <t>tamilpsd-5698.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2880">
+      <c r="A2880" s="3" t="inlineStr">
+        <is>
+          <t>30.psd</t>
+        </is>
+      </c>
+      <c r="B2880" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5699.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2881">
+      <c r="A2881" t="inlineStr">
+        <is>
+          <t>48.psd</t>
+        </is>
+      </c>
+      <c r="B2881" t="inlineStr">
+        <is>
+          <t>tamilpsd-5700.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2882">
+      <c r="A2882" s="3" t="inlineStr">
+        <is>
+          <t>32.psd</t>
+        </is>
+      </c>
+      <c r="B2882" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5705.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2883">
+      <c r="A2883" t="inlineStr">
+        <is>
+          <t>12.psd</t>
+        </is>
+      </c>
+      <c r="B2883" t="inlineStr">
+        <is>
+          <t>tamilpsd-5706.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2884">
+      <c r="A2884" s="3" t="inlineStr">
+        <is>
+          <t>13.psd</t>
+        </is>
+      </c>
+      <c r="B2884" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5707.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2885">
+      <c r="A2885" t="inlineStr">
+        <is>
+          <t>59.psd</t>
+        </is>
+      </c>
+      <c r="B2885" t="inlineStr">
+        <is>
+          <t>tamilpsd-5708.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2886">
+      <c r="A2886" s="3" t="inlineStr">
+        <is>
+          <t>60.psd</t>
+        </is>
+      </c>
+      <c r="B2886" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5709.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2887">
+      <c r="A2887" t="inlineStr">
+        <is>
+          <t>61.psd</t>
+        </is>
+      </c>
+      <c r="B2887" t="inlineStr">
+        <is>
+          <t>tamilpsd-5710.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2888">
+      <c r="A2888" s="3" t="inlineStr">
+        <is>
+          <t>25.psd</t>
+        </is>
+      </c>
+      <c r="B2888" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5711.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2889">
+      <c r="A2889" t="inlineStr">
+        <is>
+          <t>26.psd</t>
+        </is>
+      </c>
+      <c r="B2889" t="inlineStr">
+        <is>
+          <t>tamilpsd-5712.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2890">
+      <c r="A2890" s="3" t="inlineStr">
+        <is>
+          <t>27.psd</t>
+        </is>
+      </c>
+      <c r="B2890" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5713.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2891">
+      <c r="A2891" t="inlineStr">
+        <is>
+          <t>51.psd</t>
+        </is>
+      </c>
+      <c r="B2891" t="inlineStr">
+        <is>
+          <t>tamilpsd-5714.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2892">
+      <c r="A2892" s="3" t="inlineStr">
+        <is>
+          <t>52.psd</t>
+        </is>
+      </c>
+      <c r="B2892" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5715.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2893">
+      <c r="A2893" t="inlineStr">
+        <is>
+          <t>53.psd</t>
+        </is>
+      </c>
+      <c r="B2893" t="inlineStr">
+        <is>
+          <t>tamilpsd-5716.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2894">
+      <c r="A2894" s="3" t="inlineStr">
+        <is>
+          <t>46.psd</t>
+        </is>
+      </c>
+      <c r="B2894" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5717.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2895">
+      <c r="A2895" t="inlineStr">
+        <is>
+          <t>47.psd</t>
+        </is>
+      </c>
+      <c r="B2895" t="inlineStr">
+        <is>
+          <t>tamilpsd-5718.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2896">
+      <c r="A2896" s="3" t="inlineStr">
+        <is>
+          <t>45.psd</t>
+        </is>
+      </c>
+      <c r="B2896" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5721.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2897">
+      <c r="A2897" t="inlineStr">
+        <is>
+          <t>39.psd</t>
+        </is>
+      </c>
+      <c r="B2897" t="inlineStr">
+        <is>
+          <t>tamilpsd-5722.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2898">
+      <c r="A2898" s="3" t="inlineStr">
+        <is>
+          <t>40.psd</t>
+        </is>
+      </c>
+      <c r="B2898" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5723.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2899">
+      <c r="A2899" t="inlineStr">
+        <is>
+          <t>41.psd</t>
+        </is>
+      </c>
+      <c r="B2899" t="inlineStr">
+        <is>
+          <t>tamilpsd-5724.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2900">
+      <c r="A2900" s="3" t="inlineStr">
+        <is>
+          <t>42.psd</t>
+        </is>
+      </c>
+      <c r="B2900" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5725.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2901">
+      <c r="A2901" t="inlineStr">
+        <is>
+          <t>33.psd</t>
+        </is>
+      </c>
+      <c r="B2901" t="inlineStr">
+        <is>
+          <t>tamilpsd-5726.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2902">
+      <c r="A2902" s="3" t="inlineStr">
+        <is>
+          <t>35.psd</t>
+        </is>
+      </c>
+      <c r="B2902" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5728.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2903">
+      <c r="A2903" t="inlineStr">
+        <is>
+          <t>36.psd</t>
+        </is>
+      </c>
+      <c r="B2903" t="inlineStr">
+        <is>
+          <t>tamilpsd-5729.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2904">
+      <c r="A2904" s="3" t="inlineStr">
+        <is>
+          <t>37.psd</t>
+        </is>
+      </c>
+      <c r="B2904" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5730.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2905">
+      <c r="A2905" t="inlineStr">
+        <is>
+          <t>38.psd</t>
+        </is>
+      </c>
+      <c r="B2905" t="inlineStr">
+        <is>
+          <t>tamilpsd-5731.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2906">
+      <c r="A2906" s="3" t="inlineStr">
+        <is>
+          <t>17.psd</t>
+        </is>
+      </c>
+      <c r="B2906" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5733.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2907">
+      <c r="A2907" t="inlineStr">
+        <is>
+          <t>18.psd</t>
+        </is>
+      </c>
+      <c r="B2907" t="inlineStr">
+        <is>
+          <t>tamilpsd-5734.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2908">
+      <c r="A2908" s="3" t="inlineStr">
+        <is>
+          <t>20.psd</t>
+        </is>
+      </c>
+      <c r="B2908" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5736.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2909">
+      <c r="A2909" t="inlineStr">
+        <is>
+          <t>22.psd</t>
+        </is>
+      </c>
+      <c r="B2909" t="inlineStr">
+        <is>
+          <t>tamilpsd-5738.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2910">
+      <c r="A2910" s="3" t="inlineStr">
+        <is>
+          <t>23.psd</t>
+        </is>
+      </c>
+      <c r="B2910" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5739.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2911">
+      <c r="A2911" t="inlineStr">
+        <is>
+          <t>3811.psd</t>
+        </is>
+      </c>
+      <c r="B2911" t="inlineStr">
+        <is>
+          <t>tamilpsd-5740.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2912">
+      <c r="A2912" s="3" t="inlineStr">
+        <is>
+          <t>3810.psd</t>
+        </is>
+      </c>
+      <c r="B2912" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5741.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2913">
+      <c r="A2913" t="inlineStr">
+        <is>
+          <t>3809.psd</t>
+        </is>
+      </c>
+      <c r="B2913" t="inlineStr">
+        <is>
+          <t>tamilpsd-5742.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2914">
+      <c r="A2914" s="3" t="inlineStr">
+        <is>
+          <t>3808.psd</t>
+        </is>
+      </c>
+      <c r="B2914" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5743.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2915">
+      <c r="A2915" t="inlineStr">
+        <is>
+          <t>3807.psd</t>
+        </is>
+      </c>
+      <c r="B2915" t="inlineStr">
+        <is>
+          <t>tamilpsd-5744.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2916">
+      <c r="A2916" s="3" t="inlineStr">
+        <is>
+          <t>3806.psd</t>
+        </is>
+      </c>
+      <c r="B2916" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5745.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2917">
+      <c r="A2917" t="inlineStr">
+        <is>
+          <t>3805.psd</t>
+        </is>
+      </c>
+      <c r="B2917" t="inlineStr">
+        <is>
+          <t>tamilpsd-5746.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2918">
+      <c r="A2918" s="3" t="inlineStr">
+        <is>
+          <t>3804.psd</t>
+        </is>
+      </c>
+      <c r="B2918" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5747.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2919">
+      <c r="A2919" t="inlineStr">
+        <is>
+          <t>3803.psd</t>
+        </is>
+      </c>
+      <c r="B2919" t="inlineStr">
+        <is>
+          <t>tamilpsd-5748.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2920">
+      <c r="A2920" s="3" t="inlineStr">
+        <is>
+          <t>3802.psd</t>
+        </is>
+      </c>
+      <c r="B2920" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5749.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2921">
+      <c r="A2921" t="inlineStr">
+        <is>
+          <t>3801.psd</t>
+        </is>
+      </c>
+      <c r="B2921" t="inlineStr">
+        <is>
+          <t>tamilpsd-5750.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2922">
+      <c r="A2922" s="3" t="inlineStr">
+        <is>
+          <t>3800.psd</t>
+        </is>
+      </c>
+      <c r="B2922" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5751.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2923">
+      <c r="A2923" t="inlineStr">
+        <is>
+          <t>3799.psd</t>
+        </is>
+      </c>
+      <c r="B2923" t="inlineStr">
+        <is>
+          <t>tamilpsd-5752.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2924">
+      <c r="A2924" s="3" t="inlineStr">
+        <is>
+          <t>3798.psd</t>
+        </is>
+      </c>
+      <c r="B2924" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5753.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2925">
+      <c r="A2925" t="inlineStr">
+        <is>
+          <t>3797.psd</t>
+        </is>
+      </c>
+      <c r="B2925" t="inlineStr">
+        <is>
+          <t>tamilpsd-5754.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2926">
+      <c r="A2926" s="3" t="inlineStr">
+        <is>
+          <t>3796.psd</t>
+        </is>
+      </c>
+      <c r="B2926" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5755.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2927">
+      <c r="A2927" t="inlineStr">
+        <is>
+          <t>3795.psd</t>
+        </is>
+      </c>
+      <c r="B2927" t="inlineStr">
+        <is>
+          <t>tamilpsd-5756.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2928">
+      <c r="A2928" s="3" t="inlineStr">
+        <is>
+          <t>3794.psd</t>
+        </is>
+      </c>
+      <c r="B2928" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5757.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2929">
+      <c r="A2929" t="inlineStr">
+        <is>
+          <t>3793.psd</t>
+        </is>
+      </c>
+      <c r="B2929" t="inlineStr">
+        <is>
+          <t>tamilpsd-5758.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2930">
+      <c r="A2930" s="3" t="inlineStr">
+        <is>
+          <t>3792.psd</t>
+        </is>
+      </c>
+      <c r="B2930" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5759.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2931">
+      <c r="A2931" t="inlineStr">
+        <is>
+          <t>3791.psd</t>
+        </is>
+      </c>
+      <c r="B2931" t="inlineStr">
+        <is>
+          <t>tamilpsd-5760.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2932">
+      <c r="A2932" s="3" t="inlineStr">
+        <is>
+          <t>3790.psd</t>
+        </is>
+      </c>
+      <c r="B2932" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5761.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2933">
+      <c r="A2933" t="inlineStr">
+        <is>
+          <t>3789.psd</t>
+        </is>
+      </c>
+      <c r="B2933" t="inlineStr">
+        <is>
+          <t>tamilpsd-5762.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2934">
+      <c r="A2934" s="3" t="inlineStr">
+        <is>
+          <t>3788.psd</t>
+        </is>
+      </c>
+      <c r="B2934" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5763.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2935">
+      <c r="A2935" t="inlineStr">
+        <is>
+          <t>3787.psd</t>
+        </is>
+      </c>
+      <c r="B2935" t="inlineStr">
+        <is>
+          <t>tamilpsd-5764.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2936">
+      <c r="A2936" s="3" t="inlineStr">
+        <is>
+          <t>3786.psd</t>
+        </is>
+      </c>
+      <c r="B2936" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5765.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2937">
+      <c r="A2937" t="inlineStr">
+        <is>
+          <t>3785.psd</t>
+        </is>
+      </c>
+      <c r="B2937" t="inlineStr">
+        <is>
+          <t>tamilpsd-5766.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2938">
+      <c r="A2938" s="3" t="inlineStr">
+        <is>
+          <t>3784.psd</t>
+        </is>
+      </c>
+      <c r="B2938" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5767.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2939">
+      <c r="A2939" t="inlineStr">
+        <is>
+          <t>3783.psd</t>
+        </is>
+      </c>
+      <c r="B2939" t="inlineStr">
+        <is>
+          <t>tamilpsd-5768.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2940">
+      <c r="A2940" s="3" t="inlineStr">
+        <is>
+          <t>3781.psd</t>
+        </is>
+      </c>
+      <c r="B2940" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5769.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2941">
+      <c r="A2941" t="inlineStr">
+        <is>
+          <t>3782.psd</t>
+        </is>
+      </c>
+      <c r="B2941" t="inlineStr">
+        <is>
+          <t>tamilpsd-5770.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2942">
+      <c r="A2942" s="3" t="inlineStr">
+        <is>
+          <t>3780.psd</t>
+        </is>
+      </c>
+      <c r="B2942" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5771.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2943">
+      <c r="A2943" t="inlineStr">
+        <is>
+          <t>3779.psd</t>
+        </is>
+      </c>
+      <c r="B2943" t="inlineStr">
+        <is>
+          <t>tamilpsd-5772.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2944">
+      <c r="A2944" s="3" t="inlineStr">
+        <is>
+          <t>3778.psd</t>
+        </is>
+      </c>
+      <c r="B2944" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5773.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2945">
+      <c r="A2945" t="inlineStr">
+        <is>
+          <t>3776.psd</t>
+        </is>
+      </c>
+      <c r="B2945" t="inlineStr">
+        <is>
+          <t>tamilpsd-5774.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2946">
+      <c r="A2946" s="3" t="inlineStr">
+        <is>
+          <t>3777.psd</t>
+        </is>
+      </c>
+      <c r="B2946" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5775.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2947">
+      <c r="A2947" t="inlineStr">
+        <is>
+          <t>3775.psd</t>
+        </is>
+      </c>
+      <c r="B2947" t="inlineStr">
+        <is>
+          <t>tamilpsd-5776.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2948">
+      <c r="A2948" s="3" t="inlineStr">
+        <is>
+          <t>3774.psd</t>
+        </is>
+      </c>
+      <c r="B2948" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5777.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2949">
+      <c r="A2949" t="inlineStr">
+        <is>
+          <t>3773.psd</t>
+        </is>
+      </c>
+      <c r="B2949" t="inlineStr">
+        <is>
+          <t>tamilpsd-5778.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2950">
+      <c r="A2950" s="3" t="inlineStr">
+        <is>
+          <t>3772.psd</t>
+        </is>
+      </c>
+      <c r="B2950" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5779.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2951">
+      <c r="A2951" t="inlineStr">
+        <is>
+          <t>3771.psd</t>
+        </is>
+      </c>
+      <c r="B2951" t="inlineStr">
+        <is>
+          <t>tamilpsd-5780.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2952">
+      <c r="A2952" s="3" t="inlineStr">
+        <is>
+          <t>3770.psd</t>
+        </is>
+      </c>
+      <c r="B2952" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5781.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2953">
+      <c r="A2953" t="inlineStr">
+        <is>
+          <t>3769.psd</t>
+        </is>
+      </c>
+      <c r="B2953" t="inlineStr">
+        <is>
+          <t>tamilpsd-5782.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2954">
+      <c r="A2954" s="3" t="inlineStr">
+        <is>
+          <t>3768.psd</t>
+        </is>
+      </c>
+      <c r="B2954" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5783.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2955">
+      <c r="A2955" t="inlineStr">
+        <is>
+          <t>3767.psd</t>
+        </is>
+      </c>
+      <c r="B2955" t="inlineStr">
+        <is>
+          <t>tamilpsd-5784.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2956">
+      <c r="A2956" s="3" t="inlineStr">
+        <is>
+          <t>3766.psd</t>
+        </is>
+      </c>
+      <c r="B2956" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5785.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2957">
+      <c r="A2957" t="inlineStr">
+        <is>
+          <t>3765.psd</t>
+        </is>
+      </c>
+      <c r="B2957" t="inlineStr">
+        <is>
+          <t>tamilpsd-5786.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2958">
+      <c r="A2958" s="3" t="inlineStr">
+        <is>
+          <t>3764.psd</t>
+        </is>
+      </c>
+      <c r="B2958" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5787.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2959">
+      <c r="A2959" t="inlineStr">
+        <is>
+          <t>3763.psd</t>
+        </is>
+      </c>
+      <c r="B2959" t="inlineStr">
+        <is>
+          <t>tamilpsd-5788.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2960">
+      <c r="A2960" s="3" t="inlineStr">
+        <is>
+          <t>3762.psd</t>
+        </is>
+      </c>
+      <c r="B2960" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-5789.psd</t>
+        </is>
+      </c>
+    </row>
+    <row r="2961">
+      <c r="A2961" t="inlineStr">
+        <is>
+          <t>3761.psd</t>
+        </is>
+      </c>
+      <c r="B2961" t="inlineStr">
+        <is>
+          <t>tamilpsd-5790.psd</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
🤖 Progress: 2026-04-21 06:18 UTC
</commit_message>
<xml_diff>
--- a/rename_log.xlsx
+++ b/rename_log.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4258"/>
+  <dimension ref="A1:B4259"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -51193,6 +51193,18 @@
         </is>
       </c>
     </row>
+    <row r="4259">
+      <c r="A4259" t="inlineStr">
+        <is>
+          <t>3246.psd</t>
+        </is>
+      </c>
+      <c r="B4259" t="inlineStr">
+        <is>
+          <t>tamilpsd-7754.psd</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
🤖 Progress: 2026-04-21 07:34 UTC
</commit_message>
<xml_diff>
--- a/rename_log.xlsx
+++ b/rename_log.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4259"/>
+  <dimension ref="A1:B4269"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -51205,6 +51205,126 @@
         </is>
       </c>
     </row>
+    <row r="4260">
+      <c r="A4260" s="3" t="inlineStr">
+        <is>
+          <t>6152.png</t>
+        </is>
+      </c>
+      <c r="B4260" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-7756.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="4261">
+      <c r="A4261" t="inlineStr">
+        <is>
+          <t>6151.png</t>
+        </is>
+      </c>
+      <c r="B4261" t="inlineStr">
+        <is>
+          <t>tamilpsd-7757.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="4262">
+      <c r="A4262" s="3" t="inlineStr">
+        <is>
+          <t>6150.png</t>
+        </is>
+      </c>
+      <c r="B4262" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-7758.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="4263">
+      <c r="A4263" t="inlineStr">
+        <is>
+          <t>6149.png</t>
+        </is>
+      </c>
+      <c r="B4263" t="inlineStr">
+        <is>
+          <t>tamilpsd-7759.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="4264">
+      <c r="A4264" s="3" t="inlineStr">
+        <is>
+          <t>6148.png</t>
+        </is>
+      </c>
+      <c r="B4264" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-7760.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="4265">
+      <c r="A4265" t="inlineStr">
+        <is>
+          <t>6147.png</t>
+        </is>
+      </c>
+      <c r="B4265" t="inlineStr">
+        <is>
+          <t>tamilpsd-7761.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="4266">
+      <c r="A4266" s="3" t="inlineStr">
+        <is>
+          <t>6146.png</t>
+        </is>
+      </c>
+      <c r="B4266" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-7762.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="4267">
+      <c r="A4267" t="inlineStr">
+        <is>
+          <t>6145.png</t>
+        </is>
+      </c>
+      <c r="B4267" t="inlineStr">
+        <is>
+          <t>tamilpsd-7763.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="4268">
+      <c r="A4268" s="3" t="inlineStr">
+        <is>
+          <t>6144.png</t>
+        </is>
+      </c>
+      <c r="B4268" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-7764.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="4269">
+      <c r="A4269" t="inlineStr">
+        <is>
+          <t>6143.png</t>
+        </is>
+      </c>
+      <c r="B4269" t="inlineStr">
+        <is>
+          <t>tamilpsd-7765.png</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
🤖 Progress: 2026-04-26 08:59 UTC
</commit_message>
<xml_diff>
--- a/rename_log.xlsx
+++ b/rename_log.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4738"/>
+  <dimension ref="A1:B4746"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -56953,6 +56953,102 @@
         </is>
       </c>
     </row>
+    <row r="4739">
+      <c r="A4739" t="inlineStr">
+        <is>
+          <t>6116.png</t>
+        </is>
+      </c>
+      <c r="B4739" t="inlineStr">
+        <is>
+          <t>tamilpsd-10645.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="4740">
+      <c r="A4740" s="3" t="inlineStr">
+        <is>
+          <t>6115.png</t>
+        </is>
+      </c>
+      <c r="B4740" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-10646.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="4741">
+      <c r="A4741" t="inlineStr">
+        <is>
+          <t>6114.png</t>
+        </is>
+      </c>
+      <c r="B4741" t="inlineStr">
+        <is>
+          <t>tamilpsd-10647.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="4742">
+      <c r="A4742" s="3" t="inlineStr">
+        <is>
+          <t>6113.png</t>
+        </is>
+      </c>
+      <c r="B4742" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-10648.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="4743">
+      <c r="A4743" t="inlineStr">
+        <is>
+          <t>6112.png</t>
+        </is>
+      </c>
+      <c r="B4743" t="inlineStr">
+        <is>
+          <t>tamilpsd-10649.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="4744">
+      <c r="A4744" s="3" t="inlineStr">
+        <is>
+          <t>6111.png</t>
+        </is>
+      </c>
+      <c r="B4744" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-10650.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="4745">
+      <c r="A4745" t="inlineStr">
+        <is>
+          <t>6110.png</t>
+        </is>
+      </c>
+      <c r="B4745" t="inlineStr">
+        <is>
+          <t>tamilpsd-10651.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="4746">
+      <c r="A4746" s="3" t="inlineStr">
+        <is>
+          <t>6109.png</t>
+        </is>
+      </c>
+      <c r="B4746" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-10652.png</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
🤖 Progress: 2026-04-26 12:42 UTC
</commit_message>
<xml_diff>
--- a/rename_log.xlsx
+++ b/rename_log.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4746"/>
+  <dimension ref="A1:C4796"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -57049,6 +57049,856 @@
         </is>
       </c>
     </row>
+    <row r="4747">
+      <c r="A4747" t="inlineStr">
+        <is>
+          <t>6108.png</t>
+        </is>
+      </c>
+      <c r="B4747" t="inlineStr">
+        <is>
+          <t>tamilpsd-10654.png</t>
+        </is>
+      </c>
+      <c r="C4747" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6IlhUZ2tZQUxpWWhMb2hwUk1XdGJrSVE9PSIsInZhbHVlIjoiUURHWlNxYlJpSEpzUm9yM0cwOTc5dz09IiwibWFjIjoiM2RhZjlmNDhmNGI0YjdlMDJkYWNhMDkxNWRkMDA3NzJmNzgwNTUyNGZkZjEzMTc2N2Q1MTk1ZTY3YmM3NWE4MSIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4748">
+      <c r="A4748" s="3" t="inlineStr">
+        <is>
+          <t>5496.png</t>
+        </is>
+      </c>
+      <c r="B4748" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-10655.png</t>
+        </is>
+      </c>
+      <c r="C4748" s="3" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6Im13L1hSS0M1NzB2bGlGcE53YVJRWmc9PSIsInZhbHVlIjoiRHVCMHlTRGZubStzQVZnZzRyS1oxdz09IiwibWFjIjoiZTg0MGZkYzExOTBkY2JkMDkxMzkzMDgzOGJmYTFhMTAxOTI5ZDJmYTc2MjI0MmE3ZDlmNmMyYzc0NjVkYzA5YiIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4749">
+      <c r="A4749" t="inlineStr">
+        <is>
+          <t>5491.png</t>
+        </is>
+      </c>
+      <c r="B4749" t="inlineStr">
+        <is>
+          <t>tamilpsd-10656.png</t>
+        </is>
+      </c>
+      <c r="C4749" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6IklQZXVQeVhIN3MveUkwOVFiSGxDcHc9PSIsInZhbHVlIjoiTXNuZjR5MGk3b1BISjZRSEgvYzV5QT09IiwibWFjIjoiZDk4ZTBmNzljMGQ0NTA3YWM5YzliNTFlNzg4OWVmNDA3OWNjMWUxMzBjM2RlNzA5YzZiZmY4MWZlM2RlYTFkNyIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4750">
+      <c r="A4750" s="3" t="inlineStr">
+        <is>
+          <t>5493.png</t>
+        </is>
+      </c>
+      <c r="B4750" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-10657.png</t>
+        </is>
+      </c>
+      <c r="C4750" s="3" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6IjNjWkVvQWhUUk1tMjVhbHkyVVorMWc9PSIsInZhbHVlIjoiT2Jub1F0OXJ1RUsvaFRJbFo4bVNWdz09IiwibWFjIjoiNmNkYmRiZjdlOTlhM2YyYTE4NGE0ZmE1MTAzYzE5MDJlOWM4YmNjYzNiNzY1ZmVlM2U2NjE4ZmNmNWY1MmE2MiIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4751">
+      <c r="A4751" t="inlineStr">
+        <is>
+          <t>5495.png</t>
+        </is>
+      </c>
+      <c r="B4751" t="inlineStr">
+        <is>
+          <t>tamilpsd-10658.png</t>
+        </is>
+      </c>
+      <c r="C4751" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6Ilg0UjBjemd0bFJsWDR5NUpUeHg4Tmc9PSIsInZhbHVlIjoiSDVtU1o1OUtKMWlLV0szVi9iYW1qdz09IiwibWFjIjoiYjlhYjM3YTJjY2UwZTBmYTFiYWQwMGM1ZDBkYTEyOGRiM2I1ZmE4NmIyNGNjYmMzNmM5NmJjYzVlZmY2MDRhZiIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4752">
+      <c r="A4752" s="3" t="inlineStr">
+        <is>
+          <t>5497.png</t>
+        </is>
+      </c>
+      <c r="B4752" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-10659.png</t>
+        </is>
+      </c>
+      <c r="C4752" s="3" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6InRzWjd0SUZVNjQ3ekpFU1l1dmhwNkE9PSIsInZhbHVlIjoiTk1iQzVtS2ZQVUo5NVRDeXNHUGVJdz09IiwibWFjIjoiNTU1NWFjYjFlZmFjYmUwMDVmM2ZhMmRhZjdjYTQzYjQxN2QxODM5MTBjNWI5NDg4Y2ZiZDEyNzg1NmVmNzdmYiIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4753">
+      <c r="A4753" t="inlineStr">
+        <is>
+          <t>5034.png</t>
+        </is>
+      </c>
+      <c r="B4753" t="inlineStr">
+        <is>
+          <t>tamilpsd-10660.png</t>
+        </is>
+      </c>
+      <c r="C4753" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6IkpLMGM1bk9OYXhIeS8xTmYwTU9ERHc9PSIsInZhbHVlIjoicU1hM0xjaHA1OTRmdlNZeW5zUnRYZz09IiwibWFjIjoiODI0ODM4YzE3Y2RlNjMyM2YxZjc0ODY4M2M4ZTU0MDU1Yzc4ZTlhNjE4ZWE3ZDA3NWU1MDNiZTg4M2MxODRhMSIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4754">
+      <c r="A4754" s="3" t="inlineStr">
+        <is>
+          <t>5032.png</t>
+        </is>
+      </c>
+      <c r="B4754" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-10661.png</t>
+        </is>
+      </c>
+      <c r="C4754" s="3" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6Ikp5NThDQnY3SDRNZEl1aVlxMHFNU1E9PSIsInZhbHVlIjoiUGJjZ2ROYVJydmhaaUpobnMwZ1F5dz09IiwibWFjIjoiNDMyNmEwMjUyOWMyNGI4MDBmNzEyNDNmNGIwMjkxMjkxMzhkM2FlY2JhYWJhNzE1NGFiZmRiZmQ2YzY2MWM1NyIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4755">
+      <c r="A4755" t="inlineStr">
+        <is>
+          <t>5035.png</t>
+        </is>
+      </c>
+      <c r="B4755" t="inlineStr">
+        <is>
+          <t>tamilpsd-10662.png</t>
+        </is>
+      </c>
+      <c r="C4755" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6ImpSc05vWWFKMkMyUDdYTXpvck5Ganc9PSIsInZhbHVlIjoiYWpQT1M4U1V1WmdZRnR0RHhxN2tpUT09IiwibWFjIjoiYjFmODI0YzA4NmM1NGU2NmNiYTFlZDNhMTk5ZTAxMDE0MDU3YWE4M2Y1YjAyNzYyMDBhMDk3Mjk2ZTA0YzBjNyIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4756">
+      <c r="A4756" s="3" t="inlineStr">
+        <is>
+          <t>5033.png</t>
+        </is>
+      </c>
+      <c r="B4756" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-10663.png</t>
+        </is>
+      </c>
+      <c r="C4756" s="3" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6IkxDeXRsVWxCdmhBNUY4R1IvTXZBcnc9PSIsInZhbHVlIjoiR3BSVmtEQzdZNVVQcENqQ3RxNE9YUT09IiwibWFjIjoiZjVkYjg1OWI5ZjMzOWUwZGY0NTgyZWFlNDc0MTc0ZmMxMjk0NmZkMjU0MDU0YTFjYzdmMDMxYTNmM2QxZGJjZSIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4757">
+      <c r="A4757" t="inlineStr">
+        <is>
+          <t>5028.png</t>
+        </is>
+      </c>
+      <c r="B4757" t="inlineStr">
+        <is>
+          <t>tamilpsd-10664.png</t>
+        </is>
+      </c>
+      <c r="C4757" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6InN4OW9zQzI2WW5yazYrRUdqYWd0Y3c9PSIsInZhbHVlIjoiMFJVMk5HdjVibk13UXlmUnoyV2pzZz09IiwibWFjIjoiMTgxMWFhNDZjYTZhYTkxOWMyNTM5OTI5MGViZDZjNTVhMmM4ZGE5ZTRkOWQ4NWYxMTZjMTBkYjJjMmIzODIxYyIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4758">
+      <c r="A4758" s="3" t="inlineStr">
+        <is>
+          <t>5027.png</t>
+        </is>
+      </c>
+      <c r="B4758" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-10665.png</t>
+        </is>
+      </c>
+      <c r="C4758" s="3" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6IjBuZExEakMwNnM1dUs0bEt6Yy8rbXc9PSIsInZhbHVlIjoiS09VWFZ4dE9ta2FhS1JHajZVR2ZCZz09IiwibWFjIjoiYTI0YWRlNjljOTg2OGE4Mjk3ZTBhNmZmODk1M2VjNjc3NzViMDEzMzdmYjhkMWUwNjQ4MTdlZGEwMGIzOTI3YSIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4759">
+      <c r="A4759" t="inlineStr">
+        <is>
+          <t>5026.png</t>
+        </is>
+      </c>
+      <c r="B4759" t="inlineStr">
+        <is>
+          <t>tamilpsd-10666.png</t>
+        </is>
+      </c>
+      <c r="C4759" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6IlFQUDRlekhLamh2WU9oeFc2UmVzM0E9PSIsInZhbHVlIjoiTWJtK05uUWoxaDNDaUtrc1NYNHkxUT09IiwibWFjIjoiNjdjZmU2YWVmYzI4Njk0N2ZlNmUxNTJmZWE3MTU2ZmQ5NDlmNWNkODYyNDg2YWNmNGJmN2Q3MjU1MTE3ZDJiZCIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4760">
+      <c r="A4760" s="3" t="inlineStr">
+        <is>
+          <t>5029.png</t>
+        </is>
+      </c>
+      <c r="B4760" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-10667.png</t>
+        </is>
+      </c>
+      <c r="C4760" s="3" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6IkFsRTdnWVc5dVAxaDdOY2p5OTJCclE9PSIsInZhbHVlIjoiSTV2Y3lDd1YvSkVzaVhSQzN3MzZ4QT09IiwibWFjIjoiMjk3YjZkZWM2NmIxNTEwMjcxYjk2NDZhZTI0NTc5YTJkYTNlOWFlZTlkYTg5YjI3ZWYwZWI1NDMyOTlmNDc0NCIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4761">
+      <c r="A4761" t="inlineStr">
+        <is>
+          <t>5031.png</t>
+        </is>
+      </c>
+      <c r="B4761" t="inlineStr">
+        <is>
+          <t>tamilpsd-10668.png</t>
+        </is>
+      </c>
+      <c r="C4761" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6ImZFZE54aGtEWUluOEtCZDRCZE5TbkE9PSIsInZhbHVlIjoiQmFlSGJVcTBXN3FCQUwzbVd0MlJxUT09IiwibWFjIjoiOGFmZTgyZTAxOTkyNzE0ZDdjZTVjZTg3OWY3NThmZjFmNTg3NGUzMjAxYTEzNjg3YmI5ODM0MTY4MTFjOGE1ZCIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4762">
+      <c r="A4762" s="3" t="inlineStr">
+        <is>
+          <t>5030.png</t>
+        </is>
+      </c>
+      <c r="B4762" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-10669.png</t>
+        </is>
+      </c>
+      <c r="C4762" s="3" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6IklvRUk2SW1WZEgwMVpLcEw1cjhkZnc9PSIsInZhbHVlIjoiVkhORnQwK1BLRUs3R0NYTlJQUkJJQT09IiwibWFjIjoiMzY4YWRkMWI2ZjVjYmRmNzdlMThmY2JkZjQ4ZWU2MzdlMGMzNjVlMTc4MTBmMmRiNDFhZWQxZDIwZGVlZWQxZCIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4763">
+      <c r="A4763" t="inlineStr">
+        <is>
+          <t>5025.png</t>
+        </is>
+      </c>
+      <c r="B4763" t="inlineStr">
+        <is>
+          <t>tamilpsd-10670.png</t>
+        </is>
+      </c>
+      <c r="C4763" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6ImNseVdHUjk1bGsvbitBckRCYlp6Z1E9PSIsInZhbHVlIjoiSTRkbWZmUXFsQm5hblpWZlc2WDhYQT09IiwibWFjIjoiZThhMjc2MDA3ZGNhZTZkNGQxNTBjZjE1NjIyYTQ2ODcyZDE2YjQyYzFiMGY3OTUyNjE2YWFjN2Y5Y2VmMjAyZSIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4764">
+      <c r="A4764" s="3" t="inlineStr">
+        <is>
+          <t>5024.png</t>
+        </is>
+      </c>
+      <c r="B4764" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-10671.png</t>
+        </is>
+      </c>
+      <c r="C4764" s="3" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6IjNBcW1vcmN1Q1YzYnpYMzZUSWM2L3c9PSIsInZhbHVlIjoiM0FwaEFjVEFyZklUM1Y1VzZGWjhXZz09IiwibWFjIjoiOTIzODM1MzlhNzc0ODE2MWNjYTM0Zjg2YzI2YjA4OTllMWI4Y2FiZTdkMjMxNWQ2ZDAyOGQwMmMwN2U3MjZjMCIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4765">
+      <c r="A4765" t="inlineStr">
+        <is>
+          <t>5021.png</t>
+        </is>
+      </c>
+      <c r="B4765" t="inlineStr">
+        <is>
+          <t>tamilpsd-10672.png</t>
+        </is>
+      </c>
+      <c r="C4765" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6InM4WWpGRWhtRnhjdzcveCt1b2piYXc9PSIsInZhbHVlIjoiRDBwSmhMb1VLaG82d25OQUhLR3dIQT09IiwibWFjIjoiMDI2Njg1N2MxMmVlY2E5ZjY4YmIzZDdlYzU5OTdlNzJkZTBjY2I4MmUzNmVmZTE0MzYxNDhhOGFkY2M1OTQxYiIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4766">
+      <c r="A4766" s="3" t="inlineStr">
+        <is>
+          <t>5023.png</t>
+        </is>
+      </c>
+      <c r="B4766" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-10673.png</t>
+        </is>
+      </c>
+      <c r="C4766" s="3" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6IlUyRUpRWG9SZ3lLVHE4cFZicVoxUHc9PSIsInZhbHVlIjoidVpDaHgwM1Zjajl5QnRWMDNVc2o3Zz09IiwibWFjIjoiNzFiMWE1YzE1OWQ0OTljNTJhN2RlZTkzZWE3ZDQ1MmRiMzhmNDE4ZmQ5ZjVmZDA1M2ZkMjc0MGQ4NDJmNzYyOSIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4767">
+      <c r="A4767" t="inlineStr">
+        <is>
+          <t>5020.png</t>
+        </is>
+      </c>
+      <c r="B4767" t="inlineStr">
+        <is>
+          <t>tamilpsd-10674.png</t>
+        </is>
+      </c>
+      <c r="C4767" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6IlluNEhGTmduZFh0Ykw2anpyNFdyRnc9PSIsInZhbHVlIjoiVzg5MGl6aEl0OGtSS0kyRWRFRExGQT09IiwibWFjIjoiZDViOWQ5MDYwYjc2YjkwNjgwODdmZmIxNjY4NjJhNGM0MGQxMzMzYWM5MmRiMmQ2YjU0NzRlYmI2NGU4NDc5YyIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4768">
+      <c r="A4768" s="3" t="inlineStr">
+        <is>
+          <t>5019.png</t>
+        </is>
+      </c>
+      <c r="B4768" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-10675.png</t>
+        </is>
+      </c>
+      <c r="C4768" s="3" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6Ijk3YnVVSkNieUpWY3BQREg2cHZvZWc9PSIsInZhbHVlIjoiQk13ekFnODVYb1VhZTNISThDcUI2Zz09IiwibWFjIjoiNGY4Yzk4NGUxNjc4NDAxZWFmMWU5NjllZTM2OWMxMzk0MzVhNGFjYzIxMTYzMDYxY2UzMWQ0NjQ0MzU3MmE3NyIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4769">
+      <c r="A4769" t="inlineStr">
+        <is>
+          <t>5022.png</t>
+        </is>
+      </c>
+      <c r="B4769" t="inlineStr">
+        <is>
+          <t>tamilpsd-10676.png</t>
+        </is>
+      </c>
+      <c r="C4769" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6Im02YmlnMW5MWmRVV1JLMmt1c2xiNUE9PSIsInZhbHVlIjoiS1FTdnVXdHRaTWplRDExUWFNNWFrUT09IiwibWFjIjoiMmIzODZhOTU2ZWU4OTVhYjM3ZTdhMjNiMDEwNmFjMGVmYmJiOTg4N2QxNWU1NDdmNGZiMDgwYTUzNzcwOWM5MyIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4770">
+      <c r="A4770" s="3" t="inlineStr">
+        <is>
+          <t>5018.png</t>
+        </is>
+      </c>
+      <c r="B4770" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-10677.png</t>
+        </is>
+      </c>
+      <c r="C4770" s="3" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6IlJUSGFkdTRQdVVWSGt6UXN4OGZvMEE9PSIsInZhbHVlIjoiK3hGSkFsVjExN1dReXFPQmFGQUxkQT09IiwibWFjIjoiMzQ0NzIzZjU5NjdjZWNhZjU2Zjg3YjcwZDRhYjMyNTlhMWIwZmU2Nzk5NDk2MjgzY2NiMDA1Yjk0MzEwYjczOCIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4771">
+      <c r="A4771" t="inlineStr">
+        <is>
+          <t>5016.png</t>
+        </is>
+      </c>
+      <c r="B4771" t="inlineStr">
+        <is>
+          <t>tamilpsd-10678.png</t>
+        </is>
+      </c>
+      <c r="C4771" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6IlBMZ214bnk5VWl0alJZSWdqcXU1OHc9PSIsInZhbHVlIjoiT1dOWTJHWlU5ci9oa0gxOC96cGVuQT09IiwibWFjIjoiN2FiMWY3YjI1ZGJhNDllMjdmMWY1YTUyZjZiMmQ3YWEyMDgzOWMxNmNkOGUyODA3ZGQwY2E4MThhZWFmMzZlNyIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4772">
+      <c r="A4772" s="3" t="inlineStr">
+        <is>
+          <t>5017.png</t>
+        </is>
+      </c>
+      <c r="B4772" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-10679.png</t>
+        </is>
+      </c>
+      <c r="C4772" s="3" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6ImNmTzQ1UC9BWk5oQnpXWVNmdis1OEE9PSIsInZhbHVlIjoiL0QrNUxlSDM5M1lnZFNESHI2cHhjdz09IiwibWFjIjoiYzMzY2RhMTE4YTJkMGQ5NTY5NDQ3ODBiYTZjOWU5NGVlZGNhZTRkZTY5YTc3M2VmMDUxYTk4YzM2OTU1ZjcxNiIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4773">
+      <c r="A4773" t="inlineStr">
+        <is>
+          <t>5013.png</t>
+        </is>
+      </c>
+      <c r="B4773" t="inlineStr">
+        <is>
+          <t>tamilpsd-10680.png</t>
+        </is>
+      </c>
+      <c r="C4773" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6IjN1Ly90UEpCUU5yOXppRHcyZU5hdWc9PSIsInZhbHVlIjoiWGtSSGZ4bjRXVUFqeTZ5WGFWN0x0UT09IiwibWFjIjoiM2I5MzFhNjQ3ZmYxYzAzMGYwMzZkZDVlMGY0NjBlMDQ4NjZiYzU2NzY4Y2M0MTFmZTA3Yjc2NGMyZWRlZDRhZiIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4774">
+      <c r="A4774" s="3" t="inlineStr">
+        <is>
+          <t>5015.png</t>
+        </is>
+      </c>
+      <c r="B4774" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-10681.png</t>
+        </is>
+      </c>
+      <c r="C4774" s="3" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6IkpOeGtaSjd0VkdIRk1MajcwUHZUdkE9PSIsInZhbHVlIjoiS2ZSNloxamROcXNFY0tnWnhkN0o5UT09IiwibWFjIjoiYWE3Mjg4MDdkZGUyNDBhYjk5MzcyMGY2NGJmNWM4OGY5ZTEzZmYwMjdkZjg1NDQ2NTJlYjlmNTY2OTlhMWU2MCIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4775">
+      <c r="A4775" t="inlineStr">
+        <is>
+          <t>5014.png</t>
+        </is>
+      </c>
+      <c r="B4775" t="inlineStr">
+        <is>
+          <t>tamilpsd-10682.png</t>
+        </is>
+      </c>
+      <c r="C4775" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6ImVYaExydlN6ZE12dEJJQ3pBYVRzRXc9PSIsInZhbHVlIjoielQ4NjR5Tyt5ajBOeWVJSzNpRDJqdz09IiwibWFjIjoiMDc2ZTdjNTkxN2RiNmQ3ZTZkOWFmYjJmYzljZjgzOTdkM2I0ODk2ZWRiZjk2MmM1MjI0YjZlZTQzZWU3YzVjOSIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4776">
+      <c r="A4776" s="3" t="inlineStr">
+        <is>
+          <t>5012.png</t>
+        </is>
+      </c>
+      <c r="B4776" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-10683.png</t>
+        </is>
+      </c>
+      <c r="C4776" s="3" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6ImFLTlEwM0ZQd0NCWmRLaVExTDhWQnc9PSIsInZhbHVlIjoid045R2lOeUR6WldTUlVhalpkTDNxZz09IiwibWFjIjoiNzZiNjNlMTA4MWUxZTk5ZDdkYWUwZTBmMjM5ZTczNGY4NWJhMDBlMWJmNjVlZWVjZWM5NDZmYzY1NzZkY2YxZCIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4777">
+      <c r="A4777" t="inlineStr">
+        <is>
+          <t>5011.png</t>
+        </is>
+      </c>
+      <c r="B4777" t="inlineStr">
+        <is>
+          <t>tamilpsd-10684.png</t>
+        </is>
+      </c>
+      <c r="C4777" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6Ik5SVTFMQ25MZkJrS1ZVdFFLcTczSEE9PSIsInZhbHVlIjoibkhXdUt0cUFQYUpxR2ZvZ2oxY3J0UT09IiwibWFjIjoiOWRhNjhiZGU3Mzk3MWMzNDMxOGI4ODQ0ZDNhMzEyNTYzMGYyYTcxY2EyZmQ5NzU3NmI4NzEyN2VmZDQ0YWJiMCIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4778">
+      <c r="A4778" s="3" t="inlineStr">
+        <is>
+          <t>4994.png</t>
+        </is>
+      </c>
+      <c r="B4778" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-10685.png</t>
+        </is>
+      </c>
+      <c r="C4778" s="3" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6IlBIeVhIcjErQUpzSElwaFhhZ00zYnc9PSIsInZhbHVlIjoiZHdzR0lYZUV5THhXMjR1eWNPbE9odz09IiwibWFjIjoiMTVmOGUyMGI1MjJmNWMxZTNkMjVmY2IzODJkMDBlYWE5ZGEwOGRlYWM2Zjc1NzlkNTFiNGY5ZjlhYjlhZGJmNiIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4779">
+      <c r="A4779" t="inlineStr">
+        <is>
+          <t>4995.png</t>
+        </is>
+      </c>
+      <c r="B4779" t="inlineStr">
+        <is>
+          <t>tamilpsd-10686.png</t>
+        </is>
+      </c>
+      <c r="C4779" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6InVpRFNBS3dmNGN2TEhmdlpsRVBzdEE9PSIsInZhbHVlIjoiZDBvUlhhdzdxV2F6ZEVtTGVuZ1NWZz09IiwibWFjIjoiZjVlM2QyZGY2NGUwNzRiZjkzZGI2OGQ0MDY2MGUzMDJmNGM3OTQxMWVkMzg2ZTlkOTAxMmFmOTU4ZDFmOTE2NyIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4780">
+      <c r="A4780" s="3" t="inlineStr">
+        <is>
+          <t>4992.png</t>
+        </is>
+      </c>
+      <c r="B4780" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-10687.png</t>
+        </is>
+      </c>
+      <c r="C4780" s="3" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6InFrbHJ5ckpaVUdpaVFBcWlWbVhIYXc9PSIsInZhbHVlIjoiMTd3VVI0OGE0TDZGMnNDOWFOL1Y1Zz09IiwibWFjIjoiZmRkYThkYTIzNDNlYzVkMWI1OGM1ZjM4Y2UyMjQyYjM1ZjZmNmUxM2NkMWUzYmIwOWY5YTY0OTE0YTI1OWZjMCIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4781">
+      <c r="A4781" t="inlineStr">
+        <is>
+          <t>4991.png</t>
+        </is>
+      </c>
+      <c r="B4781" t="inlineStr">
+        <is>
+          <t>tamilpsd-10688.png</t>
+        </is>
+      </c>
+      <c r="C4781" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6InZIZnU4bmJoVEczZ1hQSXd0T3NRMnc9PSIsInZhbHVlIjoiLytvZmNKQ1NDUG43eTROcXZGY1hoZz09IiwibWFjIjoiZWRmNmFmOGIwYzZhYzc1MWY4NDNiNjE5OGM2YTdjZjM5ZTU5MGEyNDhmZjBkZWVlNGE4NTUzZDNmYzgyNzhhNSIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4782">
+      <c r="A4782" s="3" t="inlineStr">
+        <is>
+          <t>4993.png</t>
+        </is>
+      </c>
+      <c r="B4782" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-10689.png</t>
+        </is>
+      </c>
+      <c r="C4782" s="3" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6IkJaeE5sNHV5SWtSM09OQjlaUGJCWVE9PSIsInZhbHVlIjoiQm1sMzMraDVrR1lLOEluZlk3MDJ2Zz09IiwibWFjIjoiYjBlYWM4YjY2ZDhiMmI1MDlkNTQwYWFhMWQ1MDQ0NzdjZTc3N2MyODMxNDA4M2Q3NDI4YzFhNmE3MTk4NGM4MiIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4783">
+      <c r="A4783" t="inlineStr">
+        <is>
+          <t>5036.png</t>
+        </is>
+      </c>
+      <c r="B4783" t="inlineStr">
+        <is>
+          <t>tamilpsd-10690.png</t>
+        </is>
+      </c>
+      <c r="C4783" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6ImRjbFZ2ekFySjVHN3ZiVG52NjkzVGc9PSIsInZhbHVlIjoiQXJoZXoyVlRuOXdZQ1FtUFJlVWRUUT09IiwibWFjIjoiMmQ4YjUwMGQzMGMzNWNhYWUyNWExODI3NDM2MjA4OTgxODUzYzBiZjM5ZDc2ODA5YmRkY2UyYzM2MDhkYmFkYyIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4784">
+      <c r="A4784" s="3" t="inlineStr">
+        <is>
+          <t>4990.png</t>
+        </is>
+      </c>
+      <c r="B4784" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-10691.png</t>
+        </is>
+      </c>
+      <c r="C4784" s="3" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6IjNpaTBzNjRuYzhxWDZrY2txcWRqbkE9PSIsInZhbHVlIjoiYXRYZlV1SkwvaFJYdWpGZHdzZUFXUT09IiwibWFjIjoiNjY1ZWY0MWFiZTg5NjBmYWVhN2JjNjY0NjYwZGYxZDZlODNiZWM5ODU0YTFmMTRlNGIwODUyODA0NjUyZWVhNiIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4785">
+      <c r="A4785" t="inlineStr">
+        <is>
+          <t>4985.png</t>
+        </is>
+      </c>
+      <c r="B4785" t="inlineStr">
+        <is>
+          <t>tamilpsd-10692.png</t>
+        </is>
+      </c>
+      <c r="C4785" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6Im9wcDZ4QXMrZE1UZm45TCs0c2tFOEE9PSIsInZhbHVlIjoiVkhRSTJxR2QwQWloVEtoaHM0R2svUT09IiwibWFjIjoiNDU2YTBiZGI2NDk2ZGZlODM1MGM2YzI4YzhjZmViMmQ5MzViYjJmNGUxMmZkMDEyYWE4ZmUxMzY2OTEzMTVlMyIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4786">
+      <c r="A4786" s="3" t="inlineStr">
+        <is>
+          <t>4984.png</t>
+        </is>
+      </c>
+      <c r="B4786" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-10693.png</t>
+        </is>
+      </c>
+      <c r="C4786" s="3" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6Ilk0T3kwZ2pOT0Fnb3NHck5uYlZQQ2c9PSIsInZhbHVlIjoiYVF6MHBqWDliRkZ1WVpBUTJaQ2dyUT09IiwibWFjIjoiOGU0YTAwZTlmZTgyN2Y4OWQ0ZmNjMjRhMWRiMTMyMGZkMjM3MmE0MDNmZDUwOGU5ZTZhNjBiYTg5MjNmNmI4YSIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4787">
+      <c r="A4787" t="inlineStr">
+        <is>
+          <t>4980.png</t>
+        </is>
+      </c>
+      <c r="B4787" t="inlineStr">
+        <is>
+          <t>tamilpsd-10694.png</t>
+        </is>
+      </c>
+      <c r="C4787" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6IllORSszbEpnN3BQYzB5MG45SGRNMnc9PSIsInZhbHVlIjoiSXFqY1lwMmtQUTViU2I3UDhKQjZLQT09IiwibWFjIjoiNzZhOTEwMzNhY2U2MDg3M2E3ODJjNWVlNWMzMTUyNmE4ZWIwOWQ3OGE5Y2FlYWM5NGEyNDllYmIwM2NmMjEzMSIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4788">
+      <c r="A4788" s="3" t="inlineStr">
+        <is>
+          <t>4983.png</t>
+        </is>
+      </c>
+      <c r="B4788" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-10695.png</t>
+        </is>
+      </c>
+      <c r="C4788" s="3" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6IkZhUzVuZmtXWVhmVWpnWG81Z1ZCcGc9PSIsInZhbHVlIjoicU1aR0J4ZHZjdm9tUndOR1F1bDdCZz09IiwibWFjIjoiNzI0ZTY0NzVkYjExMjRhMjVhYTQwNjdhYjRiNzM2ODExYTAwZmJlMzRiYTg5NWNlMzc4Mzg5MGI0NzM1ZTI5NSIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4789">
+      <c r="A4789" t="inlineStr">
+        <is>
+          <t>4981.png</t>
+        </is>
+      </c>
+      <c r="B4789" t="inlineStr">
+        <is>
+          <t>tamilpsd-10696.png</t>
+        </is>
+      </c>
+      <c r="C4789" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6ImZzeUQ4a1pxVVArdzljSys4VGR6Vmc9PSIsInZhbHVlIjoibWs5dzJYWVFWcU1hU041MXRwa0cxZz09IiwibWFjIjoiOTI2MjhhZDVhZGQyMGI4OTRhMDdlM2M0OWNiMGRkMWJjYTdmNDAxZWY4NjE5YjY0NDg4NmMzZjIzZGY1NjVjZiIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4790">
+      <c r="A4790" s="3" t="inlineStr">
+        <is>
+          <t>4978.png</t>
+        </is>
+      </c>
+      <c r="B4790" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-10697.png</t>
+        </is>
+      </c>
+      <c r="C4790" s="3" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6ImlwV05FR2VNQUNsS1lNekY1bWlEblE9PSIsInZhbHVlIjoiVmtsYU1aME8wZjhhVmQrTkJKN3VIZz09IiwibWFjIjoiZGJmMzMwMDdmZjJlZGJlODM3YjUzNmJhZTcyYzllNTAzOTQ1ODMxM2IwMzc3Y2M0OTBhNjk2MGI2Yzg4ZjhlMSIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4791">
+      <c r="A4791" t="inlineStr">
+        <is>
+          <t>4977.png</t>
+        </is>
+      </c>
+      <c r="B4791" t="inlineStr">
+        <is>
+          <t>tamilpsd-10698.png</t>
+        </is>
+      </c>
+      <c r="C4791" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6Ilo4RWdUWTlsTDFtT2cxTG8yL29CVlE9PSIsInZhbHVlIjoiVDVNeFh5Y3gySFBFZnpZWlllRDQwdz09IiwibWFjIjoiZGY5Yzc0MjQ2NTY0YWM3Mjc2ZDJlZjg5ZWE5NDUyOGY3ZjQ5OGI1ZDI4YTFhZThmYWE5NjEyZDI5NzA4YjYwNiIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4792">
+      <c r="A4792" s="3" t="inlineStr">
+        <is>
+          <t>4974.png</t>
+        </is>
+      </c>
+      <c r="B4792" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-10699.png</t>
+        </is>
+      </c>
+      <c r="C4792" s="3" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6IkJHdVgzS29mMjY0ck1XaU1kbDVHcGc9PSIsInZhbHVlIjoiR3RMM3BCTEdReEVBMENtRkowck9Ndz09IiwibWFjIjoiMmFlN2JkNmFiZDg5ZjNhMGEyNjMwZWY4MDQyYmZkYmQ4YjE2ZDkxNTFiMDIyYmM0NjU4ZDQzNmNiMDAyM2U2YiIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4793">
+      <c r="A4793" t="inlineStr">
+        <is>
+          <t>4975.png</t>
+        </is>
+      </c>
+      <c r="B4793" t="inlineStr">
+        <is>
+          <t>tamilpsd-10700.png</t>
+        </is>
+      </c>
+      <c r="C4793" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6IkYybnhMTFBMN2g3R1BVcGJidkVsclE9PSIsInZhbHVlIjoiNUpFYUhqT3R2ZE5rRmNtZytqNkFsUT09IiwibWFjIjoiNDA5YmU2YmFkMGNmYWQyNTAwNDllM2VjZGY1YTA5ZjYzM2RiNmNjYzhjOGY0OGU1YTNjMzQ1MmM5ZTQ5NTZlOSIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4794">
+      <c r="A4794" s="3" t="inlineStr">
+        <is>
+          <t>4973.png</t>
+        </is>
+      </c>
+      <c r="B4794" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-10701.png</t>
+        </is>
+      </c>
+      <c r="C4794" s="3" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6IlVWQ1lSMjdtb0FDWXp0TUtrRUhsdnc9PSIsInZhbHVlIjoieXhmbWxMT3JQMTVJWHZ4VXFqVFE0dz09IiwibWFjIjoiYmU5M2I4ZTM2MDBlMmUxOGRjY2FjYjFjYWZiN2ZmMDcwNGEwYzkzMzllYWMzMDM0MmE3YmM3ZTg2NGQyNDVmMCIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4795">
+      <c r="A4795" t="inlineStr">
+        <is>
+          <t>4976.png</t>
+        </is>
+      </c>
+      <c r="B4795" t="inlineStr">
+        <is>
+          <t>tamilpsd-10702.png</t>
+        </is>
+      </c>
+      <c r="C4795" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6IklmZEJ2bGVRYzRGbzM0cE5FQTFxNWc9PSIsInZhbHVlIjoiekY4V2puSHdGM2lOZUlVZmlYeGw3Zz09IiwibWFjIjoiN2Y0OTE4ZjQyYjJlN2U5M2FkZmY1NjVjMGM5ZjVhMTQ1NjQ0MzlkZmNkOTQ1YWQ1ZTUwNGY1OGZkMGY1YzNlNyIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4796">
+      <c r="A4796" s="3" t="inlineStr">
+        <is>
+          <t>4972.png</t>
+        </is>
+      </c>
+      <c r="B4796" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-10703.png</t>
+        </is>
+      </c>
+      <c r="C4796" s="3" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6IlNDU3N2ZTc4ZGVJKzNKQ3V3OFVxRUE9PSIsInZhbHVlIjoiM1AwQU41ckZPQ3dKYUVCNXFRcGppQT09IiwibWFjIjoiNDQ5MDQzMjg1ZTA5M2M5YzA2OWQ4YzQ1Y2JlOWExZjRmODY3ZTUyMjg1ZGQ4ODhjZDJkZGI4Yzg0MGY4MzQ4MyIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
🤖 Progress: 2026-04-26 14:56 UTC
</commit_message>
<xml_diff>
--- a/rename_log.xlsx
+++ b/rename_log.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4796"/>
+  <dimension ref="A1:C4845"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -57899,6 +57899,839 @@
         </is>
       </c>
     </row>
+    <row r="4797">
+      <c r="A4797" t="inlineStr">
+        <is>
+          <t>4989.png</t>
+        </is>
+      </c>
+      <c r="B4797" t="inlineStr">
+        <is>
+          <t>tamilpsd-10704.png</t>
+        </is>
+      </c>
+      <c r="C4797" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6IlVYTUZHYlRmOHMrUU80UkVIMWFleVE9PSIsInZhbHVlIjoiWWMwSE5NVGh3bWNmUVpXcTBFOVpIZz09IiwibWFjIjoiNGMxYmYxYzkxZmViMTE2YTg2MzcxMGYxNzQyODQyM2NiYzFhMDQ2ODRjMTc2ZWZkMTA1ZjlhYjBmZWQzZGYxZCIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4798">
+      <c r="A4798" s="3" t="inlineStr">
+        <is>
+          <t>4988.png</t>
+        </is>
+      </c>
+      <c r="B4798" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-10705.png</t>
+        </is>
+      </c>
+      <c r="C4798" s="3" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6InY2a2tYaU9sRVNaNHFKdmM0UE13SEE9PSIsInZhbHVlIjoiT1hIMk56Ukc1dFJreS9jbUtSdi9Mdz09IiwibWFjIjoiNTJkZDJkNGMyMmIzMWNkMTQ5MGY0M2U1M2YwODMxZDVkZmU1YmVhZWVmM2NiMmI0YzEyMWYyNjY2OTY5NzBhYSIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4799">
+      <c r="A4799" t="inlineStr">
+        <is>
+          <t>4987.png</t>
+        </is>
+      </c>
+      <c r="B4799" t="inlineStr">
+        <is>
+          <t>tamilpsd-10706.png</t>
+        </is>
+      </c>
+      <c r="C4799" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6ImtBaUl1cC9EK2xMaVJTbVlRanJFUlE9PSIsInZhbHVlIjoibDl3Mk5hdkVYTXltSW4vaXpUYzJhUT09IiwibWFjIjoiYjU2ZjcyODIzNjQzZmU0YWM2ZTk0MDRmOWFhOWNiZGZkODc0YmY0OTZiOWI1MzMyNWFjYjljNWQ1MjcwOWVlNiIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4800">
+      <c r="A4800" s="3" t="inlineStr">
+        <is>
+          <t>4986.png</t>
+        </is>
+      </c>
+      <c r="B4800" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-10707.png</t>
+        </is>
+      </c>
+      <c r="C4800" s="3" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6IjBuYlhiMExBNnlySktuZGZuTG5SUFE9PSIsInZhbHVlIjoiZldSMUN6S2hOczU3MGNpbUxHcXJMQT09IiwibWFjIjoiNzA1NzNhYjZjZThmMzk1MWZkNWQwZWUzYzc0N2M0YjliYzg5M2M2MGMxN2Y2ZmFjMzk2YzEyYzA5ZjhhOWRjMSIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4801">
+      <c r="A4801" t="inlineStr">
+        <is>
+          <t>4889.png</t>
+        </is>
+      </c>
+      <c r="B4801" t="inlineStr">
+        <is>
+          <t>tamilpsd-10708.png</t>
+        </is>
+      </c>
+      <c r="C4801" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6ImNWNjF6NjIralAwa2RldWpZWFU0bFE9PSIsInZhbHVlIjoiMkwzSzlmWDRxQkZwMVgvVHBCZ1J4dz09IiwibWFjIjoiZGVlMjNjYmU5M2YxZjI3MDIyZmUwYWZlNzM5NDQyY2I2ZTljMzZlYjFhNjgyNGFmYmM3MTE0Y2ZiM2M5M2E0ZiIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4802">
+      <c r="A4802" s="3" t="inlineStr">
+        <is>
+          <t>4888.png</t>
+        </is>
+      </c>
+      <c r="B4802" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-10709.png</t>
+        </is>
+      </c>
+      <c r="C4802" s="3" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6IjhUYTdTMWc0eXQwNUpZWG5TREttS0E9PSIsInZhbHVlIjoidEkxTVFFQWM0V1hEWThXNmtmNmZxUT09IiwibWFjIjoiNDE1ODkxZTQ1MmJjY2NiZmE4ZmU5NDViM2ZmMzQ1MTIxMWNlYjA0ODc4YjMzNDcwZjg2OTJiNjI1MmRiNTIwNCIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4803">
+      <c r="A4803" t="inlineStr">
+        <is>
+          <t>4887.png</t>
+        </is>
+      </c>
+      <c r="B4803" t="inlineStr">
+        <is>
+          <t>tamilpsd-10710.png</t>
+        </is>
+      </c>
+      <c r="C4803" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6ImxuOUNVQzFtTE9jZkNZZXltZ0tmQVE9PSIsInZhbHVlIjoiQVI0OW9xd2ZIeVBranBSRWVYSmdBZz09IiwibWFjIjoiNGNjNTZjMmRhNmYyMTRhZDUwN2UyMmE5OGY3ODlmOTI4MTQ1ODZjNzJkOThhYmZiZmM2YzlhN2IxYmIxY2UwNCIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4804">
+      <c r="A4804" s="3" t="inlineStr">
+        <is>
+          <t>4886.png</t>
+        </is>
+      </c>
+      <c r="B4804" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-10711.png</t>
+        </is>
+      </c>
+      <c r="C4804" s="3" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6IlFwUnN4OURIMFhmSjdpMDFQRHYyMGc9PSIsInZhbHVlIjoiei85WmFxeDk1TTkzTE8wdHZPN0tTdz09IiwibWFjIjoiNTViZTNmODM4MjFjMjdkY2I1ZWIzMjU1Y2UzNDU5YmMxNDY2NDI0Mzc4NGI4ZDZkNzBkYjdlMTk5NWY4MzA2ZCIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4805">
+      <c r="A4805" t="inlineStr">
+        <is>
+          <t>4885.png</t>
+        </is>
+      </c>
+      <c r="B4805" t="inlineStr">
+        <is>
+          <t>tamilpsd-10712.png</t>
+        </is>
+      </c>
+      <c r="C4805" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6Im9WcmREQlg5aCs5VlIrbGVHZ2J4NGc9PSIsInZhbHVlIjoiLzBBK3I1NFVQeUF4ZW9DUDVndXlKQT09IiwibWFjIjoiNzRiZTZjNDExNDBhNDc1OGFmOTUyNmNhMjY4Mjc5YmNjYTc2NzE0MmE0OTc2ZjVkMDAzM2Q1ZTljMmQ0NWE4YSIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4806">
+      <c r="A4806" s="3" t="inlineStr">
+        <is>
+          <t>4884.png</t>
+        </is>
+      </c>
+      <c r="B4806" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-10713.png</t>
+        </is>
+      </c>
+      <c r="C4806" s="3" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6IlpadkJONGFxMmpGdUZKYysvUGx5cWc9PSIsInZhbHVlIjoiYUd6MVFCNzcxcklqSXUzbHB0OWwrQT09IiwibWFjIjoiNTcyOGE2NjQyMjExZDEyOGI5ZWM2ZGJmY2EyYzMwMGQ1NmY3ODc2MjI4YTQ3NWEzYTkzYzgzYjVjOWVmZDZlZSIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4807">
+      <c r="A4807" t="inlineStr">
+        <is>
+          <t>4883.png</t>
+        </is>
+      </c>
+      <c r="B4807" t="inlineStr">
+        <is>
+          <t>tamilpsd-10714.png</t>
+        </is>
+      </c>
+      <c r="C4807" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6IkdNdjB3VVEwaEhDbHlnZ2RhVkQ2ZWc9PSIsInZhbHVlIjoiNm9iUkZzVUVFUldnYXBOZFZjSGJWQT09IiwibWFjIjoiZjNiNjU4NWFiMzM0YjlhYjkwMjgyMDVkOGFmZDY5MDRiYWFlZGE1YmMxMjI3OGFiMmQzYjMzNGQ0NTc4MGUxNiIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4808">
+      <c r="A4808" s="3" t="inlineStr">
+        <is>
+          <t>4882.png</t>
+        </is>
+      </c>
+      <c r="B4808" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-10715.png</t>
+        </is>
+      </c>
+      <c r="C4808" s="3" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6IlJ3QTNHais3UE9sbE96N085OHBXOHc9PSIsInZhbHVlIjoid0w4OTBTZGNxU3NoRTVpbWMrQW11dz09IiwibWFjIjoiMTI3ZDc2Mjk4NTc4MTNlNGZhYTliMjU0ZDZhMGM1ZWRiODcwZjQ3ZjgxMGY0MjFhMzUwMjQ1YTgyNzkwM2EzOCIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4809">
+      <c r="A4809" t="inlineStr">
+        <is>
+          <t>4881.png</t>
+        </is>
+      </c>
+      <c r="B4809" t="inlineStr">
+        <is>
+          <t>tamilpsd-10716.png</t>
+        </is>
+      </c>
+      <c r="C4809" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6ImVpZVZqKy94eUtSZVVjZ1BNOW11NUE9PSIsInZhbHVlIjoiVDdvV1QrODhncVFEcWNBODRNODk3UT09IiwibWFjIjoiODlhMWQxNTk3OTkzMjE0NWVhYzFlZjg0Y2I1NTEwYWZjZTc2MGY2ODhkMmYyNDgwNTFjMjExN2VhYjc4OTBiNyIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4810">
+      <c r="A4810" s="3" t="inlineStr">
+        <is>
+          <t>4880.png</t>
+        </is>
+      </c>
+      <c r="B4810" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-10717.png</t>
+        </is>
+      </c>
+      <c r="C4810" s="3" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6InIwSGJZREdibDErc214WGVOZ3duTnc9PSIsInZhbHVlIjoiL05Ndk1XQzdYYWFqdVIwZUNTeHBuZz09IiwibWFjIjoiYzBhNzY0Mjk5NDk1NDFhODAyMTUxODcxZGU3Mjg4NmRlMGE3YjdkODFlM2U2OGRlMjM2MzJmOGVhY2I1NTU4NSIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4811">
+      <c r="A4811" t="inlineStr">
+        <is>
+          <t>4879.png</t>
+        </is>
+      </c>
+      <c r="B4811" t="inlineStr">
+        <is>
+          <t>tamilpsd-10718.png</t>
+        </is>
+      </c>
+      <c r="C4811" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6Im5ZamlUL3UzenNhQzNKVTV0VXhoVkE9PSIsInZhbHVlIjoiSEpEcVF0Q2xCTzBiQzNKUVlsMDVjZz09IiwibWFjIjoiNDUxNjc3MDNmZGIxZWI0YzBjYTQyYWQyMjQ1YjcyMmZlODI3ZTk3NWY2NDc3YmE2Y2NlMGUxMmJiMGQ5Y2Q5MSIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4812">
+      <c r="A4812" s="3" t="inlineStr">
+        <is>
+          <t>4878.png</t>
+        </is>
+      </c>
+      <c r="B4812" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-10719.png</t>
+        </is>
+      </c>
+      <c r="C4812" s="3" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6ImRKL2Q0RkZIWXM3alhGUGcydks2bnc9PSIsInZhbHVlIjoiZDR5ZkhsQUJ0RUluT2NaVU4yNEhCdz09IiwibWFjIjoiZWI0NjVkYWUyZjgxODhlYjFhMWQ4M2VkMTFlMTkwMDJkY2FiNDgwMjFmNTgwNTVjYWNjNDI4MTNhZWY4NGJiYSIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4813">
+      <c r="A4813" t="inlineStr">
+        <is>
+          <t>4877.png</t>
+        </is>
+      </c>
+      <c r="B4813" t="inlineStr">
+        <is>
+          <t>tamilpsd-10720.png</t>
+        </is>
+      </c>
+      <c r="C4813" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6ImtHWVBqZ3Bvd1VrY0lNTFh2M250SXc9PSIsInZhbHVlIjoibnNBaUFUcGpUUDc5Yk5jamdrejFKZz09IiwibWFjIjoiZGIzNTkyM2Y0ZjI5MWJjYjYyNjViNjBiYjMyNTVkNDU4MDdlMzQxNmE1NmQ3YjU4ODg4NjczYzJmYTVjMzc4MSIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4814">
+      <c r="A4814" s="3" t="inlineStr">
+        <is>
+          <t>4876.png</t>
+        </is>
+      </c>
+      <c r="B4814" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-10721.png</t>
+        </is>
+      </c>
+      <c r="C4814" s="3" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6Ijd2SnpVaThKT2xYb2IwenRKekxxK0E9PSIsInZhbHVlIjoib3YrVzlHNmJ5Q2FvMTNXRzVyNUQwZz09IiwibWFjIjoiNTdmNTFhNGJhMmVjODIzNTZjZWExNmJmMjRiOWVmNzdiMDhmMjkyOGY5NmRhMzFmYzViNThiMWVmODVlYmFjMyIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4815">
+      <c r="A4815" t="inlineStr">
+        <is>
+          <t>4875.png</t>
+        </is>
+      </c>
+      <c r="B4815" t="inlineStr">
+        <is>
+          <t>tamilpsd-10722.png</t>
+        </is>
+      </c>
+      <c r="C4815" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6IjQzSVVtOUp0enlXZllBVHpPN0ZTTVE9PSIsInZhbHVlIjoiTnpZYjE4R0pmZmppMlhNMXEyVWQwdz09IiwibWFjIjoiNTU3ZmU1YWViYjVjYWY3NTdiMGRlMzU5NzhkN2NmZDRlNjUxNTkyYzU5NzAwZTI4YzNkYTBjODdmZWRhMDU5OCIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4816">
+      <c r="A4816" s="3" t="inlineStr">
+        <is>
+          <t>4874.png</t>
+        </is>
+      </c>
+      <c r="B4816" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-10723.png</t>
+        </is>
+      </c>
+      <c r="C4816" s="3" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6ImhRekNyQzJxeDNLb1NMQU53S0p4TFE9PSIsInZhbHVlIjoiT0s4RGEvaWoxR2g2Q2J4Ui92T1NIQT09IiwibWFjIjoiNTMzZTIxMDg0MjQxMWRjZWIzNDQzMzBiNTc5ZWM1NzdiNmFmZjlhYjVmMGJkY2IxZjNiMTA4ZjFlNzgwYTU0MCIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4817">
+      <c r="A4817" t="inlineStr">
+        <is>
+          <t>4873.png</t>
+        </is>
+      </c>
+      <c r="B4817" t="inlineStr">
+        <is>
+          <t>tamilpsd-10724.png</t>
+        </is>
+      </c>
+      <c r="C4817" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6IlJQTDJ3NWxNd2x1enRKejZiZVdZVmc9PSIsInZhbHVlIjoiV3E0YmhBSEtTVHNyMFNkaEVvcDJyUT09IiwibWFjIjoiNDJjZjQzY2UxMTJlMDQ3YjYyZmQwZGU3M2Y4NzdlZWZiOGI1NTdjOWVlYmMxODc4OWRhMjk3Mjg3NTdmYjkyMiIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4818">
+      <c r="A4818" s="3" t="inlineStr">
+        <is>
+          <t>4872.png</t>
+        </is>
+      </c>
+      <c r="B4818" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-10725.png</t>
+        </is>
+      </c>
+      <c r="C4818" s="3" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6ImI3N3YwQlc5SW9tUkx2UktlZ0tzVXc9PSIsInZhbHVlIjoiUWl6YmFubmo5L3R0OFB6WFE5Sjd0dz09IiwibWFjIjoiNGFiN2Q4YjA3MzNjMGIzYWYyNmI1MGIxYzNlZTBhMTZjYzAwYzc3NDliNWQzYjk0Y2YxYzFlNmNlYzljYTQzMCIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4819">
+      <c r="A4819" t="inlineStr">
+        <is>
+          <t>4871.png</t>
+        </is>
+      </c>
+      <c r="B4819" t="inlineStr">
+        <is>
+          <t>tamilpsd-10726.png</t>
+        </is>
+      </c>
+      <c r="C4819" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6IlVOQ0xxcFlncThzWW11WWZmMjh4bXc9PSIsInZhbHVlIjoiZFRLQWhnNW55S2gvdnhEb3RtaW1YQT09IiwibWFjIjoiNzk5YjVhYmNjOTgzYTViM2JkNTdlMGI1NWUwMDk5NTEwZGIyMTVhMzNhYTc5OGJkZDgyYmI1OTdlMmRmZmFmOSIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4820">
+      <c r="A4820" s="3" t="inlineStr">
+        <is>
+          <t>4870.png</t>
+        </is>
+      </c>
+      <c r="B4820" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-10727.png</t>
+        </is>
+      </c>
+      <c r="C4820" s="3" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6Ilg0RnhKTW1zeGVxVGh3YllXdm9SUmc9PSIsInZhbHVlIjoiZ2RuQTNzeHM4S2U0YndDVEluMmRmUT09IiwibWFjIjoiZGY3OGRlOWMxZWNmY2FiNzk0YzVjZDIzODgyNTMzZjg1ZTI1ZDliMTJhMWY0NTg4MWI2MDdjNTUyOTk2MTY4NSIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4821">
+      <c r="A4821" t="inlineStr">
+        <is>
+          <t>4919.png</t>
+        </is>
+      </c>
+      <c r="B4821" t="inlineStr">
+        <is>
+          <t>tamilpsd-10728.png</t>
+        </is>
+      </c>
+      <c r="C4821" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6IjhHaTk2VTdjbmE2N0k1b0xSRWxEN2c9PSIsInZhbHVlIjoiekNkaFUxVDc2TFhseHlhYTVTMmZGdz09IiwibWFjIjoiMGZiYWJhZjRjMmQzOTcwZDMwZWVkZDZjMjFhOWM2YmE1ZDRkZTg4NGZhZDRlZGZlMjViMmZjYjQ3MDdhZmUzMCIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4822">
+      <c r="A4822" s="3" t="inlineStr">
+        <is>
+          <t>4918.png</t>
+        </is>
+      </c>
+      <c r="B4822" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-10729.png</t>
+        </is>
+      </c>
+      <c r="C4822" s="3" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6IkVXR0VtdmxBR1NHSGhKcEExVmxHV1E9PSIsInZhbHVlIjoiWW9BVzBua1h6L3BjemI4QzZ2YXVzZz09IiwibWFjIjoiMGUyM2FlNjhmOTYxZWU0NDM2ZDQ4ODgyNTU4NGFkMTBkYWE4MTNmMWFhZmI2NTM3OTFlOTRhZjRlNTE1NDk4MyIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4823">
+      <c r="A4823" t="inlineStr">
+        <is>
+          <t>4917.png</t>
+        </is>
+      </c>
+      <c r="B4823" t="inlineStr">
+        <is>
+          <t>tamilpsd-10730.png</t>
+        </is>
+      </c>
+      <c r="C4823" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6Ikl0WTBsTTBxRmxveXd0L3NvSmZQU0E9PSIsInZhbHVlIjoiNlZsUEdRU1cxTzZtTlh2alQ3M2dJZz09IiwibWFjIjoiMjViZWI2Y2ViY2NiMWM2ZDhmOWM4M2Y2MmUyYjk0ODQxZWEzODJmMjQ1ZDYwMjAxMGVhMWRhYWQwYTBhMzViOSIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4824">
+      <c r="A4824" s="3" t="inlineStr">
+        <is>
+          <t>4916.png</t>
+        </is>
+      </c>
+      <c r="B4824" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-10731.png</t>
+        </is>
+      </c>
+      <c r="C4824" s="3" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6IkYrM2krR2hGenFEdDE3TVRlM0ppNVE9PSIsInZhbHVlIjoic1VYb1hGcHJrd3VudXhBT3dJTmZSdz09IiwibWFjIjoiM2JiNDU1YjMwMGMwYmQ3ZmUxMmNiZTliNGQ1NzBjMDgxNTg0YzI4NTg5MTNhYjg5OTIyYTQ0NzA0MTY4M2QwMSIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4825">
+      <c r="A4825" t="inlineStr">
+        <is>
+          <t>4915.png</t>
+        </is>
+      </c>
+      <c r="B4825" t="inlineStr">
+        <is>
+          <t>tamilpsd-10732.png</t>
+        </is>
+      </c>
+      <c r="C4825" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6Ik8vaHd0bUU4eFdIb1VWZnRMdzJWdEE9PSIsInZhbHVlIjoiVmQvenVEMTNERjRjYmF6ME9FcUFZQT09IiwibWFjIjoiMzhiNGZkZWRlM2QwZWI1MDY0NWU3MzQzMTFkNWZiMDkzN2FjOWRiODFjOGU2OTk0NmI3ODFkNjUwZTA4MTliZSIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4826">
+      <c r="A4826" s="3" t="inlineStr">
+        <is>
+          <t>4914.png</t>
+        </is>
+      </c>
+      <c r="B4826" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-10733.png</t>
+        </is>
+      </c>
+      <c r="C4826" s="3" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6Imk3UnZuWTFWRWoyWUhwUXJrbFA0R0E9PSIsInZhbHVlIjoiQ1pyR05jMzlHWWJUazFQbStNSEdDUT09IiwibWFjIjoiMTU2YjgyMTRiNDQyMzg4YzhiMDQ5OWFhYWEyYzBhOTk4MzI1MWQ1ZDU5NzI5YzA1YzZiM2E4YmM3YTcyYzhiYSIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4827">
+      <c r="A4827" t="inlineStr">
+        <is>
+          <t>4913.png</t>
+        </is>
+      </c>
+      <c r="B4827" t="inlineStr">
+        <is>
+          <t>tamilpsd-10734.png</t>
+        </is>
+      </c>
+      <c r="C4827" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6ImkyVG0wLy9jTnFHWkVHeDRsb1FyZlE9PSIsInZhbHVlIjoiWWhiS1MwdHV6aEVKcWkyTjJQdTlRZz09IiwibWFjIjoiNjE0NTBlMGMzMGUxYTdkNmQ3YTEwYTc0NTM0YTM1Yjk1MTRlMjVhZDcxMmNlZjRlMjA4Mjk1MWY3YWZhOTBjMSIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4828">
+      <c r="A4828" s="3" t="inlineStr">
+        <is>
+          <t>4912.png</t>
+        </is>
+      </c>
+      <c r="B4828" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-10735.png</t>
+        </is>
+      </c>
+      <c r="C4828" s="3" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6IlJ6aVRUcDVwR3RaRklvZ3E2WmI2d3c9PSIsInZhbHVlIjoiVkdwVHhxQmpwbVZna214ZklpVmFsQT09IiwibWFjIjoiYTlhMTBhMmU4NjMwYjhjMjAzOGVlZjRiOTA4ZWYzZWJlZTVlMzYxMWI4MTA5ZjY0NzUxYTIxNGQ0NzYwM2YyYSIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4829">
+      <c r="A4829" t="inlineStr">
+        <is>
+          <t>4910.png</t>
+        </is>
+      </c>
+      <c r="B4829" t="inlineStr">
+        <is>
+          <t>tamilpsd-10736.png</t>
+        </is>
+      </c>
+      <c r="C4829" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6ImttQ0FhU1JxSEJ6WUc0MmVRT05lUnc9PSIsInZhbHVlIjoiOVQwUFFMdi8zSXBwNkJtVWExdmlHQT09IiwibWFjIjoiNTk0NzcyZjJiMGRkMzE5OTNiZDRkOWJiY2JjNjQ2ODVjYmIyMDNmMjdiODY3ZDAxNjI0NjYzZDM4ODIxYzM3MCIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4830">
+      <c r="A4830" s="3" t="inlineStr">
+        <is>
+          <t>4911.png</t>
+        </is>
+      </c>
+      <c r="B4830" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-10737.png</t>
+        </is>
+      </c>
+      <c r="C4830" s="3" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6Ii9jcW9oMFhoWHZNV2czVWNxdnhGMmc9PSIsInZhbHVlIjoiZVZrSGVhaXJ4N0gyVjR0QjVwQ3BmQT09IiwibWFjIjoiYzhhMjMzMzUzZjA1NzhmY2ZiNDgyMGQ3YmY4ZDM5ODA5OTZhNGRhNGNiOTUzOTc5N2YzZDc3MTlhZGNjN2VlOSIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4831">
+      <c r="A4831" t="inlineStr">
+        <is>
+          <t>4909.png</t>
+        </is>
+      </c>
+      <c r="B4831" t="inlineStr">
+        <is>
+          <t>tamilpsd-10738.png</t>
+        </is>
+      </c>
+      <c r="C4831" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6Imx0OXAxanh3MU5EZDEvVXZiRHlGTWc9PSIsInZhbHVlIjoiSEc4L283dXRxSU9Tai9BNkgrNGNuUT09IiwibWFjIjoiMmRiODE1M2ZhM2JlMzc4Y2I0ODdhZjg3NzMzY2I2ZGExY2M3ODkyYjg2OGRlMmQ4Y2MzY2QzYTFjMzIyZjZiMSIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4832">
+      <c r="A4832" s="3" t="inlineStr">
+        <is>
+          <t>4908.png</t>
+        </is>
+      </c>
+      <c r="B4832" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-10739.png</t>
+        </is>
+      </c>
+      <c r="C4832" s="3" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6IkxEMTRESFgxcktiZzF3NjU2dFBubUE9PSIsInZhbHVlIjoiQzdERmZIMHR0V3lRZndRRzdzemNwQT09IiwibWFjIjoiYmE2OWNiN2YzNDhiZmRmNGE4OTU4MmJkMjNlZTc2MWRjMjJlNDYzZmFkNzBlODZkYjZhNjQzM2QxYzVlOWE0ZSIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4833">
+      <c r="A4833" t="inlineStr">
+        <is>
+          <t>4906.png</t>
+        </is>
+      </c>
+      <c r="B4833" t="inlineStr">
+        <is>
+          <t>tamilpsd-10740.png</t>
+        </is>
+      </c>
+      <c r="C4833" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6ImpURHVTWi8wQWtSaWJLUkljdXozbVE9PSIsInZhbHVlIjoiYlBQY2xEMlpJMVpYbzlsVjVZb2VXZz09IiwibWFjIjoiODRiM2UwOWU3MWU5ZjU1YzQ3NTBmZDJhNTNlMDBlN2M3YjI3MDZkODY0YjFiNGM0ZDg2ZWM2YzIwYWRjZTE2OCIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4834">
+      <c r="A4834" s="3" t="inlineStr">
+        <is>
+          <t>4907.png</t>
+        </is>
+      </c>
+      <c r="B4834" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-10741.png</t>
+        </is>
+      </c>
+      <c r="C4834" s="3" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6Inhta0U4YWNKZFZxeVBoY1VmUGNLU1E9PSIsInZhbHVlIjoiK1dUdENhZ0M2Qnc3VGtWQUZrNG5TUT09IiwibWFjIjoiYmMzNWFhN2Y5ZjkzMWEzZDQyY2E2ZjNmNWFjMmExNGIzYzQ0ZmY0ZWU4ODMwZjY0NTZhMjYzMzRlNjlkMTVlYSIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4835">
+      <c r="A4835" t="inlineStr">
+        <is>
+          <t>4905.png</t>
+        </is>
+      </c>
+      <c r="B4835" t="inlineStr">
+        <is>
+          <t>tamilpsd-10742.png</t>
+        </is>
+      </c>
+      <c r="C4835" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6ImROTFZBeHFwZnpmcnM3Wk53d1JDOGc9PSIsInZhbHVlIjoic3NONWNjemtIZ1ZKZzhRSkRqWkw5QT09IiwibWFjIjoiYThiNWZkNzM2ZmExYjNmZjJmOWRiNGJkNDQ4OTVkMzZhMzYyNGNmMjc1ZGJmYmE2MjQ3ZGJjYzIwZjYxNjZkZCIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4836">
+      <c r="A4836" s="3" t="inlineStr">
+        <is>
+          <t>4903.png</t>
+        </is>
+      </c>
+      <c r="B4836" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-10743.png</t>
+        </is>
+      </c>
+      <c r="C4836" s="3" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6Iks0dGwvNStIczNCcFNBL3YyZkVJU0E9PSIsInZhbHVlIjoiNXgvU1orMjNnY1JDdDU3Z2FURnh6dz09IiwibWFjIjoiYTlmNDE5ODc2ZWJkYzQ4MTVmYmVjOWYzODUwZjJjNWM5ZDdiNjIwZmMzNGVkNTI0NzA0NGNjZTYxZTRkZDAwOCIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4837">
+      <c r="A4837" t="inlineStr">
+        <is>
+          <t>4904.png</t>
+        </is>
+      </c>
+      <c r="B4837" t="inlineStr">
+        <is>
+          <t>tamilpsd-10744.png</t>
+        </is>
+      </c>
+      <c r="C4837" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6IjM3ZzNZRm0zRSt2Wk05ejdsMGI3MUE9PSIsInZhbHVlIjoiZ0tBYWxnNHp5cTBnc3JxUml6aklLUT09IiwibWFjIjoiZDMzY2Q2YjdkMDJmNTYyN2JiNDM2NGRmOTkyZDZjMjdhMTlkMzM3YzY1NTg3YjQ4MjkzNmExOTI0N2EyZmIyZiIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4838">
+      <c r="A4838" s="3" t="inlineStr">
+        <is>
+          <t>4902.png</t>
+        </is>
+      </c>
+      <c r="B4838" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-10745.png</t>
+        </is>
+      </c>
+      <c r="C4838" s="3" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6ImNiWWp2Q09memJTOHZoR0xNelRZd1E9PSIsInZhbHVlIjoiTzlRNFQwV1ROTWJtbEtaWmNvTFpsZz09IiwibWFjIjoiYjAxNmQ2NGIzZDE5NTYxMjcyZGUyNTNjNjlhZTMyOTQ2MzVkZTM2YmY1YTAzMjFkNmU2YzBjNDMyNjMwZTZkMSIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4839">
+      <c r="A4839" t="inlineStr">
+        <is>
+          <t>4901.png</t>
+        </is>
+      </c>
+      <c r="B4839" t="inlineStr">
+        <is>
+          <t>tamilpsd-10746.png</t>
+        </is>
+      </c>
+      <c r="C4839" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6IkVkVlpscDNMSDNjSnMwRTkzSHEvS1E9PSIsInZhbHVlIjoiVS9QZFdVdHNaVU9HZytPOHhGRk1Ldz09IiwibWFjIjoiZTI0YTJjZGVjNDkzYTNmY2VhZDMxMTk4ZDYyNjlmMjU0ODVkZDk5MzYyZmY4YjFkMjc5OTkzNDA4NzhhMDM4OSIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4840">
+      <c r="A4840" s="3" t="inlineStr">
+        <is>
+          <t>4900.png</t>
+        </is>
+      </c>
+      <c r="B4840" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-10747.png</t>
+        </is>
+      </c>
+      <c r="C4840" s="3" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6IkxLV0xaMWwwb1ZPYmprcjV6UjFGa2c9PSIsInZhbHVlIjoiNDhuVklmSDRoV21oeFZNZTFVQWdlZz09IiwibWFjIjoiZGNkNmIyNTc5ZDg1YzVhNmJlMWUxZTZhY2NkMTQyNDRlYWEzOTY5YzczZWFlYTJiNmYyODU1ZmUzMTQzNmU4OCIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4841">
+      <c r="A4841" t="inlineStr">
+        <is>
+          <t>4899.png</t>
+        </is>
+      </c>
+      <c r="B4841" t="inlineStr">
+        <is>
+          <t>tamilpsd-10748.png</t>
+        </is>
+      </c>
+      <c r="C4841" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6IkFpWkZ3ZUNLM3lnVklWeVZYZDZWZVE9PSIsInZhbHVlIjoiK2xCYnJWelk0dkNZcmhTOW9uVG9LUT09IiwibWFjIjoiYjIxZTBiMTE5MTQ5YjRhYzBmODgyZDQwMDg5ZmJiNWU5NTQzZDAwYmM0YTU0YjZmN2MwY2EyZGVmZGIwYzc5NSIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4842">
+      <c r="A4842" s="3" t="inlineStr">
+        <is>
+          <t>4898.png</t>
+        </is>
+      </c>
+      <c r="B4842" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-10749.png</t>
+        </is>
+      </c>
+      <c r="C4842" s="3" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6InNUK0NNZFRTbjNMVm5KMm45Y2t0bWc9PSIsInZhbHVlIjoidUx0eTE5RFc1aFNvRWQxY2R3bUMvUT09IiwibWFjIjoiYzFiMjExYTBlMjA3MGJjY2U3MGU1NTU4NDBiNjE2ODAzOTAxMTRhZjM3YWE4YjQ1YWEyMmFlYzEzNDcwNTc4MiIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4843">
+      <c r="A4843" t="inlineStr">
+        <is>
+          <t>4896.png</t>
+        </is>
+      </c>
+      <c r="B4843" t="inlineStr">
+        <is>
+          <t>tamilpsd-10750.png</t>
+        </is>
+      </c>
+      <c r="C4843" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6IlBWcVI3WUJIbFdSSEdDRUNqQzZEQlE9PSIsInZhbHVlIjoiSGwrU3k3aTdocEp4a0EyVGZ6TnNGdz09IiwibWFjIjoiYzI1MWFjOTQ4ZDkzNjYxYWU4Y2ZhNzEzNDY3NmRkMDRlMTQ2ZTZhZGY0MzlkZDA2OTc0MTIyYTU0OGE4YzI3ZSIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4844">
+      <c r="A4844" s="3" t="inlineStr">
+        <is>
+          <t>4897.png</t>
+        </is>
+      </c>
+      <c r="B4844" s="3" t="inlineStr">
+        <is>
+          <t>tamilpsd-10751.png</t>
+        </is>
+      </c>
+      <c r="C4844" s="3" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6IkJPbXVZQlc4Rk9DVXNEWUxaZ01UK0E9PSIsInZhbHVlIjoibTVXVHhmbVZoTGxsMXNRdUxNSU5wZz09IiwibWFjIjoiYWRmOGYzMGVjYWFkNmE0MDQxZDk0MWUxOTVmZWQzMTE1YzEzMTY1ZjE1YjI1OWQyMzkyNjYwNWQ1MzJlMDJhZiIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
+    <row r="4845">
+      <c r="A4845" t="inlineStr">
+        <is>
+          <t>4895.png</t>
+        </is>
+      </c>
+      <c r="B4845" t="inlineStr">
+        <is>
+          <t>tamilpsd-10752.png</t>
+        </is>
+      </c>
+      <c r="C4845" t="inlineStr">
+        <is>
+          <t>https://forpsd.com/download/eyJpdiI6Iks0WEZOVzRjeEtPb3ZIMHZNTmNtZ3c9PSIsInZhbHVlIjoiQ2pFNnJVT3JxUE9RZzYrUld0cFlPUT09IiwibWFjIjoiN2MxZTI3N2NmMDM2NWUzNTM5YjIyMTQzMDdkZjc2OWYyMTUxMzgwMmZkZDgxNzQ0NDVlMGYyMTM2ZTM4MGU1MyIsInRhZyI6IiJ9</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>